<commit_message>
chore: list every demographic field in the acknowledgement and preview templates
</commit_message>
<xml_diff>
--- a/mosip_master/xlsx/template.xlsx
+++ b/mosip_master/xlsx/template.xlsx
@@ -11600,22 +11600,22 @@
     <t>தேவைப்பட்ட நடவடிக்கை: SBI காலாவதி</t>
   </si>
   <si>
-    <t>&lt;!DOCTYPE html&gt;&lt;html $rtl&gt;&lt;head&gt;&lt;meta charset="UTF-8"/&gt;&lt;style&gt;body,.head,.headings,th,td,p,b,strong{font-family:system-ui,"Segoe UI","Nirmala UI","Iskoola Pota","Latha",sans-serif;}table, .head{font-size:13px;}.demoDiv{width: 85%;float: left;}.photoDiv{width: 15%;float:right;}.form{display:block;width:100%;}.section{padding:24px;width:800px;max-width:800px;margin-left:auto;margin-right:auto;box-sizing:border-box;}.headings{color:#808080;font-size:11px;}p{display:inline;}.dataTable{word-wrap:break-word;table-layout:fixed;width:100%;}.headerTable{width:90%;}.uinHeaderTable{width:100%;}h5{display:inline;position:absolute;}.iris{top:-15px;left:152px;}.irisWithoutException{top:-15px;left:114px;}.tableWithoutException{width:50%;text-align:center;table-layout:fixed;margin:0 auto;}.biometricsTable{width:100%;text-align:center;table-layout:fixed;}.biometrics{position:relative;}.leftLittle{top:15px;left:11px;display:inline;position:absolute;}.leftRing{top:3px;left:23px;}.leftMiddle{top:-7px;left:37px;}.leftIndex{top:3px;left:54px;}.rightIndex{top:3px;left:26px;}.rightMiddle{top:-7px;left:39px;}.rightRing{top:3px;left:55px;}.rightLittle{top:15px;left:68px;}.leftThumb{top:-4px;left:24px;}.rightThumb{top:-4px;left:54px;}.parentStyle{top:-15px;left:152px;}.parentIris1{top:-15px;left:212px;}.parentIris2{top:-15px;left:214px;}li span{color:black;font-size:12px;} li{color:lightgrey}button{float:right;font-size:12px;border:none;background-color:transparent;outline:none;}button:active{background-color:black;color:white;} .bottom{vertical-align:bottom;}.consent-block{font-size:13px;border-radius: 8px;margin-top: 10px;margin-bottom: 10px;border: 2px solid #E88E3F;padding-top: -50px;padding:10px;}.consent-text{margin-left: 7px;margin-bottom: 4px;}input[type="radio"] {display: none;} input[type="radio"] + label:before { content: ""; display: inline-block; width: 15px; height: 15px; padding: 3px; margin-right: 5px; background-clip: content-box; border: 1px solid grey; background-color: #fff; border-radius: 50%;}input[type="radio"]:checked + label:before { background-color: #FF4081; border-color:#FF4081;}*,*:before,*:after { box-sizing: border-box;}.consent-block label { display: inline-flex; align-items: center;}.demoDiv&gt;table{width:100%}.demoDiv&gt;table&gt;tbody&gt;tr&gt;th{color:#808080;font-size:10px; width:25%; text-align: left;padding: 2px;font-weight:normal;}.demoDiv&gt;table&gt;tbody&gt;tr&gt;td{width:25%; text-align: left;padding: 2px}.ackPostBioBlock{display:block;clear:both;width:100%!important;max-width:100%;}.ackPostBioBlock hr{width:100%;}.ackPostBioBlock .dataTable{width:100%!important;max-width:100%;table-layout:fixed;border-collapse:collapse;display:table!important;}.ackPostBioBlock .headings,.ackPostBioBlock p.head,.ackPostBioBlock td&gt;p{display:block;}&lt;/style&gt;&lt;script&gt;function changeColour(element) { var div = document.getElementById("radioId"); if(element.value == "yes"){div.style = "border: 2px solid #68A933";} if(element.value == "no"){div.style = "border: 2px solid #FF0000";}} document.onreadystatechange = function () {if(document.readyState === "complete"){var body = document.getElementsByTagName("body")[0]; body.addEventListener("dragstart", function(event) {event.preventDefault();}); body.addEventListener("selectstart", function(event) {event.preventDefault();});}}&lt;/script&gt;&lt;/head&gt; &lt;body&gt; &lt;div class=section&gt; &lt;div class=form&gt; &lt;table class=headerTable&gt; &lt;tr&gt; #if ( !$isPreview &amp;&amp; $QRCodeSource ) &lt;td class=bottom&gt; &lt;img src="${QRCodeSource}" width=85 height=85/&gt; &lt;/td&gt; #end &lt;td class=bottom&gt;&lt;p class=headings&gt;${ApplicationIDLabel}&lt;/p&gt;&lt;br/&gt;${ApplicationID}&lt;/td&gt; #if ( $UIN ) &lt;td class=bottom&gt;&lt;p class=headings&gt;${UINLabel}&lt;/p&gt;&lt;br/&gt;${UIN}&lt;/td&gt; #end &lt;td class=bottom&gt;&lt;p class=headings&gt;${DateLabel}&lt;/p&gt;&lt;br/&gt;${Date}&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; &lt;br/&gt;#if ( $name ) &lt;table class=headerTable&gt; &lt;tr&gt;&lt;td&gt;&lt;p class=headings&gt;${NameLabel}&lt;/p&gt;&lt;br/&gt;${NameValue}&lt;/td&gt;&lt;/tr&gt; &lt;/table&gt; #end &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;${DemographicInfo}&lt;/p&gt; &lt;hr/&gt;&lt;div class="demoDiv"&gt;&lt;table&gt; &lt;tr&gt; #if( $demographics.get("name") ) &lt;th&gt;$demographics.get("name").get("label")&lt;/th&gt; #end #if( $demographics.get("surname") ) &lt;th&gt;$demographics.get("surname").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("name") ) &lt;td&gt;$demographics.get("name").get("value")&lt;/td&gt; #end #if( $demographics.get("surname") ) &lt;td&gt;$demographics.get("surname").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("fullName") ) &lt;th&gt;$demographics.get("fullName").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("fullName") ) &lt;td&gt;$demographics.get("fullName").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("dateOfBirth") ) &lt;th&gt;$demographics.get("dateOfBirth").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("dateOfBirth") ) &lt;td&gt;$demographics.get("dateOfBirth").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("gender") ) &lt;th&gt;$demographics.get("gender").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("gender") ) &lt;td&gt;$demographics.get("gender").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("phone") ) &lt;th&gt;$demographics.get("phone").get("label")&lt;/th&gt; #end #if( $demographics.get("email") ) &lt;th&gt;$demographics.get("email").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("phone") ) &lt;td&gt;$demographics.get("phone").get("value")&lt;/td&gt; #end #if( $demographics.get("email") ) &lt;td&gt;$demographics.get("email").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;/table&gt;&lt;table&gt; #if( $demographics.get("addressLine1") ) &lt;hr/&gt;&lt;h1 class="headings"&gt;Address&lt;/h1&gt; #end &lt;tr&gt; #if( $demographics.get("addressLine1") ) &lt;th&gt;$demographics.get("addressLine1").get("label")&lt;/th&gt; #end #if( $demographics.get("addressLine2") ) &lt;th&gt;$demographics.get("addressLine2").get("label")&lt;/th&gt; #end #if( $demographics.get("addressLine3") ) &lt;th&gt;$demographics.get("addressLine3").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("addressLine1") ) &lt;td&gt;$demographics.get("addressLine1").get("value")&lt;/td&gt; #end #if( $demographics.get("addressLine2") ) &lt;td&gt;$demographics.get("addressLine2").get("value")&lt;/td&gt; #end #if( $demographics.get("addressLine3") ) &lt;td&gt;$demographics.get("addressLine3").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;/table&gt;&lt;table&gt;&lt;tr&gt; #if( $demographics.get("region") ) &lt;th&gt;$demographics.get("region").get("label")&lt;/th&gt; #end #if( $demographics.get("province") ) &lt;th&gt;$demographics.get("province").get("label")&lt;/th&gt; #end #if( $demographics.get("city") ) &lt;th&gt;$demographics.get("city").get("label")&lt;/th&gt; #end #if( $demographics.get("district") ) &lt;th&gt;$demographics.get("district").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("region") ) &lt;td&gt;$demographics.get("region").get("value")&lt;/td&gt; #end #if( $demographics.get("province") ) &lt;td&gt;$demographics.get("province").get("value")&lt;/td&gt; #end #if( $demographics.get("city") ) &lt;td&gt;$demographics.get("city").get("value")&lt;/td&gt; #end #if( $demographics.get("district") ) &lt;td&gt;$demographics.get("district").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;/table&gt;&lt;table&gt;&lt;tr&gt; #if( $demographics.get("divisionalSecretariat") ) &lt;th&gt;$demographics.get("divisionalSecretariat").get("label")&lt;/th&gt; #end #if( $demographics.get("grammaNiladhari") ) &lt;th&gt;$demographics.get("grammaNiladhari").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("divisionalSecretariat") ) &lt;td&gt;$demographics.get("divisionalSecretariat").get("value")&lt;/td&gt; #end #if( $demographics.get("grammaNiladhari") ) &lt;td&gt;$demographics.get("grammaNiladhari").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;/table&gt;&lt;table&gt;&lt;tr&gt; #if( $demographics.get("zone") ) &lt;th&gt;$demographics.get("zone").get("label")&lt;/th&gt; #end #if( $demographics.get("postalCode") ) &lt;th&gt;$demographics.get("postalCode").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("zone") ) &lt;td&gt;$demographics.get("zone").get("value")&lt;/td&gt; #end #if( $demographics.get("postalCode") ) &lt;td&gt;$demographics.get("postalCode").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("modeOfClaim") ) &lt;th&gt;$demographics.get("modeOfClaim").get("label")&lt;/th&gt; #end&lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("modeOfClaim") ) &lt;td&gt;$demographics.get("modeOfClaim").get("value")&lt;/td&gt; #end&lt;/tr&gt;&lt;/table&gt; #if( $demographics.get("parentOrGuardianName") ) &lt;hr/&gt; &lt;table&gt; &lt;h1 class="headings"&gt;Guardian Details&lt;/h1&gt;&lt;tr&gt;&lt;th&gt;$demographics.get("parentOrGuardianName").get("label")&lt;/th&gt; #if( $demographics.get("parentOrGuardianRID") ) &lt;th&gt;$demographics.get("parentOrGuardianRID").get("label")&lt;/th&gt; #end #if( $demographics.get("parentOrGuardianUIN") ) &lt;th&gt;$demographics.get("parentOrGuardianUIN").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt;&lt;td&gt;$demographics.get("parentOrGuardianName").get("value")&lt;/td&gt; #if( $demographics.get("parentOrGuardianRID") ) &lt;td&gt;$demographics.get("parentOrGuardianRID").get("value")&lt;/td&gt; #end #if( $demographics.get("parentOrGuardianUIN") ) &lt;td&gt;$demographics.get("parentOrGuardianUIN").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;/table&gt; #end &lt;/div&gt;#if ( $ApplicantImageSource ) &lt;div class="photoDiv"&gt; &lt;table&gt; &lt;tr&gt; &lt;td&gt; &lt;p&gt;${Photo}&lt;/p&gt; &lt;/td&gt; &lt;/tr&gt; &lt;tr&gt; &lt;td&gt;&lt;img src="${ApplicantImageSource}" border=0 width=100 height=100/&gt;&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; &lt;/div&gt; #end &lt;div style="width: 100%; height: 50%; clear:both"&gt;&lt;/div&gt; &lt;br/&gt; &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;${DocumentsLabel}&lt;/p&gt; &lt;hr/&gt; &lt;table class="dataTable" style="width:100%;table-layout:fixed;border-collapse:collapse;"&gt; #foreach( $key in $documents.keySet() ) #if( $velocityCount % 2 == 1 )&lt;tr&gt;#end &lt;td style="vertical-align:top;width:50%;"&gt;&lt;p class=headings&gt;$documents.get($key).get("label")&lt;/p&gt;&lt;br/&gt;&lt;p&gt;$documents.get($key).get("value")&lt;/p&gt;&lt;/td&gt; #if( $velocityCount % 2 == 0 )&lt;/tr&gt;#end #end #if( $documents.size() % 2 == 1 )&lt;td style="vertical-align:top;width:50%;"&gt;&lt;/td&gt;&lt;/tr&gt;#end &lt;/table&gt; &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;${BiometricsLabel}&lt;/p&gt; &lt;hr/&gt; #foreach( $key in $biometrics.keySet() ) &lt;table&gt; &lt;tr&gt; &lt;td&gt;$biometrics.get($key).get("label")&lt;br/&gt; &lt;p class=headings&gt;${Fingers} ( $biometrics.get($key).get("FingerCount") ),${Iris} ( $biometrics.get($key).get("IrisCount") ),${Face} ( $biometrics.get($key).get("FaceCount") )&lt;br/&gt;&lt;/p&gt; &lt;br/&gt; &lt;/td&gt; &lt;/tr&gt; &lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftEye") ) &lt;td&gt; &lt;p class=headings&gt;${LeftEyeLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightEye") ) &lt;td&gt; &lt;p class=headings&gt;${RightEyeLabel}&lt;/p&gt; &lt;/td&gt; #end&lt;/tr&gt;&lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftEye") ) &lt;td&gt; #if( !$isPreview ) &lt;div class=biometrics&gt; &lt;h5 class=parentIris1&gt;$biometrics.get($key).get("LeftEye")&lt;/h5&gt; &lt;img src='$biometrics.get($key).get("CapturedLeftEye")' border=0 width=85 height=80/&gt; &lt;/div&gt; #end #if( $isPreview &amp;&amp; $biometrics.get($key).get("CapturedLeftEye") )&lt;img src='$biometrics.get($key).get("CapturedLeftEye")' border=0 width=85 height=80/&gt; #end &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightEye") ) &lt;td&gt;#if( !$isPreview ) &lt;div class=biometrics&gt; &lt;h5 class=parentIris1&gt;$biometrics.get($key).get("RightEye")&lt;/h5&gt; &lt;img src='$biometrics.get($key).get("CapturedRightEye")' border=0 width=85 height=80/&gt; &lt;/div&gt; #end &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftSlap") ) &lt;td&gt; &lt;p class=headings&gt;${LeftPalmLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightSlap") ) &lt;td&gt; &lt;p class=headings&gt;${RightPalmLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedThumbs") ) &lt;td&gt; &lt;p class=headings&gt;${ThumbsLabel}&lt;/p&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftSlap") ) &lt;td style=text-align:-webkit-center&gt; #if( !$isPreview ) &lt;table&gt; &lt;tr&gt; &lt;td&gt; &lt;div class=biometrics&gt; &lt;h5 class=leftLittle&gt;$biometrics.get($key).get("leftLittle")&lt;/h5&gt; &lt;h5 class=leftRing&gt;$biometrics.get($key).get("leftRing")&lt;/h5&gt; &lt;h5 class=leftMiddle&gt;$biometrics.get($key).get("leftMiddle")&lt;/h5&gt; &lt;h5 class=leftIndex&gt;$biometrics.get($key).get("leftIndex")&lt;/h5&gt; &lt;/div&gt; &lt;/td&gt;&lt;/tr&gt; &lt;tr&gt; &lt;td&gt;&lt;img src='$biometrics.get($key).get("CapturedLeftSlap")' border=0 width=85 height=80/&gt;&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; #end &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightSlap") ) &lt;td style=text-align:-webkit-center&gt; #if( !$isPreview ) &lt;table&gt; &lt;tr&gt; &lt;td&gt; &lt;div class=biometrics&gt; &lt;h5 class=rightIndex&gt;$biometrics.get($key).get("rightIndex")&lt;/h5&gt; &lt;h5 class=rightMiddle&gt;$biometrics.get($key).get("rightMiddle")&lt;/h5&gt; &lt;h5 class=rightRing&gt;$biometrics.get($key).get("rightRing")&lt;/h5&gt; &lt;h5 class=rightLittle&gt;$biometrics.get($key).get("rightLittle")&lt;/h5&gt; &lt;/div&gt; &lt;/td&gt;&lt;/tr&gt; &lt;tr&gt; &lt;td&gt;&lt;img src='$biometrics.get($key).get("CapturedRightSlap")' border=0 width=85 height=80/&gt;&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; #end &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedThumbs") ) &lt;td style=text-align:-webkit-center&gt; #if( !$isPreview ) &lt;table&gt; &lt;tr&gt; &lt;td&gt; &lt;div class=biometrics&gt; &lt;h5 class=leftThumb&gt;$biometrics.get($key).get("leftThumb")&lt;/h5&gt; &lt;h5 class=rightThumb&gt;$biometrics.get($key).get("rightThumb")&lt;/h5&gt; &lt;/div&gt; &lt;/td&gt;&lt;/tr&gt; &lt;tr&gt; &lt;td&gt;&lt;img src='$biometrics.get($key).get("CapturedThumbs")' border=0 width=85 height=80/&gt;&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; #end &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;br/&gt; &lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("FaceImageSource") ) &lt;td&gt; &lt;p class=headings&gt;${FaceLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("subType") == "applicant" &amp;&amp; $ExceptionImageSource ) &lt;td&gt; &lt;p class=headings&gt;${ExceptionPhotoLabel}&lt;/p&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;tr&gt; #if( $biometrics.get($key).get("FaceImageSource") ) &lt;td&gt;&lt;img src='$biometrics.get($key).get("FaceImageSource")' border=0 width=85 height=80/&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("subType") == "applicant" &amp;&amp; $ExceptionImageSource ) &lt;td&gt; &lt;img src="${ExceptionImageSource}" border=0 width=85 height=80/&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;/table&gt; #end &lt;br/&gt;&lt;div class="ackPostBioBlock" style="display:block;clear:both;width:100%;"&gt;#if( $SignatureSectionVisible )&lt;div data-mosip-ack-signature="1" style="display:block;width:100%;"&gt;&lt;br/&gt;&lt;hr/&gt;&lt;p class=head style="display:block;"&gt;${SignatureLabel}&lt;/p&gt;&lt;hr/&gt;&lt;/div&gt;#end&lt;table class="dataTable" style="width:100%;table-layout:fixed;border-collapse:collapse;display:table;clear:both;"&gt;#if( $SignatureSectionVisible )&lt;tr&gt;&lt;td style="vertical-align:top;width:50%;"&gt;&lt;p class=headings&gt;#if( $SignatureCaptured )${SignatureCapturedLabel}#else${SignatureNotCapturedLabel}#end&lt;/p&gt;&lt;br/&gt;&lt;p&gt;#if( $SignatureCaptured )&lt;span style="color:#2E7D32;font-size:18px;"&gt;&amp;#10004;&lt;/span&gt; &lt;span style="color:#2E7D32;"&gt;${SignatureCapturedLabel}&lt;/span&gt;#else&lt;span style="color:#808080;font-size:18px;"&gt;&amp;#10007;&lt;/span&gt; &lt;span style="color:#808080;"&gt;${SignatureNotCapturedLabel}&lt;/span&gt;#end&lt;/p&gt;&lt;/td&gt;#if( $SignatureCaptured )&lt;td style="vertical-align:top;width:50%;"&gt;&lt;p class=headings&gt;${SignatureLabel}&lt;/p&gt;&lt;br/&gt;&lt;p&gt;&lt;img data-mosip-applicant-signature="1" src="${SignatureImageSource}" border="0" width="200" height="85" style="max-width:200px;max-height:85px;object-fit:contain;border:1px solid #b0b0b0;background:#fff;display:block;"/&gt;&lt;/p&gt;&lt;/td&gt;#else&lt;td style="vertical-align:top;width:50%;"&gt;&lt;/td&gt;#end&lt;/tr&gt;#end&lt;tr&gt;&lt;td&gt;&lt;p class=headings&gt;${RONameLabel}&lt;/p&gt;&lt;br/&gt;&lt;p&gt;${ROName}&lt;/p&gt;&lt;/td&gt;&lt;td&gt;&lt;p class=headings&gt;${RegCenterLabel}&lt;/p&gt;&lt;br/&gt;&lt;p&gt;${RegCenter}&lt;/p&gt;&lt;/td&gt;&lt;/tr&gt;&lt;/table&gt;&lt;hr/&gt;&lt;br/&gt;&lt;/div&gt;&lt;div&gt;&lt;p&gt;${ImportantGuidelines}&lt;/p&gt; &lt;ul&gt; #foreach( $line in $Guidelines ) &lt;li&gt;&lt;span&gt;${line}&lt;/span&gt;&lt;/li&gt; #end &lt;/ul&gt;&lt;/div&gt;&lt;/div&gt;&lt;/div&gt;&lt;/body&gt;&lt;/html&gt;</t>
-  </si>
-  <si>
-    <t>&lt;!DOCTYPE html&gt;&lt;html $rtl&gt;&lt;head&gt;&lt;meta charset="UTF-8"/&gt;&lt;style&gt;body,.head,.headings,th,td,p,b,strong{font-family:system-ui,"Segoe UI","Nirmala UI","Iskoola Pota","Latha",sans-serif;}table, .head{font-size:13px;}.demoDiv{width: 85%;float: left;}.photoDiv{width: 15%;float:right;}.form{display:block;width:100%;}.section{padding:24px;width:800px;max-width:800px;margin-left:auto;margin-right:auto;box-sizing:border-box;}.headings{color:#808080;font-size:11px;}p{display:inline;}.dataTable{word-wrap:break-word;table-layout:fixed;width:100%;}.headerTable{width:90%;}.uinHeaderTable{width:100%;}h5{display:inline;position:absolute;}.iris{top:-15px;left:152px;}.irisWithoutException{top:-15px;left:114px;}.tableWithoutException{width:50%;text-align:center;table-layout:fixed;margin:0 auto;}.biometricsTable{width:100%;text-align:center;table-layout:fixed;}.biometrics{position:relative;}.leftLittle{top:15px;left:11px;display:inline;position:absolute;}.leftRing{top:3px;left:23px;}.leftMiddle{top:-7px;left:37px;}.leftIndex{top:3px;left:54px;}.rightIndex{top:3px;left:26px;}.rightMiddle{top:-7px;left:39px;}.rightRing{top:3px;left:55px;}.rightLittle{top:15px;left:68px;}.leftThumb{top:-4px;left:24px;}.rightThumb{top:-4px;left:54px;}.parentStyle{top:-15px;left:152px;}.parentIris1{top:-15px;left:212px;}.parentIris2{top:-15px;left:214px;}li span{color:black;font-size:12px;} li{color:lightgrey}button{float:right;font-size:12px;border:none;background-color:transparent;outline:none;}button:active{background-color:black;color:white;} .bottom{vertical-align:bottom;}.consent-block{font-size:13px;border-radius: 8px;margin-top: 10px;margin-bottom: 10px;border: 2px solid #E88E3F;padding-top: -50px;padding:10px;}.consent-text{margin-left: 7px;margin-bottom: 4px;}input[type="radio"] {display: none;} input[type="radio"] + label:before { content: ""; display: inline-block; width: 15px; height: 15px; padding: 3px; margin-right: 5px; background-clip: content-box; border: 1px solid grey; background-color: #fff; border-radius: 50%;}input[type="radio"]:checked + label:before { background-color: #FF4081; border-color:#FF4081;}*,*:before,*:after { box-sizing: border-box;}.consent-block label { display: inline-flex; align-items: center;}.demoDiv&gt;table{width:100%}.demoDiv&gt;table&gt;tbody&gt;tr&gt;th{color:#808080;font-size:10px; width:25%; text-align: left;padding: 2px;font-weight:normal;}.demoDiv&gt;table&gt;tbody&gt;tr&gt;td{width:25%; text-align: left;padding: 2px}.ackPostBioBlock{display:block;clear:both;width:100%!important;max-width:100%;}.ackPostBioBlock hr{width:100%;}.ackPostBioBlock .dataTable{width:100%!important;max-width:100%;table-layout:fixed;border-collapse:collapse;display:table!important;}.ackPostBioBlock .headings,.ackPostBioBlock p.head,.ackPostBioBlock td&gt;p{display:block;}&lt;/style&gt;&lt;script&gt;function changeColour(element) { var div = document.getElementById("radioId"); if(element.value == "yes"){div.style = "border: 2px solid #68A933";} if(element.value == "no"){div.style = "border: 2px solid #FF0000";}} document.onreadystatechange = function () {if(document.readyState === "complete"){var body = document.getElementsByTagName("body")[0]; body.addEventListener("dragstart", function(event) {event.preventDefault();}); body.addEventListener("selectstart", function(event) {event.preventDefault();});}}&lt;/script&gt;&lt;/head&gt; &lt;body&gt; &lt;div class=section&gt; &lt;div class=form&gt; &lt;table class=headerTable&gt; &lt;tr&gt; #if ( !$isPreview &amp;&amp; $QRCodeSource ) &lt;td class=bottom&gt; &lt;img src="${QRCodeSource}" width=85 height=85/&gt; &lt;/td&gt; #end &lt;td class=bottom&gt;&lt;p class=headings&gt;${ApplicationIDLabel}&lt;/p&gt;&lt;br/&gt;${ApplicationID}&lt;/td&gt; #if ( $UIN ) &lt;td class=bottom&gt;&lt;p class=headings&gt;${UINLabel}&lt;/p&gt;&lt;br/&gt;${UIN}&lt;/td&gt; #end &lt;td class=bottom&gt;&lt;p class=headings&gt;${DateLabel}&lt;/p&gt;&lt;br/&gt;${Date}&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; &lt;br/&gt;#if ( $name ) &lt;table class=headerTable&gt; &lt;tr&gt;&lt;td&gt;&lt;p class=headings&gt;${NameLabel}&lt;/p&gt;&lt;br/&gt;${NameValue}&lt;/td&gt;&lt;/tr&gt; &lt;/table&gt; #end &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;${DemographicInfo}&lt;/p&gt; &lt;hr/&gt;&lt;div class="demoDiv"&gt;&lt;table&gt; &lt;tr&gt; #if( $demographics.get("name") ) &lt;th&gt;$demographics.get("name").get("label")&lt;/th&gt; #end #if( $demographics.get("surname") ) &lt;th&gt;$demographics.get("surname").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("name") ) &lt;td&gt;$demographics.get("name").get("value")&lt;/td&gt; #end #if( $demographics.get("surname") ) &lt;td&gt;$demographics.get("surname").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("fullName") ) &lt;th&gt;$demographics.get("fullName").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("fullName") ) &lt;td&gt;$demographics.get("fullName").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("dateOfBirth") ) &lt;th&gt;$demographics.get("dateOfBirth").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("dateOfBirth") ) &lt;td&gt;$demographics.get("dateOfBirth").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("gender") ) &lt;th&gt;$demographics.get("gender").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("gender") ) &lt;td&gt;$demographics.get("gender").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("phone") ) &lt;th&gt;$demographics.get("phone").get("label")&lt;/th&gt; #end #if( $demographics.get("email") ) &lt;th&gt;$demographics.get("email").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("phone") ) &lt;td&gt;$demographics.get("phone").get("value")&lt;/td&gt; #end #if( $demographics.get("email") ) &lt;td&gt;$demographics.get("email").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;/table&gt;&lt;table&gt; #if( $demographics.get("addressLine1") ) &lt;hr/&gt;&lt;h1 class="headings"&gt;ලිපිනය&lt;/h1&gt; #end &lt;tr&gt; #if( $demographics.get("addressLine1") ) &lt;th&gt;$demographics.get("addressLine1").get("label")&lt;/th&gt; #end #if( $demographics.get("addressLine2") ) &lt;th&gt;$demographics.get("addressLine2").get("label")&lt;/th&gt; #end #if( $demographics.get("addressLine3") ) &lt;th&gt;$demographics.get("addressLine3").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("addressLine1") ) &lt;td&gt;$demographics.get("addressLine1").get("value")&lt;/td&gt; #end #if( $demographics.get("addressLine2") ) &lt;td&gt;$demographics.get("addressLine2").get("value")&lt;/td&gt; #end #if( $demographics.get("addressLine3") ) &lt;td&gt;$demographics.get("addressLine3").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;/table&gt;&lt;table&gt;&lt;tr&gt; #if( $demographics.get("region") ) &lt;th&gt;$demographics.get("region").get("label")&lt;/th&gt; #end #if( $demographics.get("province") ) &lt;th&gt;$demographics.get("province").get("label")&lt;/th&gt; #end #if( $demographics.get("city") ) &lt;th&gt;$demographics.get("city").get("label")&lt;/th&gt; #end #if( $demographics.get("district") ) &lt;th&gt;$demographics.get("district").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("region") ) &lt;td&gt;$demographics.get("region").get("value")&lt;/td&gt; #end #if( $demographics.get("province") ) &lt;td&gt;$demographics.get("province").get("value")&lt;/td&gt; #end #if( $demographics.get("city") ) &lt;td&gt;$demographics.get("city").get("value")&lt;/td&gt; #end #if( $demographics.get("district") ) &lt;td&gt;$demographics.get("district").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;/table&gt;&lt;table&gt;&lt;tr&gt; #if( $demographics.get("divisionalSecretariat") ) &lt;th&gt;$demographics.get("divisionalSecretariat").get("label")&lt;/th&gt; #end #if( $demographics.get("grammaNiladhari") ) &lt;th&gt;$demographics.get("grammaNiladhari").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("divisionalSecretariat") ) &lt;td&gt;$demographics.get("divisionalSecretariat").get("value")&lt;/td&gt; #end #if( $demographics.get("grammaNiladhari") ) &lt;td&gt;$demographics.get("grammaNiladhari").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;/table&gt;&lt;table&gt;&lt;tr&gt; #if( $demographics.get("zone") ) &lt;th&gt;$demographics.get("zone").get("label")&lt;/th&gt; #end #if( $demographics.get("postalCode") ) &lt;th&gt;$demographics.get("postalCode").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("zone") ) &lt;td&gt;$demographics.get("zone").get("value")&lt;/td&gt; #end #if( $demographics.get("postalCode") ) &lt;td&gt;$demographics.get("postalCode").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("modeOfClaim") ) &lt;th&gt;$demographics.get("modeOfClaim").get("label")&lt;/th&gt; #end&lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("modeOfClaim") ) &lt;td&gt;$demographics.get("modeOfClaim").get("value")&lt;/td&gt; #end&lt;/tr&gt;&lt;/table&gt; #if( $demographics.get("parentOrGuardianName") ) &lt;hr/&gt; &lt;table&gt; &lt;h1 class="headings"&gt;මාපිය/භාරකරු විස්තර&lt;/h1&gt;&lt;tr&gt;&lt;th&gt;$demographics.get("parentOrGuardianName").get("label")&lt;/th&gt; #if( $demographics.get("parentOrGuardianRID") ) &lt;th&gt;$demographics.get("parentOrGuardianRID").get("label")&lt;/th&gt; #end #if( $demographics.get("parentOrGuardianUIN") ) &lt;th&gt;$demographics.get("parentOrGuardianUIN").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt;&lt;td&gt;$demographics.get("parentOrGuardianName").get("value")&lt;/td&gt; #if( $demographics.get("parentOrGuardianRID") ) &lt;td&gt;$demographics.get("parentOrGuardianRID").get("value")&lt;/td&gt; #end #if( $demographics.get("parentOrGuardianUIN") ) &lt;td&gt;$demographics.get("parentOrGuardianUIN").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;/table&gt; #end &lt;/div&gt;#if ( $ApplicantImageSource ) &lt;div class="photoDiv"&gt; &lt;table&gt; &lt;tr&gt; &lt;td&gt; &lt;p&gt;${Photo}&lt;/p&gt; &lt;/td&gt; &lt;/tr&gt; &lt;tr&gt; &lt;td&gt;&lt;img src="${ApplicantImageSource}" border=0 width=100 height=100/&gt;&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; &lt;/div&gt; #end &lt;div style="width: 100%; height: 50%; clear:both"&gt;&lt;/div&gt; &lt;br/&gt; &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;${DocumentsLabel}&lt;/p&gt; &lt;hr/&gt; &lt;table class="dataTable" style="width:100%;table-layout:fixed;border-collapse:collapse;"&gt; #foreach( $key in $documents.keySet() ) #if( $velocityCount % 2 == 1 )&lt;tr&gt;#end &lt;td style="vertical-align:top;width:50%;"&gt;&lt;p class=headings&gt;$documents.get($key).get("label")&lt;/p&gt;&lt;br/&gt;&lt;p&gt;$documents.get($key).get("value")&lt;/p&gt;&lt;/td&gt; #if( $velocityCount % 2 == 0 )&lt;/tr&gt;#end #end #if( $documents.size() % 2 == 1 )&lt;td style="vertical-align:top;width:50%;"&gt;&lt;/td&gt;&lt;/tr&gt;#end &lt;/table&gt; &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;${BiometricsLabel}&lt;/p&gt; &lt;hr/&gt; #foreach( $key in $biometrics.keySet() ) &lt;table&gt; &lt;tr&gt; &lt;td&gt;$biometrics.get($key).get("label")&lt;br/&gt; &lt;p class=headings&gt;${Fingers} ( $biometrics.get($key).get("FingerCount") ),${Iris} ( $biometrics.get($key).get("IrisCount") ),${Face} ( $biometrics.get($key).get("FaceCount") )&lt;br/&gt;&lt;/p&gt; &lt;br/&gt; &lt;/td&gt; &lt;/tr&gt; &lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftEye") ) &lt;td&gt; &lt;p class=headings&gt;${LeftEyeLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightEye") ) &lt;td&gt; &lt;p class=headings&gt;${RightEyeLabel}&lt;/p&gt; &lt;/td&gt; #end&lt;/tr&gt;&lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftEye") ) &lt;td&gt; #if( !$isPreview ) &lt;div class=biometrics&gt; &lt;h5 class=parentIris1&gt;$biometrics.get($key).get("LeftEye")&lt;/h5&gt; &lt;img src='$biometrics.get($key).get("CapturedLeftEye")' border=0 width=85 height=80/&gt; &lt;/div&gt; #end #if( $isPreview &amp;&amp; $biometrics.get($key).get("CapturedLeftEye") )&lt;img src='$biometrics.get($key).get("CapturedLeftEye")' border=0 width=85 height=80/&gt; #end &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightEye") ) &lt;td&gt;#if( !$isPreview ) &lt;div class=biometrics&gt; &lt;h5 class=parentIris1&gt;$biometrics.get($key).get("RightEye")&lt;/h5&gt; &lt;img src='$biometrics.get($key).get("CapturedRightEye")' border=0 width=85 height=80/&gt; &lt;/div&gt; #end &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftSlap") ) &lt;td&gt; &lt;p class=headings&gt;${LeftPalmLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightSlap") ) &lt;td&gt; &lt;p class=headings&gt;${RightPalmLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedThumbs") ) &lt;td&gt; &lt;p class=headings&gt;${ThumbsLabel}&lt;/p&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftSlap") ) &lt;td style=text-align:-webkit-center&gt; #if( !$isPreview ) &lt;table&gt; &lt;tr&gt; &lt;td&gt; &lt;div class=biometrics&gt; &lt;h5 class=leftLittle&gt;$biometrics.get($key).get("leftLittle")&lt;/h5&gt; &lt;h5 class=leftRing&gt;$biometrics.get($key).get("leftRing")&lt;/h5&gt; &lt;h5 class=leftMiddle&gt;$biometrics.get($key).get("leftMiddle")&lt;/h5&gt; &lt;h5 class=leftIndex&gt;$biometrics.get($key).get("leftIndex")&lt;/h5&gt; &lt;/div&gt; &lt;/td&gt;&lt;/tr&gt; &lt;tr&gt; &lt;td&gt;&lt;img src='$biometrics.get($key).get("CapturedLeftSlap")' border=0 width=85 height=80/&gt;&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; #end &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightSlap") ) &lt;td style=text-align:-webkit-center&gt; #if( !$isPreview ) &lt;table&gt; &lt;tr&gt; &lt;td&gt; &lt;div class=biometrics&gt; &lt;h5 class=rightIndex&gt;$biometrics.get($key).get("rightIndex")&lt;/h5&gt; &lt;h5 class=rightMiddle&gt;$biometrics.get($key).get("rightMiddle")&lt;/h5&gt; &lt;h5 class=rightRing&gt;$biometrics.get($key).get("rightRing")&lt;/h5&gt; &lt;h5 class=rightLittle&gt;$biometrics.get($key).get("rightLittle")&lt;/h5&gt; &lt;/div&gt; &lt;/td&gt;&lt;/tr&gt; &lt;tr&gt; &lt;td&gt;&lt;img src='$biometrics.get($key).get("CapturedRightSlap")' border=0 width=85 height=80/&gt;&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; #end &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedThumbs") ) &lt;td style=text-align:-webkit-center&gt; #if( !$isPreview ) &lt;table&gt; &lt;tr&gt; &lt;td&gt; &lt;div class=biometrics&gt; &lt;h5 class=leftThumb&gt;$biometrics.get($key).get("leftThumb")&lt;/h5&gt; &lt;h5 class=rightThumb&gt;$biometrics.get($key).get("rightThumb")&lt;/h5&gt; &lt;/div&gt; &lt;/td&gt;&lt;/tr&gt; &lt;tr&gt; &lt;td&gt;&lt;img src='$biometrics.get($key).get("CapturedThumbs")' border=0 width=85 height=80/&gt;&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; #end &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;br/&gt; &lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("FaceImageSource") ) &lt;td&gt; &lt;p class=headings&gt;${FaceLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("subType") == "applicant" &amp;&amp; $ExceptionImageSource ) &lt;td&gt; &lt;p class=headings&gt;${ExceptionPhotoLabel}&lt;/p&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;tr&gt; #if( $biometrics.get($key).get("FaceImageSource") ) &lt;td&gt;&lt;img src='$biometrics.get($key).get("FaceImageSource")' border=0 width=85 height=80/&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("subType") == "applicant" &amp;&amp; $ExceptionImageSource ) &lt;td&gt; &lt;img src="${ExceptionImageSource}" border=0 width=85 height=80/&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;/table&gt; #end &lt;br/&gt;&lt;div class="ackPostBioBlock" style="display:block;clear:both;width:100%;"&gt;#if( $SignatureSectionVisible )&lt;div data-mosip-ack-signature="1" style="display:block;width:100%;"&gt;&lt;br/&gt;&lt;hr/&gt;&lt;p class=head style="display:block;"&gt;${SignatureLabel}&lt;/p&gt;&lt;hr/&gt;&lt;/div&gt;#end&lt;table class="dataTable" style="width:100%;table-layout:fixed;border-collapse:collapse;display:table;clear:both;"&gt;#if( $SignatureSectionVisible )&lt;tr&gt;&lt;td style="vertical-align:top;width:50%;"&gt;&lt;p class=headings&gt;#if( $SignatureCaptured )${SignatureCapturedLabel}#else${SignatureNotCapturedLabel}#end&lt;/p&gt;&lt;br/&gt;&lt;p&gt;#if( $SignatureCaptured )&lt;span style="color:#2E7D32;font-size:18px;"&gt;&amp;#10004;&lt;/span&gt; &lt;span style="color:#2E7D32;"&gt;${SignatureCapturedLabel}&lt;/span&gt;#else&lt;span style="color:#808080;font-size:18px;"&gt;&amp;#10007;&lt;/span&gt; &lt;span style="color:#808080;"&gt;${SignatureNotCapturedLabel}&lt;/span&gt;#end&lt;/p&gt;&lt;/td&gt;#if( $SignatureCaptured )&lt;td style="vertical-align:top;width:50%;"&gt;&lt;p class=headings&gt;${SignatureLabel}&lt;/p&gt;&lt;br/&gt;&lt;p&gt;&lt;img data-mosip-applicant-signature="1" src="${SignatureImageSource}" border="0" width="200" height="85" style="max-width:200px;max-height:85px;object-fit:contain;border:1px solid #b0b0b0;background:#fff;display:block;"/&gt;&lt;/p&gt;&lt;/td&gt;#else&lt;td style="vertical-align:top;width:50%;"&gt;&lt;/td&gt;#end&lt;/tr&gt;#end&lt;tr&gt;&lt;td&gt;&lt;p class=headings&gt;${RONameLabel}&lt;/p&gt;&lt;br/&gt;&lt;p&gt;${ROName}&lt;/p&gt;&lt;/td&gt;&lt;td&gt;&lt;p class=headings&gt;${RegCenterLabel}&lt;/p&gt;&lt;br/&gt;&lt;p&gt;${RegCenter}&lt;/p&gt;&lt;/td&gt;&lt;/tr&gt;&lt;/table&gt;&lt;hr/&gt;&lt;br/&gt;&lt;/div&gt;&lt;div&gt;&lt;p&gt;${ImportantGuidelines}&lt;/p&gt; &lt;ul&gt; #foreach( $line in $Guidelines ) &lt;li&gt;&lt;span&gt;${line}&lt;/span&gt;&lt;/li&gt; #end &lt;/ul&gt;&lt;/div&gt;&lt;/div&gt;&lt;/div&gt;&lt;/body&gt;&lt;/html&gt;</t>
-  </si>
-  <si>
-    <t>&lt;!DOCTYPE html&gt;&lt;html $rtl&gt;&lt;head&gt;&lt;meta charset="UTF-8"/&gt;&lt;style&gt;body,.head,.headings,th,td,p,b,strong{font-family:system-ui,"Segoe UI","Nirmala UI","Iskoola Pota","Latha",sans-serif;}table, .head{font-size:13px;}.demoDiv{width: 85%;float: left;}.photoDiv{width: 15%;float:right;}.form{display:block;width:100%;}.section{padding:24px;width:800px;max-width:800px;margin-left:auto;margin-right:auto;box-sizing:border-box;}.headings{color:#808080;font-size:11px;}p{display:inline;}.dataTable{word-wrap:break-word;table-layout:fixed;width:100%;}.headerTable{width:90%;}.uinHeaderTable{width:100%;}h5{display:inline;position:absolute;}.iris{top:-15px;left:152px;}.irisWithoutException{top:-15px;left:114px;}.tableWithoutException{width:50%;text-align:center;table-layout:fixed;margin:0 auto;}.biometricsTable{width:100%;text-align:center;table-layout:fixed;}.biometrics{position:relative;}.leftLittle{top:15px;left:11px;display:inline;position:absolute;}.leftRing{top:3px;left:23px;}.leftMiddle{top:-7px;left:37px;}.leftIndex{top:3px;left:54px;}.rightIndex{top:3px;left:26px;}.rightMiddle{top:-7px;left:39px;}.rightRing{top:3px;left:55px;}.rightLittle{top:15px;left:68px;}.leftThumb{top:-4px;left:24px;}.rightThumb{top:-4px;left:54px;}.parentStyle{top:-15px;left:152px;}.parentIris1{top:-15px;left:212px;}.parentIris2{top:-15px;left:214px;}li span{color:black;font-size:12px;} li{color:lightgrey}button{float:right;font-size:12px;border:none;background-color:transparent;outline:none;}button:active{background-color:black;color:white;} .bottom{vertical-align:bottom;}.consent-block{font-size:13px;border-radius: 8px;margin-top: 10px;margin-bottom: 10px;border: 2px solid #E88E3F;padding-top: -50px;padding:10px;}.consent-text{margin-left: 7px;margin-bottom: 4px;}input[type="radio"] {display: none;} input[type="radio"] + label:before { content: ""; display: inline-block; width: 15px; height: 15px; padding: 3px; margin-right: 5px; background-clip: content-box; border: 1px solid grey; background-color: #fff; border-radius: 50%;}input[type="radio"]:checked + label:before { background-color: #FF4081; border-color:#FF4081;}*,*:before,*:after { box-sizing: border-box;}.consent-block label { display: inline-flex; align-items: center;}.demoDiv&gt;table{width:100%}.demoDiv&gt;table&gt;tbody&gt;tr&gt;th{color:#808080;font-size:10px; width:25%; text-align: left;padding: 2px;font-weight:normal;}.demoDiv&gt;table&gt;tbody&gt;tr&gt;td{width:25%; text-align: left;padding: 2px}.ackPostBioBlock{display:block;clear:both;width:100%!important;max-width:100%;}.ackPostBioBlock hr{width:100%;}.ackPostBioBlock .dataTable{width:100%!important;max-width:100%;table-layout:fixed;border-collapse:collapse;display:table!important;}.ackPostBioBlock .headings,.ackPostBioBlock p.head,.ackPostBioBlock td&gt;p{display:block;}&lt;/style&gt;&lt;script&gt;function changeColour(element) { var div = document.getElementById("radioId"); if(element.value == "yes"){div.style = "border: 2px solid #68A933";} if(element.value == "no"){div.style = "border: 2px solid #FF0000";}} document.onreadystatechange = function () {if(document.readyState === "complete"){var body = document.getElementsByTagName("body")[0]; body.addEventListener("dragstart", function(event) {event.preventDefault();}); body.addEventListener("selectstart", function(event) {event.preventDefault();});}}&lt;/script&gt;&lt;/head&gt; &lt;body&gt; &lt;div class=section&gt; &lt;div class=form&gt; &lt;table class=headerTable&gt; &lt;tr&gt; #if ( !$isPreview &amp;&amp; $QRCodeSource ) &lt;td class=bottom&gt; &lt;img src="${QRCodeSource}" width=85 height=85/&gt; &lt;/td&gt; #end &lt;td class=bottom&gt;&lt;p class=headings&gt;${ApplicationIDLabel}&lt;/p&gt;&lt;br/&gt;${ApplicationID}&lt;/td&gt; #if ( $UIN ) &lt;td class=bottom&gt;&lt;p class=headings&gt;${UINLabel}&lt;/p&gt;&lt;br/&gt;${UIN}&lt;/td&gt; #end &lt;td class=bottom&gt;&lt;p class=headings&gt;${DateLabel}&lt;/p&gt;&lt;br/&gt;${Date}&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; &lt;br/&gt;#if ( $name ) &lt;table class=headerTable&gt; &lt;tr&gt;&lt;td&gt;&lt;p class=headings&gt;${NameLabel}&lt;/p&gt;&lt;br/&gt;${NameValue}&lt;/td&gt;&lt;/tr&gt; &lt;/table&gt; #end &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;${DemographicInfo}&lt;/p&gt; &lt;hr/&gt;&lt;div class="demoDiv"&gt;&lt;table&gt; &lt;tr&gt; #if( $demographics.get("name") ) &lt;th&gt;$demographics.get("name").get("label")&lt;/th&gt; #end #if( $demographics.get("surname") ) &lt;th&gt;$demographics.get("surname").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("name") ) &lt;td&gt;$demographics.get("name").get("value")&lt;/td&gt; #end #if( $demographics.get("surname") ) &lt;td&gt;$demographics.get("surname").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("fullName") ) &lt;th&gt;$demographics.get("fullName").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("fullName") ) &lt;td&gt;$demographics.get("fullName").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("dateOfBirth") ) &lt;th&gt;$demographics.get("dateOfBirth").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("dateOfBirth") ) &lt;td&gt;$demographics.get("dateOfBirth").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("gender") ) &lt;th&gt;$demographics.get("gender").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("gender") ) &lt;td&gt;$demographics.get("gender").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("phone") ) &lt;th&gt;$demographics.get("phone").get("label")&lt;/th&gt; #end #if( $demographics.get("email") ) &lt;th&gt;$demographics.get("email").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("phone") ) &lt;td&gt;$demographics.get("phone").get("value")&lt;/td&gt; #end #if( $demographics.get("email") ) &lt;td&gt;$demographics.get("email").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;/table&gt;&lt;table&gt; #if( $demographics.get("addressLine1") ) &lt;hr/&gt;&lt;h1 class="headings"&gt;முகவரி&lt;/h1&gt; #end &lt;tr&gt; #if( $demographics.get("addressLine1") ) &lt;th&gt;$demographics.get("addressLine1").get("label")&lt;/th&gt; #end #if( $demographics.get("addressLine2") ) &lt;th&gt;$demographics.get("addressLine2").get("label")&lt;/th&gt; #end #if( $demographics.get("addressLine3") ) &lt;th&gt;$demographics.get("addressLine3").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("addressLine1") ) &lt;td&gt;$demographics.get("addressLine1").get("value")&lt;/td&gt; #end #if( $demographics.get("addressLine2") ) &lt;td&gt;$demographics.get("addressLine2").get("value")&lt;/td&gt; #end #if( $demographics.get("addressLine3") ) &lt;td&gt;$demographics.get("addressLine3").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;/table&gt;&lt;table&gt;&lt;tr&gt; #if( $demographics.get("region") ) &lt;th&gt;$demographics.get("region").get("label")&lt;/th&gt; #end #if( $demographics.get("province") ) &lt;th&gt;$demographics.get("province").get("label")&lt;/th&gt; #end #if( $demographics.get("city") ) &lt;th&gt;$demographics.get("city").get("label")&lt;/th&gt; #end #if( $demographics.get("district") ) &lt;th&gt;$demographics.get("district").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("region") ) &lt;td&gt;$demographics.get("region").get("value")&lt;/td&gt; #end #if( $demographics.get("province") ) &lt;td&gt;$demographics.get("province").get("value")&lt;/td&gt; #end #if( $demographics.get("city") ) &lt;td&gt;$demographics.get("city").get("value")&lt;/td&gt; #end #if( $demographics.get("district") ) &lt;td&gt;$demographics.get("district").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;/table&gt;&lt;table&gt;&lt;tr&gt; #if( $demographics.get("divisionalSecretariat") ) &lt;th&gt;$demographics.get("divisionalSecretariat").get("label")&lt;/th&gt; #end #if( $demographics.get("grammaNiladhari") ) &lt;th&gt;$demographics.get("grammaNiladhari").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("divisionalSecretariat") ) &lt;td&gt;$demographics.get("divisionalSecretariat").get("value")&lt;/td&gt; #end #if( $demographics.get("grammaNiladhari") ) &lt;td&gt;$demographics.get("grammaNiladhari").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;/table&gt;&lt;table&gt;&lt;tr&gt; #if( $demographics.get("zone") ) &lt;th&gt;$demographics.get("zone").get("label")&lt;/th&gt; #end #if( $demographics.get("postalCode") ) &lt;th&gt;$demographics.get("postalCode").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("zone") ) &lt;td&gt;$demographics.get("zone").get("value")&lt;/td&gt; #end #if( $demographics.get("postalCode") ) &lt;td&gt;$demographics.get("postalCode").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("modeOfClaim") ) &lt;th&gt;$demographics.get("modeOfClaim").get("label")&lt;/th&gt; #end&lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("modeOfClaim") ) &lt;td&gt;$demographics.get("modeOfClaim").get("value")&lt;/td&gt; #end&lt;/tr&gt;&lt;/table&gt; #if( $demographics.get("parentOrGuardianName") ) &lt;hr/&gt; &lt;table&gt; &lt;h1 class="headings"&gt;பாலரின்/பாதுகாவலர் விவரங்கள்&lt;/h1&gt;&lt;tr&gt;&lt;th&gt;$demographics.get("parentOrGuardianName").get("label")&lt;/th&gt; #if( $demographics.get("parentOrGuardianRID") ) &lt;th&gt;$demographics.get("parentOrGuardianRID").get("label")&lt;/th&gt; #end #if( $demographics.get("parentOrGuardianUIN") ) &lt;th&gt;$demographics.get("parentOrGuardianUIN").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt;&lt;td&gt;$demographics.get("parentOrGuardianName").get("value")&lt;/td&gt; #if( $demographics.get("parentOrGuardianRID") ) &lt;td&gt;$demographics.get("parentOrGuardianRID").get("value")&lt;/td&gt; #end #if( $demographics.get("parentOrGuardianUIN") ) &lt;td&gt;$demographics.get("parentOrGuardianUIN").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;/table&gt; #end &lt;/div&gt;#if ( $ApplicantImageSource ) &lt;div class="photoDiv"&gt; &lt;table&gt; &lt;tr&gt; &lt;td&gt; &lt;p&gt;${Photo}&lt;/p&gt; &lt;/td&gt; &lt;/tr&gt; &lt;tr&gt; &lt;td&gt;&lt;img src="${ApplicantImageSource}" border=0 width=100 height=100/&gt;&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; &lt;/div&gt; #end &lt;div style="width: 100%; height: 50%; clear:both"&gt;&lt;/div&gt; &lt;br/&gt; &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;${DocumentsLabel}&lt;/p&gt; &lt;hr/&gt; &lt;table class="dataTable" style="width:100%;table-layout:fixed;border-collapse:collapse;"&gt; #foreach( $key in $documents.keySet() ) #if( $velocityCount % 2 == 1 )&lt;tr&gt;#end &lt;td style="vertical-align:top;width:50%;"&gt;&lt;p class=headings&gt;$documents.get($key).get("label")&lt;/p&gt;&lt;br/&gt;&lt;p&gt;$documents.get($key).get("value")&lt;/p&gt;&lt;/td&gt; #if( $velocityCount % 2 == 0 )&lt;/tr&gt;#end #end #if( $documents.size() % 2 == 1 )&lt;td style="vertical-align:top;width:50%;"&gt;&lt;/td&gt;&lt;/tr&gt;#end &lt;/table&gt; &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;${BiometricsLabel}&lt;/p&gt; &lt;hr/&gt; #foreach( $key in $biometrics.keySet() ) &lt;table&gt; &lt;tr&gt; &lt;td&gt;$biometrics.get($key).get("label")&lt;br/&gt; &lt;p class=headings&gt;${Fingers} ( $biometrics.get($key).get("FingerCount") ),${Iris} ( $biometrics.get($key).get("IrisCount") ),${Face} ( $biometrics.get($key).get("FaceCount") )&lt;br/&gt;&lt;/p&gt; &lt;br/&gt; &lt;/td&gt; &lt;/tr&gt; &lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftEye") ) &lt;td&gt; &lt;p class=headings&gt;${LeftEyeLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightEye") ) &lt;td&gt; &lt;p class=headings&gt;${RightEyeLabel}&lt;/p&gt; &lt;/td&gt; #end&lt;/tr&gt;&lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftEye") ) &lt;td&gt; #if( !$isPreview ) &lt;div class=biometrics&gt; &lt;h5 class=parentIris1&gt;$biometrics.get($key).get("LeftEye")&lt;/h5&gt; &lt;img src='$biometrics.get($key).get("CapturedLeftEye")' border=0 width=85 height=80/&gt; &lt;/div&gt; #end #if( $isPreview &amp;&amp; $biometrics.get($key).get("CapturedLeftEye") )&lt;img src='$biometrics.get($key).get("CapturedLeftEye")' border=0 width=85 height=80/&gt; #end &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightEye") ) &lt;td&gt;#if( !$isPreview ) &lt;div class=biometrics&gt; &lt;h5 class=parentIris1&gt;$biometrics.get($key).get("RightEye")&lt;/h5&gt; &lt;img src='$biometrics.get($key).get("CapturedRightEye")' border=0 width=85 height=80/&gt; &lt;/div&gt; #end &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftSlap") ) &lt;td&gt; &lt;p class=headings&gt;${LeftPalmLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightSlap") ) &lt;td&gt; &lt;p class=headings&gt;${RightPalmLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedThumbs") ) &lt;td&gt; &lt;p class=headings&gt;${ThumbsLabel}&lt;/p&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftSlap") ) &lt;td style=text-align:-webkit-center&gt; #if( !$isPreview ) &lt;table&gt; &lt;tr&gt; &lt;td&gt; &lt;div class=biometrics&gt; &lt;h5 class=leftLittle&gt;$biometrics.get($key).get("leftLittle")&lt;/h5&gt; &lt;h5 class=leftRing&gt;$biometrics.get($key).get("leftRing")&lt;/h5&gt; &lt;h5 class=leftMiddle&gt;$biometrics.get($key).get("leftMiddle")&lt;/h5&gt; &lt;h5 class=leftIndex&gt;$biometrics.get($key).get("leftIndex")&lt;/h5&gt; &lt;/div&gt; &lt;/td&gt;&lt;/tr&gt; &lt;tr&gt; &lt;td&gt;&lt;img src='$biometrics.get($key).get("CapturedLeftSlap")' border=0 width=85 height=80/&gt;&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; #end &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightSlap") ) &lt;td style=text-align:-webkit-center&gt; #if( !$isPreview ) &lt;table&gt; &lt;tr&gt; &lt;td&gt; &lt;div class=biometrics&gt; &lt;h5 class=rightIndex&gt;$biometrics.get($key).get("rightIndex")&lt;/h5&gt; &lt;h5 class=rightMiddle&gt;$biometrics.get($key).get("rightMiddle")&lt;/h5&gt; &lt;h5 class=rightRing&gt;$biometrics.get($key).get("rightRing")&lt;/h5&gt; &lt;h5 class=rightLittle&gt;$biometrics.get($key).get("rightLittle")&lt;/h5&gt; &lt;/div&gt; &lt;/td&gt;&lt;/tr&gt; &lt;tr&gt; &lt;td&gt;&lt;img src='$biometrics.get($key).get("CapturedRightSlap")' border=0 width=85 height=80/&gt;&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; #end &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedThumbs") ) &lt;td style=text-align:-webkit-center&gt; #if( !$isPreview ) &lt;table&gt; &lt;tr&gt; &lt;td&gt; &lt;div class=biometrics&gt; &lt;h5 class=leftThumb&gt;$biometrics.get($key).get("leftThumb")&lt;/h5&gt; &lt;h5 class=rightThumb&gt;$biometrics.get($key).get("rightThumb")&lt;/h5&gt; &lt;/div&gt; &lt;/td&gt;&lt;/tr&gt; &lt;tr&gt; &lt;td&gt;&lt;img src='$biometrics.get($key).get("CapturedThumbs")' border=0 width=85 height=80/&gt;&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; #end &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;br/&gt; &lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("FaceImageSource") ) &lt;td&gt; &lt;p class=headings&gt;${FaceLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("subType") == "applicant" &amp;&amp; $ExceptionImageSource ) &lt;td&gt; &lt;p class=headings&gt;${ExceptionPhotoLabel}&lt;/p&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;tr&gt; #if( $biometrics.get($key).get("FaceImageSource") ) &lt;td&gt;&lt;img src='$biometrics.get($key).get("FaceImageSource")' border=0 width=85 height=80/&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("subType") == "applicant" &amp;&amp; $ExceptionImageSource ) &lt;td&gt; &lt;img src="${ExceptionImageSource}" border=0 width=85 height=80/&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;/table&gt; #end &lt;br/&gt;&lt;div class="ackPostBioBlock" style="display:block;clear:both;width:100%;"&gt;#if( $SignatureSectionVisible )&lt;div data-mosip-ack-signature="1" style="display:block;width:100%;"&gt;&lt;br/&gt;&lt;hr/&gt;&lt;p class=head style="display:block;"&gt;${SignatureLabel}&lt;/p&gt;&lt;hr/&gt;&lt;/div&gt;#end&lt;table class="dataTable" style="width:100%;table-layout:fixed;border-collapse:collapse;display:table;clear:both;"&gt;#if( $SignatureSectionVisible )&lt;tr&gt;&lt;td style="vertical-align:top;width:50%;"&gt;&lt;p class=headings&gt;#if( $SignatureCaptured )${SignatureCapturedLabel}#else${SignatureNotCapturedLabel}#end&lt;/p&gt;&lt;br/&gt;&lt;p&gt;#if( $SignatureCaptured )&lt;span style="color:#2E7D32;font-size:18px;"&gt;&amp;#10004;&lt;/span&gt; &lt;span style="color:#2E7D32;"&gt;${SignatureCapturedLabel}&lt;/span&gt;#else&lt;span style="color:#808080;font-size:18px;"&gt;&amp;#10007;&lt;/span&gt; &lt;span style="color:#808080;"&gt;${SignatureNotCapturedLabel}&lt;/span&gt;#end&lt;/p&gt;&lt;/td&gt;#if( $SignatureCaptured )&lt;td style="vertical-align:top;width:50%;"&gt;&lt;p class=headings&gt;${SignatureLabel}&lt;/p&gt;&lt;br/&gt;&lt;p&gt;&lt;img data-mosip-applicant-signature="1" src="${SignatureImageSource}" border="0" width="200" height="85" style="max-width:200px;max-height:85px;object-fit:contain;border:1px solid #b0b0b0;background:#fff;display:block;"/&gt;&lt;/p&gt;&lt;/td&gt;#else&lt;td style="vertical-align:top;width:50%;"&gt;&lt;/td&gt;#end&lt;/tr&gt;#end&lt;tr&gt;&lt;td&gt;&lt;p class=headings&gt;${RONameLabel}&lt;/p&gt;&lt;br/&gt;&lt;p&gt;${ROName}&lt;/p&gt;&lt;/td&gt;&lt;td&gt;&lt;p class=headings&gt;${RegCenterLabel}&lt;/p&gt;&lt;br/&gt;&lt;p&gt;${RegCenter}&lt;/p&gt;&lt;/td&gt;&lt;/tr&gt;&lt;/table&gt;&lt;hr/&gt;&lt;br/&gt;&lt;/div&gt;&lt;div&gt;&lt;p&gt;${ImportantGuidelines}&lt;/p&gt; &lt;ul&gt; #foreach( $line in $Guidelines ) &lt;li&gt;&lt;span&gt;${line}&lt;/span&gt;&lt;/li&gt; #end &lt;/ul&gt;&lt;/div&gt;&lt;/div&gt;&lt;/div&gt;&lt;/body&gt;&lt;/html&gt;</t>
-  </si>
-  <si>
-    <t>&lt;!DOCTYPE html&gt;&lt;html $rtl&gt;&lt;head&gt;&lt;meta charset="UTF-8"/&gt;&lt;style&gt;body,.head,.headings,th,td,p,b,strong{font-family:system-ui,"Segoe UI","Nirmala UI","Iskoola Pota","Latha",sans-serif;}table, .head{font-size:13px;}.demoDiv{width: 85%;float: left;}.photoDiv{width: 15%;float:right;}.form{display:inline-block;}.section{align:center;padding:30px;width:800px;margin:auto;}.headings{color:#808080;font-size:11px;}p{display:inline;}.dataTable{word-wrap:break-word;table-layout:fixed;width:70%;}.headerTable{width:90%;}.uinHeaderTable{width:100%;}h5{display:inline;position:absolute;}.iris{top:-15px;left:152px;}.irisWithoutException{top:-15px;left:114px;}.tableWithoutException{width:50%;text-align:center;table-layout:fixed;margin:0 auto;}.biometricsTable{width:100%;text-align:center;table-layout:fixed;}.biometrics{position:relative;}.leftLittle{top:15px;left:11px;display:inline;position:absolute;}.leftRing{top:3px;left:23px;}.leftMiddle{top:-7px;left:37px;}.leftIndex{top:3px;left:54px;}.rightIndex{top:3px;left:26px;}.rightMiddle{top:-7px;left:39px;}.rightRing{top:3px;left:55px;}.rightLittle{top:15px;left:68px;}.leftThumb{top:-4px;left:24px;}.rightThumb{top:-4px;left:54px;}.parentStyle{top:-15px;left:152px;}.parentIris1{top:-15px;left:212px;}.parentIris2{top:-15px;left:214px;}li span{color:black;font-size:12px;} li{color:lightgrey}button{float:right;font-size:12px;border:none;background-color:transparent;outline:none;}button:active{background-color:black;color:white;}.bottom{vertical-align:bottom;}.consent-block{font-size:13px;border-radius: 8px;margin-top: 10px;margin-bottom: 10px;border: 2px solid #E88E3F;padding-top: -50px;padding:10px;}.consent-text{margin-left: 7px;margin-bottom: 4px;}input[type="radio"] {display: none;} input[type="radio"] + label:before { content: ""; display: inline-block; width: 15px; height: 15px; padding: 3px; margin-right: 5px; background-clip: content-box; border: 1px solid grey; background-color: #fff; border-radius: 50%;}input[type="radio"]:checked + label:before { background-color: #FF4081; border-color:#FF4081;}*,*:before,*:after { box-sizing: border-box;}.consent-block label { display: inline-flex; align-items: center;}.demoDiv&gt;table{width:100%}.demoDiv&gt;table&gt;tbody&gt;tr&gt;th{color:#808080;font-size:10px; width:25%; text-align: left;padding: 2px}.demoDiv&gt;table&gt;tbody&gt;tr&gt;td{width:25%; text-align: left;padding: 2px}&lt;/style&gt;&lt;script&gt;function changeColour(element) { var div = document.getElementById("radioId"); if(element.value == "yes"){div.style = "border: 2px solid #68A933";} if(element.value == "no"){div.style = "border: 2px solid #FF0000";}} document.onreadystatechange = function () {if(document.readyState === "complete"){var body = document.getElementsByTagName("body")[0]; body.addEventListener("dragstart", function(event) {event.preventDefault();}); body.addEventListener("selectstart", function(event) {event.preventDefault();});}}&lt;/script&gt;&lt;/head&gt;&lt;body&gt; &lt;div class=section&gt; &lt;div class=form&gt; &lt;table class=headerTable&gt; &lt;tr&gt; &lt;td class=bottom&gt;&lt;p class=headings&gt;${ApplicationIDLabel}&lt;/p&gt;&lt;br/&gt;${ApplicationID}&lt;/td&gt; #if ( $UIN ) &lt;td class=bottom&gt;&lt;p class=headings&gt;${UINLabel}&lt;/p&gt;&lt;br/&gt;${UIN}&lt;/td&gt; #end &lt;td class=bottom&gt;&lt;p class=headings&gt;${DateLabel}&lt;/p&gt;&lt;br/&gt;${Date}&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; &lt;br/&gt; #if ( $name ) &lt;table class=headerTable&gt; &lt;tr&gt;&lt;td&gt;&lt;p class=headings&gt;${NameLabel}&lt;/p&gt;&lt;br/&gt;${NameValue}&lt;/td&gt;&lt;/tr&gt; &lt;/table&gt; #end &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;&lt;b&gt;${DemographicInfo}&lt;/b&gt;&lt;/p&gt;&lt;hr/&gt;&lt;div class="demoDiv"&gt;&lt;table&gt; &lt;tr&gt; #if( $demographics.get("fullName") ) &lt;th&gt;$demographics.get("fullName").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("fullName") ) &lt;td&gt;$demographics.get("fullName").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("dateOfBirth") ) &lt;th&gt;$demographics.get("dateOfBirth").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("dateOfBirth") ) &lt;td&gt;$demographics.get("dateOfBirth").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("gender") ) &lt;th&gt;$demographics.get("gender").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("gender") ) &lt;td&gt;$demographics.get("gender").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("phone") ) &lt;th&gt;$demographics.get("phone").get("label")&lt;/th&gt; #end #if( $demographics.get("email") ) &lt;th&gt;$demographics.get("email").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("phone") ) &lt;td&gt;$demographics.get("phone").get("value")&lt;/td&gt; #end #if( $demographics.get("email") ) &lt;td&gt;$demographics.get("email").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;/table&gt;&lt;table&gt; #if( $demographics.get("addressLine1") ) &lt;hr/&gt;&lt;h1 class="headings"&gt;Address&lt;/h1&gt; #end &lt;tr&gt; #if( $demographics.get("addressLine1") ) &lt;th&gt;$demographics.get("addressLine1").get("label")&lt;/th&gt; #end #if( $demographics.get("addressLine2") ) &lt;th&gt;$demographics.get("addressLine2").get("label")&lt;/th&gt; #end #if( $demographics.get("addressLine3") ) &lt;th&gt;$demographics.get("addressLine3").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("addressLine1") ) &lt;td&gt;$demographics.get("addressLine1").get("value")&lt;/td&gt; #end #if( $demographics.get("addressLine2") ) &lt;td&gt;$demographics.get("addressLine2").get("value")&lt;/td&gt; #end #if( $demographics.get("addressLine3") ) &lt;td&gt;$demographics.get("addressLine3").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;/table&gt;&lt;table&gt;&lt;tr&gt; #if( $demographics.get("region") ) &lt;th&gt;$demographics.get("region").get("label")&lt;/th&gt; #end #if( $demographics.get("province") ) &lt;th&gt;$demographics.get("province").get("label")&lt;/th&gt; #end #if( $demographics.get("city") ) &lt;th&gt;$demographics.get("city").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("region") ) &lt;td&gt;$demographics.get("region").get("value")&lt;/td&gt; #end #if( $demographics.get("province") ) &lt;td&gt;$demographics.get("province").get("value")&lt;/td&gt; #end #if( $demographics.get("city") ) &lt;td&gt;$demographics.get("city").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;/table&gt;&lt;table&gt;&lt;tr&gt; #if( $demographics.get("zone") ) &lt;th&gt;$demographics.get("zone").get("label")&lt;/th&gt; #end #if( $demographics.get("postalCode") ) &lt;th&gt;$demographics.get("postalCode").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("zone") ) &lt;td&gt;$demographics.get("zone").get("value")&lt;/td&gt; #end #if( $demographics.get("postalCode") ) &lt;td&gt;$demographics.get("postalCode").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("modeOfClaim") ) &lt;th&gt;$demographics.get("modeOfClaim").get("label")&lt;/th&gt; #end&lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("modeOfClaim") ) &lt;td&gt;$demographics.get("modeOfClaim").get("value")&lt;/td&gt; #end&lt;/tr&gt;&lt;/table&gt; #if( $demographics.get("parentOrGuardianName") ) &lt;hr/&gt; &lt;table&gt; &lt;h1 class="headings"&gt;Gaurdian Details&lt;/h1&gt;&lt;tr&gt;&lt;th&gt;$demographics.get("parentOrGuardianName").get("label")&lt;/th&gt; #if( $demographics.get("parentOrGuardianRID") ) &lt;th&gt;$demographics.get("parentOrGuardianRID").get("label")&lt;/th&gt; #end #if( $demographics.get("parentOrGuardianUIN") ) &lt;th&gt;$demographics.get("parentOrGuardianUIN").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt;&lt;td&gt;$demographics.get("parentOrGuardianName").get("value")&lt;/td&gt; #if( $demographics.get("parentOrGuardianRID") ) &lt;td&gt;$demographics.get("parentOrGuardianRID").get("value")&lt;/td&gt; #end #if( $demographics.get("parentOrGuardianUIN") ) &lt;td&gt;$demographics.get("parentOrGuardianUIN").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;/table&gt; #end &lt;/div&gt; #if ( $ApplicantImageSource ) &lt;div class="photoDiv"&gt; &lt;table&gt; &lt;tr&gt; &lt;td&gt; &lt;p&gt;${Photo}&lt;/p&gt; &lt;/td&gt; &lt;/tr&gt; &lt;tr&gt; &lt;td&gt;&lt;img src="${ApplicantImageSource}" border=0 width=100 height=100/&gt;&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; &lt;/div&gt; #end &lt;div style="width: 100%; height: 50%; clear:both"&gt;&lt;/div&gt; &lt;br&gt; &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;&lt;b&gt;${DocumentsLabel}&lt;/b&gt;&lt;/p&gt; &lt;hr/&gt; &lt;table class=dataTable&gt; #foreach( $key in $documents.keySet() ) &lt;tr&gt; &lt;td&gt; &lt;p class=headings&gt;$documents.get($key).get("label")&lt;/p&gt; &lt;br/&gt; &lt;p&gt; $documents.get($key).get("value")&lt;/p&gt; &lt;/td&gt; &lt;/tr&gt; #end &lt;/table&gt; &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;&lt;b&gt;${BiometricsLabel}&lt;/b&gt;&lt;/p&gt; &lt;hr/&gt; #foreach( $key in $biometrics.keySet() ) &lt;table&gt; &lt;tr&gt; &lt;td&gt; $biometrics.get($key).get("label")&lt;br/&gt; &lt;p class=headings&gt;${Fingers} ( $biometrics.get($key).get("FingerCount") ),${Iris} ( $biometrics.get($key).get("IrisCount") ),${Face} ( $biometrics.get($key).get("FaceCount") )&lt;br/&gt;&lt;/p&gt; &lt;br/&gt; &lt;/td&gt; &lt;/tr&gt;&lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftEye") ) &lt;td&gt;&lt;p class=headings&gt;${LeftEyeLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightEye") ) &lt;td&gt; &lt;p class=headings&gt;${RightEyeLabel}&lt;/p&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftEye") ) &lt;td&gt; #if( $biometrics.get($key).get("CapturedLeftEye") ) &lt;img src='$biometrics.get($key).get("CapturedLeftEye")' border=0 width=85 height=80/&gt; #end &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightEye") ) &lt;td&gt; #if( $biometrics.get($key).get("CapturedRightEye") ) &lt;img src='$biometrics.get($key).get("CapturedRightEye")' border=0 width=85 height=80/&gt; #end &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftSlap") ) &lt;td&gt; &lt;p class=headings&gt;${LeftPalmLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightSlap") ) &lt;td&gt; &lt;p class=headings&gt;${RightPalmLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedThumbs") ) &lt;td&gt; &lt;p class=headings&gt;${ThumbsLabel}&lt;/p&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftSlap") ) &lt;td style="text-align:-webkit-center"&gt; &lt;img src='$biometrics.get($key).get("CapturedLeftSlap")' border=0 width=85 height=80/&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightSlap") ) &lt;td style="text-align:-webkit-center"&gt; &lt;img src='$biometrics.get($key).get("CapturedRightSlap")' border=0 width=85 height=80/&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedThumbs") ) &lt;td style="text-align:-webkit-center"&gt; &lt;img src='$biometrics.get($key).get("CapturedThumbs")' border=0 width=85 height=80/&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;br/&gt; &lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("FaceImageSource") ) &lt;td&gt; &lt;p class=headings&gt;${FaceLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("subType") == "applicant" &amp;&amp; $ExceptionImageSource ) &lt;td&gt; &lt;p class=headings&gt;${ExceptionPhotoLabel}&lt;/p&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;tr&gt; #if( $biometrics.get($key).get("FaceImageSource") ) &lt;td&gt; &lt;img src='$biometrics.get($key).get("FaceImageSource")' border=0 width=85 height=80/&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("subType") == "applicant" &amp;&amp; $ExceptionImageSource ) &lt;td&gt; &lt;img src="${ExceptionImageSource}" border=0 width=85 height=80/&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;/table&gt; #end &lt;br/&gt; &lt;/div&gt; &lt;/body&gt; &lt;/html&gt;</t>
-  </si>
-  <si>
-    <t>&lt;!DOCTYPE html&gt;&lt;html $rtl&gt;&lt;head&gt;&lt;meta charset="UTF-8"/&gt;&lt;style&gt;body,.head,.headings,th,td,p,b,strong{font-family:system-ui,"Segoe UI","Nirmala UI","Iskoola Pota","Latha",sans-serif;}table, .head{font-size:13px;}.demoDiv{width: 85%;float: left;}.photoDiv{width: 15%;float:right;}.form{display:inline-block;}.section{align:center;padding:30px;width:800px;margin:auto;}.headings{color:#808080;font-size:11px;}p{display:inline;}.dataTable{word-wrap:break-word;table-layout:fixed;width:70%;}.headerTable{width:90%;}.uinHeaderTable{width:100%;}h5{display:inline;position:absolute;}.iris{top:-15px;left:152px;}.irisWithoutException{top:-15px;left:114px;}.tableWithoutException{width:50%;text-align:center;table-layout:fixed;margin:0 auto;}.biometricsTable{width:100%;text-align:center;table-layout:fixed;}.biometrics{position:relative;}.leftLittle{top:15px;left:11px;display:inline;position:absolute;}.leftRing{top:3px;left:23px;}.leftMiddle{top:-7px;left:37px;}.leftIndex{top:3px;left:54px;}.rightIndex{top:3px;left:26px;}.rightMiddle{top:-7px;left:39px;}.rightRing{top:3px;left:55px;}.rightLittle{top:15px;left:68px;}.leftThumb{top:-4px;left:24px;}.rightThumb{top:-4px;left:54px;}.parentStyle{top:-15px;left:152px;}.parentIris1{top:-15px;left:212px;}.parentIris2{top:-15px;left:214px;}li span{color:black;font-size:12px;} li{color:lightgrey}button{float:right;font-size:12px;border:none;background-color:transparent;outline:none;}button:active{background-color:black;color:white;}.bottom{vertical-align:bottom;}.consent-block{font-size:13px;border-radius: 8px;margin-top: 10px;margin-bottom: 10px;border: 2px solid #E88E3F;padding-top: -50px;padding:10px;}.consent-text{margin-left: 7px;margin-bottom: 4px;}input[type="radio"] {display: none;} input[type="radio"] + label:before { content: ""; display: inline-block; width: 15px; height: 15px; padding: 3px; margin-right: 5px; background-clip: content-box; border: 1px solid grey; background-color: #fff; border-radius: 50%;}input[type="radio"]:checked + label:before { background-color: #FF4081; border-color:#FF4081;}*,*:before,*:after { box-sizing: border-box;}.consent-block label { display: inline-flex; align-items: center;}.demoDiv&gt;table{width:100%}.demoDiv&gt;table&gt;tbody&gt;tr&gt;th{color:#808080;font-size:10px; width:25%; text-align: left;padding: 2px}.demoDiv&gt;table&gt;tbody&gt;tr&gt;td{width:25%; text-align: left;padding: 2px}&lt;/style&gt;&lt;script&gt;function changeColour(element) { var div = document.getElementById("radioId"); if(element.value == "yes"){div.style = "border: 2px solid #68A933";} if(element.value == "no"){div.style = "border: 2px solid #FF0000";}} document.onreadystatechange = function () {if(document.readyState === "complete"){var body = document.getElementsByTagName("body")[0]; body.addEventListener("dragstart", function(event) {event.preventDefault();}); body.addEventListener("selectstart", function(event) {event.preventDefault();});}}&lt;/script&gt;&lt;/head&gt;&lt;body&gt; &lt;div class=section&gt; &lt;div class=form&gt; &lt;table class=headerTable&gt; &lt;tr&gt; &lt;td class=bottom&gt;&lt;p class=headings&gt;${ApplicationIDLabel}&lt;/p&gt;&lt;br/&gt;${ApplicationID}&lt;/td&gt; #if ( $UIN ) &lt;td class=bottom&gt;&lt;p class=headings&gt;${UINLabel}&lt;/p&gt;&lt;br/&gt;${UIN}&lt;/td&gt; #end &lt;td class=bottom&gt;&lt;p class=headings&gt;${DateLabel}&lt;/p&gt;&lt;br/&gt;${Date}&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; &lt;br/&gt; #if ( $name ) &lt;table class=headerTable&gt; &lt;tr&gt;&lt;td&gt;&lt;p class=headings&gt;${NameLabel}&lt;/p&gt;&lt;br/&gt;${NameValue}&lt;/td&gt;&lt;/tr&gt; &lt;/table&gt; #end &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;&lt;b&gt;${DemographicInfo}&lt;/b&gt;&lt;/p&gt;&lt;hr/&gt;&lt;div class="demoDiv"&gt;&lt;table&gt; &lt;tr&gt; #if( $demographics.get("fullName") ) &lt;th&gt;$demographics.get("fullName").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("fullName") ) &lt;td&gt;$demographics.get("fullName").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("dateOfBirth") ) &lt;th&gt;$demographics.get("dateOfBirth").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("dateOfBirth") ) &lt;td&gt;$demographics.get("dateOfBirth").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("gender") ) &lt;th&gt;$demographics.get("gender").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("gender") ) &lt;td&gt;$demographics.get("gender").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("phone") ) &lt;th&gt;$demographics.get("phone").get("label")&lt;/th&gt; #end #if( $demographics.get("email") ) &lt;th&gt;$demographics.get("email").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("phone") ) &lt;td&gt;$demographics.get("phone").get("value")&lt;/td&gt; #end #if( $demographics.get("email") ) &lt;td&gt;$demographics.get("email").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;/table&gt;&lt;table&gt; #if( $demographics.get("addressLine1") ) &lt;hr/&gt;&lt;h1 class="headings"&gt;ලිපිනය&lt;/h1&gt; #end &lt;tr&gt; #if( $demographics.get("addressLine1") ) &lt;th&gt;$demographics.get("addressLine1").get("label")&lt;/th&gt; #end #if( $demographics.get("addressLine2") ) &lt;th&gt;$demographics.get("addressLine2").get("label")&lt;/th&gt; #end #if( $demographics.get("addressLine3") ) &lt;th&gt;$demographics.get("addressLine3").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("addressLine1") ) &lt;td&gt;$demographics.get("addressLine1").get("value")&lt;/td&gt; #end #if( $demographics.get("addressLine2") ) &lt;td&gt;$demographics.get("addressLine2").get("value")&lt;/td&gt; #end #if( $demographics.get("addressLine3") ) &lt;td&gt;$demographics.get("addressLine3").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;/table&gt;&lt;table&gt;&lt;tr&gt; #if( $demographics.get("region") ) &lt;th&gt;$demographics.get("region").get("label")&lt;/th&gt; #end #if( $demographics.get("province") ) &lt;th&gt;$demographics.get("province").get("label")&lt;/th&gt; #end #if( $demographics.get("city") ) &lt;th&gt;$demographics.get("city").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("region") ) &lt;td&gt;$demographics.get("region").get("value")&lt;/td&gt; #end #if( $demographics.get("province") ) &lt;td&gt;$demographics.get("province").get("value")&lt;/td&gt; #end #if( $demographics.get("city") ) &lt;td&gt;$demographics.get("city").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;/table&gt;&lt;table&gt;&lt;tr&gt; #if( $demographics.get("zone") ) &lt;th&gt;$demographics.get("zone").get("label")&lt;/th&gt; #end #if( $demographics.get("postalCode") ) &lt;th&gt;$demographics.get("postalCode").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("zone") ) &lt;td&gt;$demographics.get("zone").get("value")&lt;/td&gt; #end #if( $demographics.get("postalCode") ) &lt;td&gt;$demographics.get("postalCode").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("modeOfClaim") ) &lt;th&gt;$demographics.get("modeOfClaim").get("label")&lt;/th&gt; #end&lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("modeOfClaim") ) &lt;td&gt;$demographics.get("modeOfClaim").get("value")&lt;/td&gt; #end&lt;/tr&gt;&lt;/table&gt; #if( $demographics.get("parentOrGuardianName") ) &lt;hr/&gt; &lt;table&gt; &lt;h1 class="headings"&gt;මාපිය/භාරකරු විස්තර&lt;/h1&gt;&lt;tr&gt;&lt;th&gt;$demographics.get("parentOrGuardianName").get("label")&lt;/th&gt; #if( $demographics.get("parentOrGuardianRID") ) &lt;th&gt;$demographics.get("parentOrGuardianRID").get("label")&lt;/th&gt; #end #if( $demographics.get("parentOrGuardianUIN") ) &lt;th&gt;$demographics.get("parentOrGuardianUIN").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt;&lt;td&gt;$demographics.get("parentOrGuardianName").get("value")&lt;/td&gt; #if( $demographics.get("parentOrGuardianRID") ) &lt;td&gt;$demographics.get("parentOrGuardianRID").get("value")&lt;/td&gt; #end #if( $demographics.get("parentOrGuardianUIN") ) &lt;td&gt;$demographics.get("parentOrGuardianUIN").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;/table&gt; #end &lt;/div&gt; #if ( $ApplicantImageSource ) &lt;div class="photoDiv"&gt; &lt;table&gt; &lt;tr&gt; &lt;td&gt; &lt;p&gt;${Photo}&lt;/p&gt; &lt;/td&gt; &lt;/tr&gt; &lt;tr&gt; &lt;td&gt;&lt;img src="${ApplicantImageSource}" border=0 width=100 height=100/&gt;&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; &lt;/div&gt; #end &lt;div style="width: 100%; height: 50%; clear:both"&gt;&lt;/div&gt; &lt;br&gt; &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;&lt;b&gt;${DocumentsLabel}&lt;/b&gt;&lt;/p&gt; &lt;hr/&gt; &lt;table class=dataTable&gt; #foreach( $key in $documents.keySet() ) &lt;tr&gt; &lt;td&gt; &lt;p class=headings&gt;$documents.get($key).get("label")&lt;/p&gt; &lt;br/&gt; &lt;p&gt; $documents.get($key).get("value")&lt;/p&gt; &lt;/td&gt; &lt;/tr&gt; #end &lt;/table&gt; &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;&lt;b&gt;${BiometricsLabel}&lt;/b&gt;&lt;/p&gt; &lt;hr/&gt; #foreach( $key in $biometrics.keySet() ) &lt;table&gt; &lt;tr&gt; &lt;td&gt; $biometrics.get($key).get("label")&lt;br/&gt; &lt;p class=headings&gt;${Fingers} ( $biometrics.get($key).get("FingerCount") ),${Iris} ( $biometrics.get($key).get("IrisCount") ),${Face} ( $biometrics.get($key).get("FaceCount") )&lt;br/&gt;&lt;/p&gt; &lt;br/&gt; &lt;/td&gt; &lt;/tr&gt;&lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftEye") ) &lt;td&gt;&lt;p class=headings&gt;${LeftEyeLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightEye") ) &lt;td&gt; &lt;p class=headings&gt;${RightEyeLabel}&lt;/p&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftEye") ) &lt;td&gt; #if( $biometrics.get($key).get("CapturedLeftEye") ) &lt;img src='$biometrics.get($key).get("CapturedLeftEye")' border=0 width=85 height=80/&gt; #end &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightEye") ) &lt;td&gt; #if( $biometrics.get($key).get("CapturedRightEye") ) &lt;img src='$biometrics.get($key).get("CapturedRightEye")' border=0 width=85 height=80/&gt; #end &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftSlap") ) &lt;td&gt; &lt;p class=headings&gt;${LeftPalmLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightSlap") ) &lt;td&gt; &lt;p class=headings&gt;${RightPalmLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedThumbs") ) &lt;td&gt; &lt;p class=headings&gt;${ThumbsLabel}&lt;/p&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftSlap") ) &lt;td style="text-align:-webkit-center"&gt; &lt;img src='$biometrics.get($key).get("CapturedLeftSlap")' border=0 width=85 height=80/&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightSlap") ) &lt;td style="text-align:-webkit-center"&gt; &lt;img src='$biometrics.get($key).get("CapturedRightSlap")' border=0 width=85 height=80/&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedThumbs") ) &lt;td style="text-align:-webkit-center"&gt; &lt;img src='$biometrics.get($key).get("CapturedThumbs")' border=0 width=85 height=80/&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;br/&gt; &lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("FaceImageSource") ) &lt;td&gt; &lt;p class=headings&gt;${FaceLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("subType") == "applicant" &amp;&amp; $ExceptionImageSource ) &lt;td&gt; &lt;p class=headings&gt;${ExceptionPhotoLabel}&lt;/p&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;tr&gt; #if( $biometrics.get($key).get("FaceImageSource") ) &lt;td&gt; &lt;img src='$biometrics.get($key).get("FaceImageSource")' border=0 width=85 height=80/&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("subType") == "applicant" &amp;&amp; $ExceptionImageSource ) &lt;td&gt; &lt;img src="${ExceptionImageSource}" border=0 width=85 height=80/&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;/table&gt; #end &lt;br/&gt; &lt;/div&gt; &lt;/body&gt; &lt;/html&gt;</t>
-  </si>
-  <si>
-    <t>&lt;!DOCTYPE html&gt;&lt;html $rtl&gt;&lt;head&gt;&lt;meta charset="UTF-8"/&gt;&lt;style&gt;body,.head,.headings,th,td,p,b,strong{font-family:system-ui,"Segoe UI","Nirmala UI","Iskoola Pota","Latha",sans-serif;}table, .head{font-size:13px;}.demoDiv{width: 85%;float: left;}.photoDiv{width: 15%;float:right;}.form{display:inline-block;}.section{align:center;padding:30px;width:800px;margin:auto;}.headings{color:#808080;font-size:11px;}p{display:inline;}.dataTable{word-wrap:break-word;table-layout:fixed;width:70%;}.headerTable{width:90%;}.uinHeaderTable{width:100%;}h5{display:inline;position:absolute;}.iris{top:-15px;left:152px;}.irisWithoutException{top:-15px;left:114px;}.tableWithoutException{width:50%;text-align:center;table-layout:fixed;margin:0 auto;}.biometricsTable{width:100%;text-align:center;table-layout:fixed;}.biometrics{position:relative;}.leftLittle{top:15px;left:11px;display:inline;position:absolute;}.leftRing{top:3px;left:23px;}.leftMiddle{top:-7px;left:37px;}.leftIndex{top:3px;left:54px;}.rightIndex{top:3px;left:26px;}.rightMiddle{top:-7px;left:39px;}.rightRing{top:3px;left:55px;}.rightLittle{top:15px;left:68px;}.leftThumb{top:-4px;left:24px;}.rightThumb{top:-4px;left:54px;}.parentStyle{top:-15px;left:152px;}.parentIris1{top:-15px;left:212px;}.parentIris2{top:-15px;left:214px;}li span{color:black;font-size:12px;} li{color:lightgrey}button{float:right;font-size:12px;border:none;background-color:transparent;outline:none;}button:active{background-color:black;color:white;}.bottom{vertical-align:bottom;}.consent-block{font-size:13px;border-radius: 8px;margin-top: 10px;margin-bottom: 10px;border: 2px solid #E88E3F;padding-top: -50px;padding:10px;}.consent-text{margin-left: 7px;margin-bottom: 4px;}input[type="radio"] {display: none;} input[type="radio"] + label:before { content: ""; display: inline-block; width: 15px; height: 15px; padding: 3px; margin-right: 5px; background-clip: content-box; border: 1px solid grey; background-color: #fff; border-radius: 50%;}input[type="radio"]:checked + label:before { background-color: #FF4081; border-color:#FF4081;}*,*:before,*:after { box-sizing: border-box;}.consent-block label { display: inline-flex; align-items: center;}.demoDiv&gt;table{width:100%}.demoDiv&gt;table&gt;tbody&gt;tr&gt;th{color:#808080;font-size:10px; width:25%; text-align: left;padding: 2px}.demoDiv&gt;table&gt;tbody&gt;tr&gt;td{width:25%; text-align: left;padding: 2px}&lt;/style&gt;&lt;script&gt;function changeColour(element) { var div = document.getElementById("radioId"); if(element.value == "yes"){div.style = "border: 2px solid #68A933";} if(element.value == "no"){div.style = "border: 2px solid #FF0000";}} document.onreadystatechange = function () {if(document.readyState === "complete"){var body = document.getElementsByTagName("body")[0]; body.addEventListener("dragstart", function(event) {event.preventDefault();}); body.addEventListener("selectstart", function(event) {event.preventDefault();});}}&lt;/script&gt;&lt;/head&gt;&lt;body&gt; &lt;div class=section&gt; &lt;div class=form&gt; &lt;table class=headerTable&gt; &lt;tr&gt; &lt;td class=bottom&gt;&lt;p class=headings&gt;${ApplicationIDLabel}&lt;/p&gt;&lt;br/&gt;${ApplicationID}&lt;/td&gt; #if ( $UIN ) &lt;td class=bottom&gt;&lt;p class=headings&gt;${UINLabel}&lt;/p&gt;&lt;br/&gt;${UIN}&lt;/td&gt; #end &lt;td class=bottom&gt;&lt;p class=headings&gt;${DateLabel}&lt;/p&gt;&lt;br/&gt;${Date}&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; &lt;br/&gt; #if ( $name ) &lt;table class=headerTable&gt; &lt;tr&gt;&lt;td&gt;&lt;p class=headings&gt;${NameLabel}&lt;/p&gt;&lt;br/&gt;${NameValue}&lt;/td&gt;&lt;/tr&gt; &lt;/table&gt; #end &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;&lt;b&gt;${DemographicInfo}&lt;/b&gt;&lt;/p&gt;&lt;hr/&gt;&lt;div class="demoDiv"&gt;&lt;table&gt; &lt;tr&gt; #if( $demographics.get("fullName") ) &lt;th&gt;$demographics.get("fullName").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("fullName") ) &lt;td&gt;$demographics.get("fullName").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("dateOfBirth") ) &lt;th&gt;$demographics.get("dateOfBirth").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("dateOfBirth") ) &lt;td&gt;$demographics.get("dateOfBirth").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("gender") ) &lt;th&gt;$demographics.get("gender").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("gender") ) &lt;td&gt;$demographics.get("gender").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("phone") ) &lt;th&gt;$demographics.get("phone").get("label")&lt;/th&gt; #end #if( $demographics.get("email") ) &lt;th&gt;$demographics.get("email").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("phone") ) &lt;td&gt;$demographics.get("phone").get("value")&lt;/td&gt; #end #if( $demographics.get("email") ) &lt;td&gt;$demographics.get("email").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;/table&gt;&lt;table&gt; #if( $demographics.get("addressLine1") ) &lt;hr/&gt;&lt;h1 class="headings"&gt;முகவரி&lt;/h1&gt; #end &lt;tr&gt; #if( $demographics.get("addressLine1") ) &lt;th&gt;$demographics.get("addressLine1").get("label")&lt;/th&gt; #end #if( $demographics.get("addressLine2") ) &lt;th&gt;$demographics.get("addressLine2").get("label")&lt;/th&gt; #end #if( $demographics.get("addressLine3") ) &lt;th&gt;$demographics.get("addressLine3").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("addressLine1") ) &lt;td&gt;$demographics.get("addressLine1").get("value")&lt;/td&gt; #end #if( $demographics.get("addressLine2") ) &lt;td&gt;$demographics.get("addressLine2").get("value")&lt;/td&gt; #end #if( $demographics.get("addressLine3") ) &lt;td&gt;$demographics.get("addressLine3").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;/table&gt;&lt;table&gt;&lt;tr&gt; #if( $demographics.get("region") ) &lt;th&gt;$demographics.get("region").get("label")&lt;/th&gt; #end #if( $demographics.get("province") ) &lt;th&gt;$demographics.get("province").get("label")&lt;/th&gt; #end #if( $demographics.get("city") ) &lt;th&gt;$demographics.get("city").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("region") ) &lt;td&gt;$demographics.get("region").get("value")&lt;/td&gt; #end #if( $demographics.get("province") ) &lt;td&gt;$demographics.get("province").get("value")&lt;/td&gt; #end #if( $demographics.get("city") ) &lt;td&gt;$demographics.get("city").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;/table&gt;&lt;table&gt;&lt;tr&gt; #if( $demographics.get("zone") ) &lt;th&gt;$demographics.get("zone").get("label")&lt;/th&gt; #end #if( $demographics.get("postalCode") ) &lt;th&gt;$demographics.get("postalCode").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("zone") ) &lt;td&gt;$demographics.get("zone").get("value")&lt;/td&gt; #end #if( $demographics.get("postalCode") ) &lt;td&gt;$demographics.get("postalCode").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("modeOfClaim") ) &lt;th&gt;$demographics.get("modeOfClaim").get("label")&lt;/th&gt; #end&lt;/tr&gt;&lt;tr&gt; #if( $demographics.get("modeOfClaim") ) &lt;td&gt;$demographics.get("modeOfClaim").get("value")&lt;/td&gt; #end&lt;/tr&gt;&lt;/table&gt; #if( $demographics.get("parentOrGuardianName") ) &lt;hr/&gt; &lt;table&gt; &lt;h1 class="headings"&gt;பெற்றோர்/பாதுகாவலர் விவரங்கள்&lt;/h1&gt;&lt;tr&gt;&lt;th&gt;$demographics.get("parentOrGuardianName").get("label")&lt;/th&gt; #if( $demographics.get("parentOrGuardianRID") ) &lt;th&gt;$demographics.get("parentOrGuardianRID").get("label")&lt;/th&gt; #end #if( $demographics.get("parentOrGuardianUIN") ) &lt;th&gt;$demographics.get("parentOrGuardianUIN").get("label")&lt;/th&gt; #end &lt;/tr&gt;&lt;tr&gt;&lt;td&gt;$demographics.get("parentOrGuardianName").get("value")&lt;/td&gt; #if( $demographics.get("parentOrGuardianRID") ) &lt;td&gt;$demographics.get("parentOrGuardianRID").get("value")&lt;/td&gt; #end #if( $demographics.get("parentOrGuardianUIN") ) &lt;td&gt;$demographics.get("parentOrGuardianUIN").get("value")&lt;/td&gt; #end &lt;/tr&gt;&lt;/table&gt; #end &lt;/div&gt; #if ( $ApplicantImageSource ) &lt;div class="photoDiv"&gt; &lt;table&gt; &lt;tr&gt; &lt;td&gt; &lt;p&gt;${Photo}&lt;/p&gt; &lt;/td&gt; &lt;/tr&gt; &lt;tr&gt; &lt;td&gt;&lt;img src="${ApplicantImageSource}" border=0 width=100 height=100/&gt;&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; &lt;/div&gt; #end &lt;div style="width: 100%; height: 50%; clear:both"&gt;&lt;/div&gt; &lt;br&gt; &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;&lt;b&gt;${DocumentsLabel}&lt;/b&gt;&lt;/p&gt; &lt;hr/&gt; &lt;table class=dataTable&gt; #foreach( $key in $documents.keySet() ) &lt;tr&gt; &lt;td&gt; &lt;p class=headings&gt;$documents.get($key).get("label")&lt;/p&gt; &lt;br/&gt; &lt;p&gt; $documents.get($key).get("value")&lt;/p&gt; &lt;/td&gt; &lt;/tr&gt; #end &lt;/table&gt; &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;&lt;b&gt;${BiometricsLabel}&lt;/b&gt;&lt;/p&gt; &lt;hr/&gt; #foreach( $key in $biometrics.keySet() ) &lt;table&gt; &lt;tr&gt; &lt;td&gt; $biometrics.get($key).get("label")&lt;br/&gt; &lt;p class=headings&gt;${Fingers} ( $biometrics.get($key).get("FingerCount") ),${Iris} ( $biometrics.get($key).get("IrisCount") ),${Face} ( $biometrics.get($key).get("FaceCount") )&lt;br/&gt;&lt;/p&gt; &lt;br/&gt; &lt;/td&gt; &lt;/tr&gt;&lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftEye") ) &lt;td&gt;&lt;p class=headings&gt;${LeftEyeLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightEye") ) &lt;td&gt; &lt;p class=headings&gt;${RightEyeLabel}&lt;/p&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftEye") ) &lt;td&gt; #if( $biometrics.get($key).get("CapturedLeftEye") ) &lt;img src='$biometrics.get($key).get("CapturedLeftEye")' border=0 width=85 height=80/&gt; #end &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightEye") ) &lt;td&gt; #if( $biometrics.get($key).get("CapturedRightEye") ) &lt;img src='$biometrics.get($key).get("CapturedRightEye")' border=0 width=85 height=80/&gt; #end &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftSlap") ) &lt;td&gt; &lt;p class=headings&gt;${LeftPalmLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightSlap") ) &lt;td&gt; &lt;p class=headings&gt;${RightPalmLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedThumbs") ) &lt;td&gt; &lt;p class=headings&gt;${ThumbsLabel}&lt;/p&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftSlap") ) &lt;td style="text-align:-webkit-center"&gt; &lt;img src='$biometrics.get($key).get("CapturedLeftSlap")' border=0 width=85 height=80/&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightSlap") ) &lt;td style="text-align:-webkit-center"&gt; &lt;img src='$biometrics.get($key).get("CapturedRightSlap")' border=0 width=85 height=80/&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedThumbs") ) &lt;td style="text-align:-webkit-center"&gt; &lt;img src='$biometrics.get($key).get("CapturedThumbs")' border=0 width=85 height=80/&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;br/&gt; &lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("FaceImageSource") ) &lt;td&gt; &lt;p class=headings&gt;${FaceLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("subType") == "applicant" &amp;&amp; $ExceptionImageSource ) &lt;td&gt; &lt;p class=headings&gt;${ExceptionPhotoLabel}&lt;/p&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;tr&gt; #if( $biometrics.get($key).get("FaceImageSource") ) &lt;td&gt; &lt;img src='$biometrics.get($key).get("FaceImageSource")' border=0 width=85 height=80/&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("subType") == "applicant" &amp;&amp; $ExceptionImageSource ) &lt;td&gt; &lt;img src="${ExceptionImageSource}" border=0 width=85 height=80/&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;/table&gt; #end &lt;br/&gt; &lt;/div&gt; &lt;/body&gt; &lt;/html&gt;</t>
+    <t xml:space="preserve">&lt;!DOCTYPE html&gt;&lt;html $rtl&gt;&lt;head&gt;&lt;meta charset="UTF-8"/&gt;&lt;style&gt;body,.head,.headings,th,td,p,b,strong{font-family:system-ui,"Segoe UI","Nirmala UI","Iskoola Pota","Latha",sans-serif;}table, .head{font-size:13px;}.demoDiv{width: 85%;float: left;}.photoDiv{width: 15%;float:right;}.form{display:block;width:100%;}.section{padding:24px;width:800px;max-width:800px;margin-left:auto;margin-right:auto;box-sizing:border-box;}.headings{color:#808080;font-size:11px;}p{display:inline;}.dataTable{word-wrap:break-word;table-layout:fixed;width:100%;}.headerTable{width:90%;}.uinHeaderTable{width:100%;}h5{display:inline;position:absolute;}.iris{top:-15px;left:152px;}.irisWithoutException{top:-15px;left:114px;}.tableWithoutException{width:50%;text-align:center;table-layout:fixed;margin:0 auto;}.biometricsTable{width:100%;text-align:center;table-layout:fixed;}.biometrics{position:relative;}.leftLittle{top:15px;left:11px;display:inline;position:absolute;}.leftRing{top:3px;left:23px;}.leftMiddle{top:-7px;left:37px;}.leftIndex{top:3px;left:54px;}.rightIndex{top:3px;left:26px;}.rightMiddle{top:-7px;left:39px;}.rightRing{top:3px;left:55px;}.rightLittle{top:15px;left:68px;}.leftThumb{top:-4px;left:24px;}.rightThumb{top:-4px;left:54px;}.parentStyle{top:-15px;left:152px;}.parentIris1{top:-15px;left:212px;}.parentIris2{top:-15px;left:214px;}li span{color:black;font-size:12px;} li{color:lightgrey}button{float:right;font-size:12px;border:none;background-color:transparent;outline:none;}button:active{background-color:black;color:white;} .bottom{vertical-align:bottom;}.consent-block{font-size:13px;border-radius: 8px;margin-top: 10px;margin-bottom: 10px;border: 2px solid #E88E3F;padding-top: -50px;padding:10px;}.consent-text{margin-left: 7px;margin-bottom: 4px;}input[type="radio"] {display: none;} input[type="radio"] + label:before { content: ""; display: inline-block; width: 15px; height: 15px; padding: 3px; margin-right: 5px; background-clip: content-box; border: 1px solid grey; background-color: #fff; border-radius: 50%;}input[type="radio"]:checked + label:before { background-color: #FF4081; border-color:#FF4081;}*,*:before,*:after { box-sizing: border-box;}.consent-block label { display: inline-flex; align-items: center;}.demoDiv&gt;table{width:100%}.demoDiv&gt;table&gt;tbody&gt;tr&gt;th{color:#808080;font-size:10px; width:25%; text-align: left;padding: 2px;font-weight:normal;}.demoDiv&gt;table&gt;tbody&gt;tr&gt;td{width:25%; text-align: left;padding: 2px}.ackPostBioBlock{display:block;clear:both;width:100%!important;max-width:100%;}.ackPostBioBlock hr{width:100%;}.ackPostBioBlock .dataTable{width:100%!important;max-width:100%;table-layout:fixed;border-collapse:collapse;display:table!important;}.ackPostBioBlock .headings,.ackPostBioBlock p.head,.ackPostBioBlock td&gt;p{display:block;}.demoSection{display:block;color:#808080;font-size:11px;font-weight:bold;margin:12px 0 4px 0;}.demoDiv&gt;p.demoSection:first-child{margin-top:0;}.demoDiv&gt;table&gt;tbody&gt;tr&gt;th{font-weight:normal;}&lt;/style&gt;&lt;script&gt;function changeColour(element) { var div = document.getElementById("radioId"); if(element.value == "yes"){div.style = "border: 2px solid #68A933";} if(element.value == "no"){div.style = "border: 2px solid #FF0000";}} document.onreadystatechange = function () {if(document.readyState === "complete"){var body = document.getElementsByTagName("body")[0]; body.addEventListener("dragstart", function(event) {event.preventDefault();}); body.addEventListener("selectstart", function(event) {event.preventDefault();});}}&lt;/script&gt;&lt;/head&gt; &lt;body&gt; &lt;div class=section&gt; &lt;div class=form&gt; &lt;table class=headerTable&gt; &lt;tr&gt; #if ( !$isPreview &amp;&amp; $QRCodeSource ) &lt;td class=bottom&gt; &lt;img src="${QRCodeSource}" width=85 height=85/&gt; &lt;/td&gt; #end &lt;td class=bottom&gt;&lt;p class=headings&gt;${ApplicationIDLabel}&lt;/p&gt;&lt;br/&gt;${ApplicationID}&lt;/td&gt; #if ( $UIN ) &lt;td class=bottom&gt;&lt;p class=headings&gt;${UINLabel}&lt;/p&gt;&lt;br/&gt;${UIN}&lt;/td&gt; #end &lt;td class=bottom&gt;&lt;p class=headings&gt;${DateLabel}&lt;/p&gt;&lt;br/&gt;${Date}&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; &lt;br/&gt;#if ( $name ) &lt;table class=headerTable&gt; &lt;tr&gt;&lt;td&gt;&lt;p class=headings&gt;${NameLabel}&lt;/p&gt;&lt;br/&gt;${NameValue}&lt;/td&gt;&lt;/tr&gt; &lt;/table&gt; #end &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;${DemographicInfo}&lt;/p&gt; &lt;hr/&gt;&lt;div class="demoDiv"&gt;#if( $demographics.get("familyName") || $demographics.get("name") || $demographics.get("surname") || $demographics.get("gender") || $demographics.get("dateOfBirth") || $demographics.get("referenceIdentityNumber") )&lt;p class="demoSection"&gt;Personal Details&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("familyName") )&lt;th&gt;$demographics.get("familyName").get("label")&lt;/th&gt;#end#if( $demographics.get("name") )&lt;th&gt;$demographics.get("name").get("label")&lt;/th&gt;#end#if( $demographics.get("surname") )&lt;th&gt;$demographics.get("surname").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("familyName") )&lt;td&gt;$demographics.get("familyName").get("value")&lt;/td&gt;#end#if( $demographics.get("name") )&lt;td&gt;$demographics.get("name").get("value")&lt;/td&gt;#end#if( $demographics.get("surname") )&lt;td&gt;$demographics.get("surname").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("gender") )&lt;th&gt;$demographics.get("gender").get("label")&lt;/th&gt;#end#if( $demographics.get("dateOfBirth") )&lt;th&gt;$demographics.get("dateOfBirth").get("label")&lt;/th&gt;#end#if( $demographics.get("referenceIdentityNumber") )&lt;th&gt;$demographics.get("referenceIdentityNumber").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("gender") )&lt;td&gt;$demographics.get("gender").get("value")&lt;/td&gt;#end#if( $demographics.get("dateOfBirth") )&lt;td&gt;$demographics.get("dateOfBirth").get("value")&lt;/td&gt;#end#if( $demographics.get("referenceIdentityNumber") )&lt;td&gt;$demographics.get("referenceIdentityNumber").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end#if( $demographics.get("placeOfBirth") || $demographics.get("districtOfBirth") || $demographics.get("divisionalSecretariatOfBirth") )&lt;p class="demoSection"&gt;Place of Birth&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("placeOfBirth") )&lt;th&gt;$demographics.get("placeOfBirth").get("label")&lt;/th&gt;#end#if( $demographics.get("districtOfBirth") )&lt;th&gt;$demographics.get("districtOfBirth").get("label")&lt;/th&gt;#end#if( $demographics.get("divisionalSecretariatOfBirth") )&lt;th&gt;$demographics.get("divisionalSecretariatOfBirth").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("placeOfBirth") )&lt;td&gt;$demographics.get("placeOfBirth").get("value")&lt;/td&gt;#end#if( $demographics.get("districtOfBirth") )&lt;td&gt;$demographics.get("districtOfBirth").get("value")&lt;/td&gt;#end#if( $demographics.get("divisionalSecretariatOfBirth") )&lt;td&gt;$demographics.get("divisionalSecretariatOfBirth").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end#if( $demographics.get("addressLine1") || $demographics.get("addressLine2") || $demographics.get("addressLine3") || $demographics.get("province") || $demographics.get("district") || $demographics.get("divisionalSecretariat") || $demographics.get("grammaNiladhari") || $demographics.get("postalCode") )&lt;p class="demoSection"&gt;Permanent Address&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("addressLine1") )&lt;th&gt;$demographics.get("addressLine1").get("label")&lt;/th&gt;#end#if( $demographics.get("addressLine2") )&lt;th&gt;$demographics.get("addressLine2").get("label")&lt;/th&gt;#end#if( $demographics.get("addressLine3") )&lt;th&gt;$demographics.get("addressLine3").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("addressLine1") )&lt;td&gt;$demographics.get("addressLine1").get("value")&lt;/td&gt;#end#if( $demographics.get("addressLine2") )&lt;td&gt;$demographics.get("addressLine2").get("value")&lt;/td&gt;#end#if( $demographics.get("addressLine3") )&lt;td&gt;$demographics.get("addressLine3").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("province") )&lt;th&gt;$demographics.get("province").get("label")&lt;/th&gt;#end#if( $demographics.get("district") )&lt;th&gt;$demographics.get("district").get("label")&lt;/th&gt;#end#if( $demographics.get("divisionalSecretariat") )&lt;th&gt;$demographics.get("divisionalSecretariat").get("label")&lt;/th&gt;#end#if( $demographics.get("grammaNiladhari") )&lt;th&gt;$demographics.get("grammaNiladhari").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("province") )&lt;td&gt;$demographics.get("province").get("value")&lt;/td&gt;#end#if( $demographics.get("district") )&lt;td&gt;$demographics.get("district").get("value")&lt;/td&gt;#end#if( $demographics.get("divisionalSecretariat") )&lt;td&gt;$demographics.get("divisionalSecretariat").get("value")&lt;/td&gt;#end#if( $demographics.get("grammaNiladhari") )&lt;td&gt;$demographics.get("grammaNiladhari").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("postalCode") )&lt;th&gt;$demographics.get("postalCode").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("postalCode") )&lt;td&gt;$demographics.get("postalCode").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end#if( $demographics.get("currentAddressLine1") || $demographics.get("currentAddressLine2") || $demographics.get("currentAddressLine3") || $demographics.get("currentProvince") || $demographics.get("currentDistrict") || $demographics.get("currentDivisionalSecretariat") || $demographics.get("currentGramaNiladhari") || $demographics.get("currentPostalCode") )&lt;p class="demoSection"&gt;Current Address&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("currentAddressLine1") )&lt;th&gt;$demographics.get("currentAddressLine1").get("label")&lt;/th&gt;#end#if( $demographics.get("currentAddressLine2") )&lt;th&gt;$demographics.get("currentAddressLine2").get("label")&lt;/th&gt;#end#if( $demographics.get("currentAddressLine3") )&lt;th&gt;$demographics.get("currentAddressLine3").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("currentAddressLine1") )&lt;td&gt;$demographics.get("currentAddressLine1").get("value")&lt;/td&gt;#end#if( $demographics.get("currentAddressLine2") )&lt;td&gt;$demographics.get("currentAddressLine2").get("value")&lt;/td&gt;#end#if( $demographics.get("currentAddressLine3") )&lt;td&gt;$demographics.get("currentAddressLine3").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("currentProvince") )&lt;th&gt;$demographics.get("currentProvince").get("label")&lt;/th&gt;#end#if( $demographics.get("currentDistrict") )&lt;th&gt;$demographics.get("currentDistrict").get("label")&lt;/th&gt;#end#if( $demographics.get("currentDivisionalSecretariat") )&lt;th&gt;$demographics.get("currentDivisionalSecretariat").get("label")&lt;/th&gt;#end#if( $demographics.get("currentGramaNiladhari") )&lt;th&gt;$demographics.get("currentGramaNiladhari").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("currentProvince") )&lt;td&gt;$demographics.get("currentProvince").get("value")&lt;/td&gt;#end#if( $demographics.get("currentDistrict") )&lt;td&gt;$demographics.get("currentDistrict").get("value")&lt;/td&gt;#end#if( $demographics.get("currentDivisionalSecretariat") )&lt;td&gt;$demographics.get("currentDivisionalSecretariat").get("value")&lt;/td&gt;#end#if( $demographics.get("currentGramaNiladhari") )&lt;td&gt;$demographics.get("currentGramaNiladhari").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("currentPostalCode") )&lt;th&gt;$demographics.get("currentPostalCode").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("currentPostalCode") )&lt;td&gt;$demographics.get("currentPostalCode").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end#if( $demographics.get("phone") || $demographics.get("email") || $demographics.get("preferredLang") )&lt;p class="demoSection"&gt;Contact Details&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("phone") )&lt;th&gt;$demographics.get("phone").get("label")&lt;/th&gt;#end#if( $demographics.get("email") )&lt;th&gt;$demographics.get("email").get("label")&lt;/th&gt;#end#if( $demographics.get("preferredLang") )&lt;th&gt;$demographics.get("preferredLang").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("phone") )&lt;td&gt;$demographics.get("phone").get("value")&lt;/td&gt;#end#if( $demographics.get("email") )&lt;td&gt;$demographics.get("email").get("value")&lt;/td&gt;#end#if( $demographics.get("preferredLang") )&lt;td&gt;$demographics.get("preferredLang").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end#if( $demographics.get("introducerName") || $demographics.get("introducerRID") || $demographics.get("introducerUIN") )&lt;p class="demoSection"&gt;Introducer Details&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("introducerName") )&lt;th&gt;$demographics.get("introducerName").get("label")&lt;/th&gt;#end#if( $demographics.get("introducerRID") )&lt;th&gt;$demographics.get("introducerRID").get("label")&lt;/th&gt;#end#if( $demographics.get("introducerUIN") )&lt;th&gt;$demographics.get("introducerUIN").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("introducerName") )&lt;td&gt;$demographics.get("introducerName").get("value")&lt;/td&gt;#end#if( $demographics.get("introducerRID") )&lt;td&gt;$demographics.get("introducerRID").get("value")&lt;/td&gt;#end#if( $demographics.get("introducerUIN") )&lt;td&gt;$demographics.get("introducerUIN").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end&lt;/div&gt; #if ( $ApplicantImageSource ) &lt;div class="photoDiv"&gt; &lt;table&gt; &lt;tr&gt; &lt;td&gt; &lt;p&gt;${Photo}&lt;/p&gt; &lt;/td&gt; &lt;/tr&gt; &lt;tr&gt; &lt;td&gt;&lt;img src="${ApplicantImageSource}" border=0 width=100 height=100/&gt;&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; &lt;/div&gt; #end &lt;div style="width: 100%; height: 50%; clear:both"&gt;&lt;/div&gt; &lt;br/&gt; &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;${DocumentsLabel}&lt;/p&gt; &lt;hr/&gt; &lt;table class="dataTable" style="width:100%;table-layout:fixed;border-collapse:collapse;"&gt; #foreach( $key in $documents.keySet() ) #if( $velocityCount % 2 == 1 )&lt;tr&gt;#end &lt;td style="vertical-align:top;width:50%;"&gt;&lt;p class=headings&gt;$documents.get($key).get("label")&lt;/p&gt;&lt;br/&gt;&lt;p&gt;$documents.get($key).get("value")&lt;/p&gt;&lt;/td&gt; #if( $velocityCount % 2 == 0 )&lt;/tr&gt;#end #end #if( $documents.size() % 2 == 1 )&lt;td style="vertical-align:top;width:50%;"&gt;&lt;/td&gt;&lt;/tr&gt;#end &lt;/table&gt; &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;${BiometricsLabel}&lt;/p&gt; &lt;hr/&gt; #foreach( $key in $biometrics.keySet() ) &lt;table&gt; &lt;tr&gt; &lt;td&gt;$biometrics.get($key).get("label")&lt;br/&gt; &lt;p class=headings&gt;${Fingers} ( $biometrics.get($key).get("FingerCount") ),${Iris} ( $biometrics.get($key).get("IrisCount") ),${Face} ( $biometrics.get($key).get("FaceCount") )&lt;br/&gt;&lt;/p&gt; &lt;br/&gt; &lt;/td&gt; &lt;/tr&gt; &lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftEye") ) &lt;td&gt; &lt;p class=headings&gt;${LeftEyeLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightEye") ) &lt;td&gt; &lt;p class=headings&gt;${RightEyeLabel}&lt;/p&gt; &lt;/td&gt; #end&lt;/tr&gt;&lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftEye") ) &lt;td&gt; #if( !$isPreview ) &lt;div class=biometrics&gt; &lt;h5 class=parentIris1&gt;$biometrics.get($key).get("LeftEye")&lt;/h5&gt; &lt;img src='$biometrics.get($key).get("CapturedLeftEye")' border=0 width=85 height=80/&gt; &lt;/div&gt; #end #if( $isPreview &amp;&amp; $biometrics.get($key).get("CapturedLeftEye") )&lt;img src='$biometrics.get($key).get("CapturedLeftEye")' border=0 width=85 height=80/&gt; #end &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightEye") ) &lt;td&gt;#if( !$isPreview ) &lt;div class=biometrics&gt; &lt;h5 class=parentIris1&gt;$biometrics.get($key).get("RightEye")&lt;/h5&gt; &lt;img src='$biometrics.get($key).get("CapturedRightEye")' border=0 width=85 height=80/&gt; &lt;/div&gt; #end &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftSlap") ) &lt;td&gt; &lt;p class=headings&gt;${LeftPalmLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightSlap") ) &lt;td&gt; &lt;p class=headings&gt;${RightPalmLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedThumbs") ) &lt;td&gt; &lt;p class=headings&gt;${ThumbsLabel}&lt;/p&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftSlap") ) &lt;td style=text-align:-webkit-center&gt; #if( !$isPreview ) &lt;table&gt; &lt;tr&gt; &lt;td&gt; &lt;div class=biometrics&gt; &lt;h5 class=leftLittle&gt;$biometrics.get($key).get("leftLittle")&lt;/h5&gt; &lt;h5 class=leftRing&gt;$biometrics.get($key).get("leftRing")&lt;/h5&gt; &lt;h5 class=leftMiddle&gt;$biometrics.get($key).get("leftMiddle")&lt;/h5&gt; &lt;h5 class=leftIndex&gt;$biometrics.get($key).get("leftIndex")&lt;/h5&gt; &lt;/div&gt; &lt;/td&gt;&lt;/tr&gt; &lt;tr&gt; &lt;td&gt;&lt;img src='$biometrics.get($key).get("CapturedLeftSlap")' border=0 width=85 height=80/&gt;&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; #end &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightSlap") ) &lt;td style=text-align:-webkit-center&gt; #if( !$isPreview ) &lt;table&gt; &lt;tr&gt; &lt;td&gt; &lt;div class=biometrics&gt; &lt;h5 class=rightIndex&gt;$biometrics.get($key).get("rightIndex")&lt;/h5&gt; &lt;h5 class=rightMiddle&gt;$biometrics.get($key).get("rightMiddle")&lt;/h5&gt; &lt;h5 class=rightRing&gt;$biometrics.get($key).get("rightRing")&lt;/h5&gt; &lt;h5 class=rightLittle&gt;$biometrics.get($key).get("rightLittle")&lt;/h5&gt; &lt;/div&gt; &lt;/td&gt;&lt;/tr&gt; &lt;tr&gt; &lt;td&gt;&lt;img src='$biometrics.get($key).get("CapturedRightSlap")' border=0 width=85 height=80/&gt;&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; #end &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedThumbs") ) &lt;td style=text-align:-webkit-center&gt; #if( !$isPreview ) &lt;table&gt; &lt;tr&gt; &lt;td&gt; &lt;div class=biometrics&gt; &lt;h5 class=leftThumb&gt;$biometrics.get($key).get("leftThumb")&lt;/h5&gt; &lt;h5 class=rightThumb&gt;$biometrics.get($key).get("rightThumb")&lt;/h5&gt; &lt;/div&gt; &lt;/td&gt;&lt;/tr&gt; &lt;tr&gt; &lt;td&gt;&lt;img src='$biometrics.get($key).get("CapturedThumbs")' border=0 width=85 height=80/&gt;&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; #end &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;br/&gt; &lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("FaceImageSource") ) &lt;td&gt; &lt;p class=headings&gt;${FaceLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("subType") == "applicant" &amp;&amp; $ExceptionImageSource ) &lt;td&gt; &lt;p class=headings&gt;${ExceptionPhotoLabel}&lt;/p&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;tr&gt; #if( $biometrics.get($key).get("FaceImageSource") ) &lt;td&gt;&lt;img src='$biometrics.get($key).get("FaceImageSource")' border=0 width=85 height=80/&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("subType") == "applicant" &amp;&amp; $ExceptionImageSource ) &lt;td&gt; &lt;img src="${ExceptionImageSource}" border=0 width=85 height=80/&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;/table&gt; #end &lt;br/&gt;&lt;div class="ackPostBioBlock" style="display:block;clear:both;width:100%;"&gt;#if( $SignatureSectionVisible )&lt;div data-mosip-ack-signature="1" style="display:block;width:100%;"&gt;&lt;br/&gt;&lt;hr/&gt;&lt;p class=head style="display:block;"&gt;${SignatureLabel}&lt;/p&gt;&lt;hr/&gt;&lt;/div&gt;#end&lt;table class="dataTable" style="width:100%;table-layout:fixed;border-collapse:collapse;display:table;clear:both;"&gt;#if( $SignatureSectionVisible )&lt;tr&gt;&lt;td style="vertical-align:top;width:50%;"&gt;&lt;p class=headings&gt;#if( $SignatureCaptured )${SignatureCapturedLabel}#else${SignatureNotCapturedLabel}#end&lt;/p&gt;&lt;br/&gt;&lt;p&gt;#if( $SignatureCaptured )&lt;span style="color:#2E7D32;font-size:18px;"&gt;&amp;#10004;&lt;/span&gt; &lt;span style="color:#2E7D32;"&gt;${SignatureCapturedLabel}&lt;/span&gt;#else&lt;span style="color:#808080;font-size:18px;"&gt;&amp;#10007;&lt;/span&gt; &lt;span style="color:#808080;"&gt;${SignatureNotCapturedLabel}&lt;/span&gt;#end&lt;/p&gt;&lt;/td&gt;#if( $SignatureCaptured )&lt;td style="vertical-align:top;width:50%;"&gt;&lt;p class=headings&gt;${SignatureLabel}&lt;/p&gt;&lt;br/&gt;&lt;p&gt;&lt;img data-mosip-applicant-signature="1" src="${SignatureImageSource}" border="0" width="200" height="85" style="max-width:200px;max-height:85px;object-fit:contain;border:1px solid #b0b0b0;background:#fff;display:block;"/&gt;&lt;/p&gt;&lt;/td&gt;#else&lt;td style="vertical-align:top;width:50%;"&gt;&lt;/td&gt;#end&lt;/tr&gt;#end&lt;tr&gt;&lt;td&gt;&lt;p class=headings&gt;${RONameLabel}&lt;/p&gt;&lt;br/&gt;&lt;p&gt;${ROName}&lt;/p&gt;&lt;/td&gt;&lt;td&gt;&lt;p class=headings&gt;${RegCenterLabel}&lt;/p&gt;&lt;br/&gt;&lt;p&gt;${RegCenter}&lt;/p&gt;&lt;/td&gt;&lt;/tr&gt;&lt;/table&gt;&lt;hr/&gt;&lt;br/&gt;&lt;/div&gt;&lt;div&gt;&lt;p&gt;${ImportantGuidelines}&lt;/p&gt; &lt;ul&gt; #foreach( $line in $Guidelines ) &lt;li&gt;&lt;span&gt;${line}&lt;/span&gt;&lt;/li&gt; #end &lt;/ul&gt;&lt;/div&gt;&lt;/div&gt;&lt;/div&gt;&lt;/body&gt;&lt;/html&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;!DOCTYPE html&gt;&lt;html $rtl&gt;&lt;head&gt;&lt;meta charset="UTF-8"/&gt;&lt;style&gt;body,.head,.headings,th,td,p,b,strong{font-family:system-ui,"Segoe UI","Nirmala UI","Iskoola Pota","Latha",sans-serif;}table, .head{font-size:13px;}.demoDiv{width: 85%;float: left;}.photoDiv{width: 15%;float:right;}.form{display:block;width:100%;}.section{padding:24px;width:800px;max-width:800px;margin-left:auto;margin-right:auto;box-sizing:border-box;}.headings{color:#808080;font-size:11px;}p{display:inline;}.dataTable{word-wrap:break-word;table-layout:fixed;width:100%;}.headerTable{width:90%;}.uinHeaderTable{width:100%;}h5{display:inline;position:absolute;}.iris{top:-15px;left:152px;}.irisWithoutException{top:-15px;left:114px;}.tableWithoutException{width:50%;text-align:center;table-layout:fixed;margin:0 auto;}.biometricsTable{width:100%;text-align:center;table-layout:fixed;}.biometrics{position:relative;}.leftLittle{top:15px;left:11px;display:inline;position:absolute;}.leftRing{top:3px;left:23px;}.leftMiddle{top:-7px;left:37px;}.leftIndex{top:3px;left:54px;}.rightIndex{top:3px;left:26px;}.rightMiddle{top:-7px;left:39px;}.rightRing{top:3px;left:55px;}.rightLittle{top:15px;left:68px;}.leftThumb{top:-4px;left:24px;}.rightThumb{top:-4px;left:54px;}.parentStyle{top:-15px;left:152px;}.parentIris1{top:-15px;left:212px;}.parentIris2{top:-15px;left:214px;}li span{color:black;font-size:12px;} li{color:lightgrey}button{float:right;font-size:12px;border:none;background-color:transparent;outline:none;}button:active{background-color:black;color:white;} .bottom{vertical-align:bottom;}.consent-block{font-size:13px;border-radius: 8px;margin-top: 10px;margin-bottom: 10px;border: 2px solid #E88E3F;padding-top: -50px;padding:10px;}.consent-text{margin-left: 7px;margin-bottom: 4px;}input[type="radio"] {display: none;} input[type="radio"] + label:before { content: ""; display: inline-block; width: 15px; height: 15px; padding: 3px; margin-right: 5px; background-clip: content-box; border: 1px solid grey; background-color: #fff; border-radius: 50%;}input[type="radio"]:checked + label:before { background-color: #FF4081; border-color:#FF4081;}*,*:before,*:after { box-sizing: border-box;}.consent-block label { display: inline-flex; align-items: center;}.demoDiv&gt;table{width:100%}.demoDiv&gt;table&gt;tbody&gt;tr&gt;th{color:#808080;font-size:10px; width:25%; text-align: left;padding: 2px;font-weight:normal;}.demoDiv&gt;table&gt;tbody&gt;tr&gt;td{width:25%; text-align: left;padding: 2px}.ackPostBioBlock{display:block;clear:both;width:100%!important;max-width:100%;}.ackPostBioBlock hr{width:100%;}.ackPostBioBlock .dataTable{width:100%!important;max-width:100%;table-layout:fixed;border-collapse:collapse;display:table!important;}.ackPostBioBlock .headings,.ackPostBioBlock p.head,.ackPostBioBlock td&gt;p{display:block;}.demoSection{display:block;color:#808080;font-size:11px;font-weight:bold;margin:12px 0 4px 0;}.demoDiv&gt;p.demoSection:first-child{margin-top:0;}.demoDiv&gt;table&gt;tbody&gt;tr&gt;th{font-weight:normal;}&lt;/style&gt;&lt;script&gt;function changeColour(element) { var div = document.getElementById("radioId"); if(element.value == "yes"){div.style = "border: 2px solid #68A933";} if(element.value == "no"){div.style = "border: 2px solid #FF0000";}} document.onreadystatechange = function () {if(document.readyState === "complete"){var body = document.getElementsByTagName("body")[0]; body.addEventListener("dragstart", function(event) {event.preventDefault();}); body.addEventListener("selectstart", function(event) {event.preventDefault();});}}&lt;/script&gt;&lt;/head&gt; &lt;body&gt; &lt;div class=section&gt; &lt;div class=form&gt; &lt;table class=headerTable&gt; &lt;tr&gt; #if ( !$isPreview &amp;&amp; $QRCodeSource ) &lt;td class=bottom&gt; &lt;img src="${QRCodeSource}" width=85 height=85/&gt; &lt;/td&gt; #end &lt;td class=bottom&gt;&lt;p class=headings&gt;${ApplicationIDLabel}&lt;/p&gt;&lt;br/&gt;${ApplicationID}&lt;/td&gt; #if ( $UIN ) &lt;td class=bottom&gt;&lt;p class=headings&gt;${UINLabel}&lt;/p&gt;&lt;br/&gt;${UIN}&lt;/td&gt; #end &lt;td class=bottom&gt;&lt;p class=headings&gt;${DateLabel}&lt;/p&gt;&lt;br/&gt;${Date}&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; &lt;br/&gt;#if ( $name ) &lt;table class=headerTable&gt; &lt;tr&gt;&lt;td&gt;&lt;p class=headings&gt;${NameLabel}&lt;/p&gt;&lt;br/&gt;${NameValue}&lt;/td&gt;&lt;/tr&gt; &lt;/table&gt; #end &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;${DemographicInfo}&lt;/p&gt; &lt;hr/&gt;&lt;div class="demoDiv"&gt;#if( $demographics.get("familyName") || $demographics.get("name") || $demographics.get("surname") || $demographics.get("gender") || $demographics.get("dateOfBirth") || $demographics.get("referenceIdentityNumber") )&lt;p class="demoSection"&gt;පෞද්ගලික විස්තර&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("familyName") )&lt;th&gt;$demographics.get("familyName").get("label")&lt;/th&gt;#end#if( $demographics.get("name") )&lt;th&gt;$demographics.get("name").get("label")&lt;/th&gt;#end#if( $demographics.get("surname") )&lt;th&gt;$demographics.get("surname").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("familyName") )&lt;td&gt;$demographics.get("familyName").get("value")&lt;/td&gt;#end#if( $demographics.get("name") )&lt;td&gt;$demographics.get("name").get("value")&lt;/td&gt;#end#if( $demographics.get("surname") )&lt;td&gt;$demographics.get("surname").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("gender") )&lt;th&gt;$demographics.get("gender").get("label")&lt;/th&gt;#end#if( $demographics.get("dateOfBirth") )&lt;th&gt;$demographics.get("dateOfBirth").get("label")&lt;/th&gt;#end#if( $demographics.get("referenceIdentityNumber") )&lt;th&gt;$demographics.get("referenceIdentityNumber").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("gender") )&lt;td&gt;$demographics.get("gender").get("value")&lt;/td&gt;#end#if( $demographics.get("dateOfBirth") )&lt;td&gt;$demographics.get("dateOfBirth").get("value")&lt;/td&gt;#end#if( $demographics.get("referenceIdentityNumber") )&lt;td&gt;$demographics.get("referenceIdentityNumber").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end#if( $demographics.get("placeOfBirth") || $demographics.get("districtOfBirth") || $demographics.get("divisionalSecretariatOfBirth") )&lt;p class="demoSection"&gt;උපන් ස්ථානය&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("placeOfBirth") )&lt;th&gt;$demographics.get("placeOfBirth").get("label")&lt;/th&gt;#end#if( $demographics.get("districtOfBirth") )&lt;th&gt;$demographics.get("districtOfBirth").get("label")&lt;/th&gt;#end#if( $demographics.get("divisionalSecretariatOfBirth") )&lt;th&gt;$demographics.get("divisionalSecretariatOfBirth").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("placeOfBirth") )&lt;td&gt;$demographics.get("placeOfBirth").get("value")&lt;/td&gt;#end#if( $demographics.get("districtOfBirth") )&lt;td&gt;$demographics.get("districtOfBirth").get("value")&lt;/td&gt;#end#if( $demographics.get("divisionalSecretariatOfBirth") )&lt;td&gt;$demographics.get("divisionalSecretariatOfBirth").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end#if( $demographics.get("addressLine1") || $demographics.get("addressLine2") || $demographics.get("addressLine3") || $demographics.get("province") || $demographics.get("district") || $demographics.get("divisionalSecretariat") || $demographics.get("grammaNiladhari") || $demographics.get("postalCode") )&lt;p class="demoSection"&gt;ස්ථිර ලිපිනය&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("addressLine1") )&lt;th&gt;$demographics.get("addressLine1").get("label")&lt;/th&gt;#end#if( $demographics.get("addressLine2") )&lt;th&gt;$demographics.get("addressLine2").get("label")&lt;/th&gt;#end#if( $demographics.get("addressLine3") )&lt;th&gt;$demographics.get("addressLine3").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("addressLine1") )&lt;td&gt;$demographics.get("addressLine1").get("value")&lt;/td&gt;#end#if( $demographics.get("addressLine2") )&lt;td&gt;$demographics.get("addressLine2").get("value")&lt;/td&gt;#end#if( $demographics.get("addressLine3") )&lt;td&gt;$demographics.get("addressLine3").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("province") )&lt;th&gt;$demographics.get("province").get("label")&lt;/th&gt;#end#if( $demographics.get("district") )&lt;th&gt;$demographics.get("district").get("label")&lt;/th&gt;#end#if( $demographics.get("divisionalSecretariat") )&lt;th&gt;$demographics.get("divisionalSecretariat").get("label")&lt;/th&gt;#end#if( $demographics.get("grammaNiladhari") )&lt;th&gt;$demographics.get("grammaNiladhari").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("province") )&lt;td&gt;$demographics.get("province").get("value")&lt;/td&gt;#end#if( $demographics.get("district") )&lt;td&gt;$demographics.get("district").get("value")&lt;/td&gt;#end#if( $demographics.get("divisionalSecretariat") )&lt;td&gt;$demographics.get("divisionalSecretariat").get("value")&lt;/td&gt;#end#if( $demographics.get("grammaNiladhari") )&lt;td&gt;$demographics.get("grammaNiladhari").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("postalCode") )&lt;th&gt;$demographics.get("postalCode").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("postalCode") )&lt;td&gt;$demographics.get("postalCode").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end#if( $demographics.get("currentAddressLine1") || $demographics.get("currentAddressLine2") || $demographics.get("currentAddressLine3") || $demographics.get("currentProvince") || $demographics.get("currentDistrict") || $demographics.get("currentDivisionalSecretariat") || $demographics.get("currentGramaNiladhari") || $demographics.get("currentPostalCode") )&lt;p class="demoSection"&gt;වත්මන් ලිපිනය&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("currentAddressLine1") )&lt;th&gt;$demographics.get("currentAddressLine1").get("label")&lt;/th&gt;#end#if( $demographics.get("currentAddressLine2") )&lt;th&gt;$demographics.get("currentAddressLine2").get("label")&lt;/th&gt;#end#if( $demographics.get("currentAddressLine3") )&lt;th&gt;$demographics.get("currentAddressLine3").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("currentAddressLine1") )&lt;td&gt;$demographics.get("currentAddressLine1").get("value")&lt;/td&gt;#end#if( $demographics.get("currentAddressLine2") )&lt;td&gt;$demographics.get("currentAddressLine2").get("value")&lt;/td&gt;#end#if( $demographics.get("currentAddressLine3") )&lt;td&gt;$demographics.get("currentAddressLine3").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("currentProvince") )&lt;th&gt;$demographics.get("currentProvince").get("label")&lt;/th&gt;#end#if( $demographics.get("currentDistrict") )&lt;th&gt;$demographics.get("currentDistrict").get("label")&lt;/th&gt;#end#if( $demographics.get("currentDivisionalSecretariat") )&lt;th&gt;$demographics.get("currentDivisionalSecretariat").get("label")&lt;/th&gt;#end#if( $demographics.get("currentGramaNiladhari") )&lt;th&gt;$demographics.get("currentGramaNiladhari").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("currentProvince") )&lt;td&gt;$demographics.get("currentProvince").get("value")&lt;/td&gt;#end#if( $demographics.get("currentDistrict") )&lt;td&gt;$demographics.get("currentDistrict").get("value")&lt;/td&gt;#end#if( $demographics.get("currentDivisionalSecretariat") )&lt;td&gt;$demographics.get("currentDivisionalSecretariat").get("value")&lt;/td&gt;#end#if( $demographics.get("currentGramaNiladhari") )&lt;td&gt;$demographics.get("currentGramaNiladhari").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("currentPostalCode") )&lt;th&gt;$demographics.get("currentPostalCode").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("currentPostalCode") )&lt;td&gt;$demographics.get("currentPostalCode").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end#if( $demographics.get("phone") || $demographics.get("email") || $demographics.get("preferredLang") )&lt;p class="demoSection"&gt;සම්බන්ධතා විස්තර&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("phone") )&lt;th&gt;$demographics.get("phone").get("label")&lt;/th&gt;#end#if( $demographics.get("email") )&lt;th&gt;$demographics.get("email").get("label")&lt;/th&gt;#end#if( $demographics.get("preferredLang") )&lt;th&gt;$demographics.get("preferredLang").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("phone") )&lt;td&gt;$demographics.get("phone").get("value")&lt;/td&gt;#end#if( $demographics.get("email") )&lt;td&gt;$demographics.get("email").get("value")&lt;/td&gt;#end#if( $demographics.get("preferredLang") )&lt;td&gt;$demographics.get("preferredLang").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end#if( $demographics.get("introducerName") || $demographics.get("introducerRID") || $demographics.get("introducerUIN") )&lt;p class="demoSection"&gt;හඳුන්වා දෙන්නාගේ විස්තර&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("introducerName") )&lt;th&gt;$demographics.get("introducerName").get("label")&lt;/th&gt;#end#if( $demographics.get("introducerRID") )&lt;th&gt;$demographics.get("introducerRID").get("label")&lt;/th&gt;#end#if( $demographics.get("introducerUIN") )&lt;th&gt;$demographics.get("introducerUIN").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("introducerName") )&lt;td&gt;$demographics.get("introducerName").get("value")&lt;/td&gt;#end#if( $demographics.get("introducerRID") )&lt;td&gt;$demographics.get("introducerRID").get("value")&lt;/td&gt;#end#if( $demographics.get("introducerUIN") )&lt;td&gt;$demographics.get("introducerUIN").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end&lt;/div&gt; #if ( $ApplicantImageSource ) &lt;div class="photoDiv"&gt; &lt;table&gt; &lt;tr&gt; &lt;td&gt; &lt;p&gt;${Photo}&lt;/p&gt; &lt;/td&gt; &lt;/tr&gt; &lt;tr&gt; &lt;td&gt;&lt;img src="${ApplicantImageSource}" border=0 width=100 height=100/&gt;&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; &lt;/div&gt; #end &lt;div style="width: 100%; height: 50%; clear:both"&gt;&lt;/div&gt; &lt;br/&gt; &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;${DocumentsLabel}&lt;/p&gt; &lt;hr/&gt; &lt;table class="dataTable" style="width:100%;table-layout:fixed;border-collapse:collapse;"&gt; #foreach( $key in $documents.keySet() ) #if( $velocityCount % 2 == 1 )&lt;tr&gt;#end &lt;td style="vertical-align:top;width:50%;"&gt;&lt;p class=headings&gt;$documents.get($key).get("label")&lt;/p&gt;&lt;br/&gt;&lt;p&gt;$documents.get($key).get("value")&lt;/p&gt;&lt;/td&gt; #if( $velocityCount % 2 == 0 )&lt;/tr&gt;#end #end #if( $documents.size() % 2 == 1 )&lt;td style="vertical-align:top;width:50%;"&gt;&lt;/td&gt;&lt;/tr&gt;#end &lt;/table&gt; &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;${BiometricsLabel}&lt;/p&gt; &lt;hr/&gt; #foreach( $key in $biometrics.keySet() ) &lt;table&gt; &lt;tr&gt; &lt;td&gt;$biometrics.get($key).get("label")&lt;br/&gt; &lt;p class=headings&gt;${Fingers} ( $biometrics.get($key).get("FingerCount") ),${Iris} ( $biometrics.get($key).get("IrisCount") ),${Face} ( $biometrics.get($key).get("FaceCount") )&lt;br/&gt;&lt;/p&gt; &lt;br/&gt; &lt;/td&gt; &lt;/tr&gt; &lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftEye") ) &lt;td&gt; &lt;p class=headings&gt;${LeftEyeLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightEye") ) &lt;td&gt; &lt;p class=headings&gt;${RightEyeLabel}&lt;/p&gt; &lt;/td&gt; #end&lt;/tr&gt;&lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftEye") ) &lt;td&gt; #if( !$isPreview ) &lt;div class=biometrics&gt; &lt;h5 class=parentIris1&gt;$biometrics.get($key).get("LeftEye")&lt;/h5&gt; &lt;img src='$biometrics.get($key).get("CapturedLeftEye")' border=0 width=85 height=80/&gt; &lt;/div&gt; #end #if( $isPreview &amp;&amp; $biometrics.get($key).get("CapturedLeftEye") )&lt;img src='$biometrics.get($key).get("CapturedLeftEye")' border=0 width=85 height=80/&gt; #end &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightEye") ) &lt;td&gt;#if( !$isPreview ) &lt;div class=biometrics&gt; &lt;h5 class=parentIris1&gt;$biometrics.get($key).get("RightEye")&lt;/h5&gt; &lt;img src='$biometrics.get($key).get("CapturedRightEye")' border=0 width=85 height=80/&gt; &lt;/div&gt; #end &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftSlap") ) &lt;td&gt; &lt;p class=headings&gt;${LeftPalmLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightSlap") ) &lt;td&gt; &lt;p class=headings&gt;${RightPalmLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedThumbs") ) &lt;td&gt; &lt;p class=headings&gt;${ThumbsLabel}&lt;/p&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftSlap") ) &lt;td style=text-align:-webkit-center&gt; #if( !$isPreview ) &lt;table&gt; &lt;tr&gt; &lt;td&gt; &lt;div class=biometrics&gt; &lt;h5 class=leftLittle&gt;$biometrics.get($key).get("leftLittle")&lt;/h5&gt; &lt;h5 class=leftRing&gt;$biometrics.get($key).get("leftRing")&lt;/h5&gt; &lt;h5 class=leftMiddle&gt;$biometrics.get($key).get("leftMiddle")&lt;/h5&gt; &lt;h5 class=leftIndex&gt;$biometrics.get($key).get("leftIndex")&lt;/h5&gt; &lt;/div&gt; &lt;/td&gt;&lt;/tr&gt; &lt;tr&gt; &lt;td&gt;&lt;img src='$biometrics.get($key).get("CapturedLeftSlap")' border=0 width=85 height=80/&gt;&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; #end &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightSlap") ) &lt;td style=text-align:-webkit-center&gt; #if( !$isPreview ) &lt;table&gt; &lt;tr&gt; &lt;td&gt; &lt;div class=biometrics&gt; &lt;h5 class=rightIndex&gt;$biometrics.get($key).get("rightIndex")&lt;/h5&gt; &lt;h5 class=rightMiddle&gt;$biometrics.get($key).get("rightMiddle")&lt;/h5&gt; &lt;h5 class=rightRing&gt;$biometrics.get($key).get("rightRing")&lt;/h5&gt; &lt;h5 class=rightLittle&gt;$biometrics.get($key).get("rightLittle")&lt;/h5&gt; &lt;/div&gt; &lt;/td&gt;&lt;/tr&gt; &lt;tr&gt; &lt;td&gt;&lt;img src='$biometrics.get($key).get("CapturedRightSlap")' border=0 width=85 height=80/&gt;&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; #end &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedThumbs") ) &lt;td style=text-align:-webkit-center&gt; #if( !$isPreview ) &lt;table&gt; &lt;tr&gt; &lt;td&gt; &lt;div class=biometrics&gt; &lt;h5 class=leftThumb&gt;$biometrics.get($key).get("leftThumb")&lt;/h5&gt; &lt;h5 class=rightThumb&gt;$biometrics.get($key).get("rightThumb")&lt;/h5&gt; &lt;/div&gt; &lt;/td&gt;&lt;/tr&gt; &lt;tr&gt; &lt;td&gt;&lt;img src='$biometrics.get($key).get("CapturedThumbs")' border=0 width=85 height=80/&gt;&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; #end &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;br/&gt; &lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("FaceImageSource") ) &lt;td&gt; &lt;p class=headings&gt;${FaceLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("subType") == "applicant" &amp;&amp; $ExceptionImageSource ) &lt;td&gt; &lt;p class=headings&gt;${ExceptionPhotoLabel}&lt;/p&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;tr&gt; #if( $biometrics.get($key).get("FaceImageSource") ) &lt;td&gt;&lt;img src='$biometrics.get($key).get("FaceImageSource")' border=0 width=85 height=80/&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("subType") == "applicant" &amp;&amp; $ExceptionImageSource ) &lt;td&gt; &lt;img src="${ExceptionImageSource}" border=0 width=85 height=80/&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;/table&gt; #end &lt;br/&gt;&lt;div class="ackPostBioBlock" style="display:block;clear:both;width:100%;"&gt;#if( $SignatureSectionVisible )&lt;div data-mosip-ack-signature="1" style="display:block;width:100%;"&gt;&lt;br/&gt;&lt;hr/&gt;&lt;p class=head style="display:block;"&gt;${SignatureLabel}&lt;/p&gt;&lt;hr/&gt;&lt;/div&gt;#end&lt;table class="dataTable" style="width:100%;table-layout:fixed;border-collapse:collapse;display:table;clear:both;"&gt;#if( $SignatureSectionVisible )&lt;tr&gt;&lt;td style="vertical-align:top;width:50%;"&gt;&lt;p class=headings&gt;#if( $SignatureCaptured )${SignatureCapturedLabel}#else${SignatureNotCapturedLabel}#end&lt;/p&gt;&lt;br/&gt;&lt;p&gt;#if( $SignatureCaptured )&lt;span style="color:#2E7D32;font-size:18px;"&gt;&amp;#10004;&lt;/span&gt; &lt;span style="color:#2E7D32;"&gt;${SignatureCapturedLabel}&lt;/span&gt;#else&lt;span style="color:#808080;font-size:18px;"&gt;&amp;#10007;&lt;/span&gt; &lt;span style="color:#808080;"&gt;${SignatureNotCapturedLabel}&lt;/span&gt;#end&lt;/p&gt;&lt;/td&gt;#if( $SignatureCaptured )&lt;td style="vertical-align:top;width:50%;"&gt;&lt;p class=headings&gt;${SignatureLabel}&lt;/p&gt;&lt;br/&gt;&lt;p&gt;&lt;img data-mosip-applicant-signature="1" src="${SignatureImageSource}" border="0" width="200" height="85" style="max-width:200px;max-height:85px;object-fit:contain;border:1px solid #b0b0b0;background:#fff;display:block;"/&gt;&lt;/p&gt;&lt;/td&gt;#else&lt;td style="vertical-align:top;width:50%;"&gt;&lt;/td&gt;#end&lt;/tr&gt;#end&lt;tr&gt;&lt;td&gt;&lt;p class=headings&gt;${RONameLabel}&lt;/p&gt;&lt;br/&gt;&lt;p&gt;${ROName}&lt;/p&gt;&lt;/td&gt;&lt;td&gt;&lt;p class=headings&gt;${RegCenterLabel}&lt;/p&gt;&lt;br/&gt;&lt;p&gt;${RegCenter}&lt;/p&gt;&lt;/td&gt;&lt;/tr&gt;&lt;/table&gt;&lt;hr/&gt;&lt;br/&gt;&lt;/div&gt;&lt;div&gt;&lt;p&gt;${ImportantGuidelines}&lt;/p&gt; &lt;ul&gt; #foreach( $line in $Guidelines ) &lt;li&gt;&lt;span&gt;${line}&lt;/span&gt;&lt;/li&gt; #end &lt;/ul&gt;&lt;/div&gt;&lt;/div&gt;&lt;/div&gt;&lt;/body&gt;&lt;/html&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;!DOCTYPE html&gt;&lt;html $rtl&gt;&lt;head&gt;&lt;meta charset="UTF-8"/&gt;&lt;style&gt;body,.head,.headings,th,td,p,b,strong{font-family:system-ui,"Segoe UI","Nirmala UI","Iskoola Pota","Latha",sans-serif;}table, .head{font-size:13px;}.demoDiv{width: 85%;float: left;}.photoDiv{width: 15%;float:right;}.form{display:block;width:100%;}.section{padding:24px;width:800px;max-width:800px;margin-left:auto;margin-right:auto;box-sizing:border-box;}.headings{color:#808080;font-size:11px;}p{display:inline;}.dataTable{word-wrap:break-word;table-layout:fixed;width:100%;}.headerTable{width:90%;}.uinHeaderTable{width:100%;}h5{display:inline;position:absolute;}.iris{top:-15px;left:152px;}.irisWithoutException{top:-15px;left:114px;}.tableWithoutException{width:50%;text-align:center;table-layout:fixed;margin:0 auto;}.biometricsTable{width:100%;text-align:center;table-layout:fixed;}.biometrics{position:relative;}.leftLittle{top:15px;left:11px;display:inline;position:absolute;}.leftRing{top:3px;left:23px;}.leftMiddle{top:-7px;left:37px;}.leftIndex{top:3px;left:54px;}.rightIndex{top:3px;left:26px;}.rightMiddle{top:-7px;left:39px;}.rightRing{top:3px;left:55px;}.rightLittle{top:15px;left:68px;}.leftThumb{top:-4px;left:24px;}.rightThumb{top:-4px;left:54px;}.parentStyle{top:-15px;left:152px;}.parentIris1{top:-15px;left:212px;}.parentIris2{top:-15px;left:214px;}li span{color:black;font-size:12px;} li{color:lightgrey}button{float:right;font-size:12px;border:none;background-color:transparent;outline:none;}button:active{background-color:black;color:white;} .bottom{vertical-align:bottom;}.consent-block{font-size:13px;border-radius: 8px;margin-top: 10px;margin-bottom: 10px;border: 2px solid #E88E3F;padding-top: -50px;padding:10px;}.consent-text{margin-left: 7px;margin-bottom: 4px;}input[type="radio"] {display: none;} input[type="radio"] + label:before { content: ""; display: inline-block; width: 15px; height: 15px; padding: 3px; margin-right: 5px; background-clip: content-box; border: 1px solid grey; background-color: #fff; border-radius: 50%;}input[type="radio"]:checked + label:before { background-color: #FF4081; border-color:#FF4081;}*,*:before,*:after { box-sizing: border-box;}.consent-block label { display: inline-flex; align-items: center;}.demoDiv&gt;table{width:100%}.demoDiv&gt;table&gt;tbody&gt;tr&gt;th{color:#808080;font-size:10px; width:25%; text-align: left;padding: 2px;font-weight:normal;}.demoDiv&gt;table&gt;tbody&gt;tr&gt;td{width:25%; text-align: left;padding: 2px}.ackPostBioBlock{display:block;clear:both;width:100%!important;max-width:100%;}.ackPostBioBlock hr{width:100%;}.ackPostBioBlock .dataTable{width:100%!important;max-width:100%;table-layout:fixed;border-collapse:collapse;display:table!important;}.ackPostBioBlock .headings,.ackPostBioBlock p.head,.ackPostBioBlock td&gt;p{display:block;}.demoSection{display:block;color:#808080;font-size:11px;font-weight:bold;margin:12px 0 4px 0;}.demoDiv&gt;p.demoSection:first-child{margin-top:0;}.demoDiv&gt;table&gt;tbody&gt;tr&gt;th{font-weight:normal;}&lt;/style&gt;&lt;script&gt;function changeColour(element) { var div = document.getElementById("radioId"); if(element.value == "yes"){div.style = "border: 2px solid #68A933";} if(element.value == "no"){div.style = "border: 2px solid #FF0000";}} document.onreadystatechange = function () {if(document.readyState === "complete"){var body = document.getElementsByTagName("body")[0]; body.addEventListener("dragstart", function(event) {event.preventDefault();}); body.addEventListener("selectstart", function(event) {event.preventDefault();});}}&lt;/script&gt;&lt;/head&gt; &lt;body&gt; &lt;div class=section&gt; &lt;div class=form&gt; &lt;table class=headerTable&gt; &lt;tr&gt; #if ( !$isPreview &amp;&amp; $QRCodeSource ) &lt;td class=bottom&gt; &lt;img src="${QRCodeSource}" width=85 height=85/&gt; &lt;/td&gt; #end &lt;td class=bottom&gt;&lt;p class=headings&gt;${ApplicationIDLabel}&lt;/p&gt;&lt;br/&gt;${ApplicationID}&lt;/td&gt; #if ( $UIN ) &lt;td class=bottom&gt;&lt;p class=headings&gt;${UINLabel}&lt;/p&gt;&lt;br/&gt;${UIN}&lt;/td&gt; #end &lt;td class=bottom&gt;&lt;p class=headings&gt;${DateLabel}&lt;/p&gt;&lt;br/&gt;${Date}&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; &lt;br/&gt;#if ( $name ) &lt;table class=headerTable&gt; &lt;tr&gt;&lt;td&gt;&lt;p class=headings&gt;${NameLabel}&lt;/p&gt;&lt;br/&gt;${NameValue}&lt;/td&gt;&lt;/tr&gt; &lt;/table&gt; #end &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;${DemographicInfo}&lt;/p&gt; &lt;hr/&gt;&lt;div class="demoDiv"&gt;#if( $demographics.get("familyName") || $demographics.get("name") || $demographics.get("surname") || $demographics.get("gender") || $demographics.get("dateOfBirth") || $demographics.get("referenceIdentityNumber") )&lt;p class="demoSection"&gt;தனிப்பட்ட விவரங்கள்&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("familyName") )&lt;th&gt;$demographics.get("familyName").get("label")&lt;/th&gt;#end#if( $demographics.get("name") )&lt;th&gt;$demographics.get("name").get("label")&lt;/th&gt;#end#if( $demographics.get("surname") )&lt;th&gt;$demographics.get("surname").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("familyName") )&lt;td&gt;$demographics.get("familyName").get("value")&lt;/td&gt;#end#if( $demographics.get("name") )&lt;td&gt;$demographics.get("name").get("value")&lt;/td&gt;#end#if( $demographics.get("surname") )&lt;td&gt;$demographics.get("surname").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("gender") )&lt;th&gt;$demographics.get("gender").get("label")&lt;/th&gt;#end#if( $demographics.get("dateOfBirth") )&lt;th&gt;$demographics.get("dateOfBirth").get("label")&lt;/th&gt;#end#if( $demographics.get("referenceIdentityNumber") )&lt;th&gt;$demographics.get("referenceIdentityNumber").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("gender") )&lt;td&gt;$demographics.get("gender").get("value")&lt;/td&gt;#end#if( $demographics.get("dateOfBirth") )&lt;td&gt;$demographics.get("dateOfBirth").get("value")&lt;/td&gt;#end#if( $demographics.get("referenceIdentityNumber") )&lt;td&gt;$demographics.get("referenceIdentityNumber").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end#if( $demographics.get("placeOfBirth") || $demographics.get("districtOfBirth") || $demographics.get("divisionalSecretariatOfBirth") )&lt;p class="demoSection"&gt;பிறந்த இடம்&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("placeOfBirth") )&lt;th&gt;$demographics.get("placeOfBirth").get("label")&lt;/th&gt;#end#if( $demographics.get("districtOfBirth") )&lt;th&gt;$demographics.get("districtOfBirth").get("label")&lt;/th&gt;#end#if( $demographics.get("divisionalSecretariatOfBirth") )&lt;th&gt;$demographics.get("divisionalSecretariatOfBirth").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("placeOfBirth") )&lt;td&gt;$demographics.get("placeOfBirth").get("value")&lt;/td&gt;#end#if( $demographics.get("districtOfBirth") )&lt;td&gt;$demographics.get("districtOfBirth").get("value")&lt;/td&gt;#end#if( $demographics.get("divisionalSecretariatOfBirth") )&lt;td&gt;$demographics.get("divisionalSecretariatOfBirth").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end#if( $demographics.get("addressLine1") || $demographics.get("addressLine2") || $demographics.get("addressLine3") || $demographics.get("province") || $demographics.get("district") || $demographics.get("divisionalSecretariat") || $demographics.get("grammaNiladhari") || $demographics.get("postalCode") )&lt;p class="demoSection"&gt;நிரந்தர முகவரி&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("addressLine1") )&lt;th&gt;$demographics.get("addressLine1").get("label")&lt;/th&gt;#end#if( $demographics.get("addressLine2") )&lt;th&gt;$demographics.get("addressLine2").get("label")&lt;/th&gt;#end#if( $demographics.get("addressLine3") )&lt;th&gt;$demographics.get("addressLine3").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("addressLine1") )&lt;td&gt;$demographics.get("addressLine1").get("value")&lt;/td&gt;#end#if( $demographics.get("addressLine2") )&lt;td&gt;$demographics.get("addressLine2").get("value")&lt;/td&gt;#end#if( $demographics.get("addressLine3") )&lt;td&gt;$demographics.get("addressLine3").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("province") )&lt;th&gt;$demographics.get("province").get("label")&lt;/th&gt;#end#if( $demographics.get("district") )&lt;th&gt;$demographics.get("district").get("label")&lt;/th&gt;#end#if( $demographics.get("divisionalSecretariat") )&lt;th&gt;$demographics.get("divisionalSecretariat").get("label")&lt;/th&gt;#end#if( $demographics.get("grammaNiladhari") )&lt;th&gt;$demographics.get("grammaNiladhari").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("province") )&lt;td&gt;$demographics.get("province").get("value")&lt;/td&gt;#end#if( $demographics.get("district") )&lt;td&gt;$demographics.get("district").get("value")&lt;/td&gt;#end#if( $demographics.get("divisionalSecretariat") )&lt;td&gt;$demographics.get("divisionalSecretariat").get("value")&lt;/td&gt;#end#if( $demographics.get("grammaNiladhari") )&lt;td&gt;$demographics.get("grammaNiladhari").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("postalCode") )&lt;th&gt;$demographics.get("postalCode").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("postalCode") )&lt;td&gt;$demographics.get("postalCode").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end#if( $demographics.get("currentAddressLine1") || $demographics.get("currentAddressLine2") || $demographics.get("currentAddressLine3") || $demographics.get("currentProvince") || $demographics.get("currentDistrict") || $demographics.get("currentDivisionalSecretariat") || $demographics.get("currentGramaNiladhari") || $demographics.get("currentPostalCode") )&lt;p class="demoSection"&gt;தற்போதைய முகவரி&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("currentAddressLine1") )&lt;th&gt;$demographics.get("currentAddressLine1").get("label")&lt;/th&gt;#end#if( $demographics.get("currentAddressLine2") )&lt;th&gt;$demographics.get("currentAddressLine2").get("label")&lt;/th&gt;#end#if( $demographics.get("currentAddressLine3") )&lt;th&gt;$demographics.get("currentAddressLine3").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("currentAddressLine1") )&lt;td&gt;$demographics.get("currentAddressLine1").get("value")&lt;/td&gt;#end#if( $demographics.get("currentAddressLine2") )&lt;td&gt;$demographics.get("currentAddressLine2").get("value")&lt;/td&gt;#end#if( $demographics.get("currentAddressLine3") )&lt;td&gt;$demographics.get("currentAddressLine3").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("currentProvince") )&lt;th&gt;$demographics.get("currentProvince").get("label")&lt;/th&gt;#end#if( $demographics.get("currentDistrict") )&lt;th&gt;$demographics.get("currentDistrict").get("label")&lt;/th&gt;#end#if( $demographics.get("currentDivisionalSecretariat") )&lt;th&gt;$demographics.get("currentDivisionalSecretariat").get("label")&lt;/th&gt;#end#if( $demographics.get("currentGramaNiladhari") )&lt;th&gt;$demographics.get("currentGramaNiladhari").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("currentProvince") )&lt;td&gt;$demographics.get("currentProvince").get("value")&lt;/td&gt;#end#if( $demographics.get("currentDistrict") )&lt;td&gt;$demographics.get("currentDistrict").get("value")&lt;/td&gt;#end#if( $demographics.get("currentDivisionalSecretariat") )&lt;td&gt;$demographics.get("currentDivisionalSecretariat").get("value")&lt;/td&gt;#end#if( $demographics.get("currentGramaNiladhari") )&lt;td&gt;$demographics.get("currentGramaNiladhari").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("currentPostalCode") )&lt;th&gt;$demographics.get("currentPostalCode").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("currentPostalCode") )&lt;td&gt;$demographics.get("currentPostalCode").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end#if( $demographics.get("phone") || $demographics.get("email") || $demographics.get("preferredLang") )&lt;p class="demoSection"&gt;தொடர்பு விவரங்கள்&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("phone") )&lt;th&gt;$demographics.get("phone").get("label")&lt;/th&gt;#end#if( $demographics.get("email") )&lt;th&gt;$demographics.get("email").get("label")&lt;/th&gt;#end#if( $demographics.get("preferredLang") )&lt;th&gt;$demographics.get("preferredLang").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("phone") )&lt;td&gt;$demographics.get("phone").get("value")&lt;/td&gt;#end#if( $demographics.get("email") )&lt;td&gt;$demographics.get("email").get("value")&lt;/td&gt;#end#if( $demographics.get("preferredLang") )&lt;td&gt;$demographics.get("preferredLang").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end#if( $demographics.get("introducerName") || $demographics.get("introducerRID") || $demographics.get("introducerUIN") )&lt;p class="demoSection"&gt;அறிமுகப்படுத்துபவர் விவரங்கள்&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("introducerName") )&lt;th&gt;$demographics.get("introducerName").get("label")&lt;/th&gt;#end#if( $demographics.get("introducerRID") )&lt;th&gt;$demographics.get("introducerRID").get("label")&lt;/th&gt;#end#if( $demographics.get("introducerUIN") )&lt;th&gt;$demographics.get("introducerUIN").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("introducerName") )&lt;td&gt;$demographics.get("introducerName").get("value")&lt;/td&gt;#end#if( $demographics.get("introducerRID") )&lt;td&gt;$demographics.get("introducerRID").get("value")&lt;/td&gt;#end#if( $demographics.get("introducerUIN") )&lt;td&gt;$demographics.get("introducerUIN").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end&lt;/div&gt; #if ( $ApplicantImageSource ) &lt;div class="photoDiv"&gt; &lt;table&gt; &lt;tr&gt; &lt;td&gt; &lt;p&gt;${Photo}&lt;/p&gt; &lt;/td&gt; &lt;/tr&gt; &lt;tr&gt; &lt;td&gt;&lt;img src="${ApplicantImageSource}" border=0 width=100 height=100/&gt;&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; &lt;/div&gt; #end &lt;div style="width: 100%; height: 50%; clear:both"&gt;&lt;/div&gt; &lt;br/&gt; &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;${DocumentsLabel}&lt;/p&gt; &lt;hr/&gt; &lt;table class="dataTable" style="width:100%;table-layout:fixed;border-collapse:collapse;"&gt; #foreach( $key in $documents.keySet() ) #if( $velocityCount % 2 == 1 )&lt;tr&gt;#end &lt;td style="vertical-align:top;width:50%;"&gt;&lt;p class=headings&gt;$documents.get($key).get("label")&lt;/p&gt;&lt;br/&gt;&lt;p&gt;$documents.get($key).get("value")&lt;/p&gt;&lt;/td&gt; #if( $velocityCount % 2 == 0 )&lt;/tr&gt;#end #end #if( $documents.size() % 2 == 1 )&lt;td style="vertical-align:top;width:50%;"&gt;&lt;/td&gt;&lt;/tr&gt;#end &lt;/table&gt; &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;${BiometricsLabel}&lt;/p&gt; &lt;hr/&gt; #foreach( $key in $biometrics.keySet() ) &lt;table&gt; &lt;tr&gt; &lt;td&gt;$biometrics.get($key).get("label")&lt;br/&gt; &lt;p class=headings&gt;${Fingers} ( $biometrics.get($key).get("FingerCount") ),${Iris} ( $biometrics.get($key).get("IrisCount") ),${Face} ( $biometrics.get($key).get("FaceCount") )&lt;br/&gt;&lt;/p&gt; &lt;br/&gt; &lt;/td&gt; &lt;/tr&gt; &lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftEye") ) &lt;td&gt; &lt;p class=headings&gt;${LeftEyeLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightEye") ) &lt;td&gt; &lt;p class=headings&gt;${RightEyeLabel}&lt;/p&gt; &lt;/td&gt; #end&lt;/tr&gt;&lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftEye") ) &lt;td&gt; #if( !$isPreview ) &lt;div class=biometrics&gt; &lt;h5 class=parentIris1&gt;$biometrics.get($key).get("LeftEye")&lt;/h5&gt; &lt;img src='$biometrics.get($key).get("CapturedLeftEye")' border=0 width=85 height=80/&gt; &lt;/div&gt; #end #if( $isPreview &amp;&amp; $biometrics.get($key).get("CapturedLeftEye") )&lt;img src='$biometrics.get($key).get("CapturedLeftEye")' border=0 width=85 height=80/&gt; #end &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightEye") ) &lt;td&gt;#if( !$isPreview ) &lt;div class=biometrics&gt; &lt;h5 class=parentIris1&gt;$biometrics.get($key).get("RightEye")&lt;/h5&gt; &lt;img src='$biometrics.get($key).get("CapturedRightEye")' border=0 width=85 height=80/&gt; &lt;/div&gt; #end &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftSlap") ) &lt;td&gt; &lt;p class=headings&gt;${LeftPalmLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightSlap") ) &lt;td&gt; &lt;p class=headings&gt;${RightPalmLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedThumbs") ) &lt;td&gt; &lt;p class=headings&gt;${ThumbsLabel}&lt;/p&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftSlap") ) &lt;td style=text-align:-webkit-center&gt; #if( !$isPreview ) &lt;table&gt; &lt;tr&gt; &lt;td&gt; &lt;div class=biometrics&gt; &lt;h5 class=leftLittle&gt;$biometrics.get($key).get("leftLittle")&lt;/h5&gt; &lt;h5 class=leftRing&gt;$biometrics.get($key).get("leftRing")&lt;/h5&gt; &lt;h5 class=leftMiddle&gt;$biometrics.get($key).get("leftMiddle")&lt;/h5&gt; &lt;h5 class=leftIndex&gt;$biometrics.get($key).get("leftIndex")&lt;/h5&gt; &lt;/div&gt; &lt;/td&gt;&lt;/tr&gt; &lt;tr&gt; &lt;td&gt;&lt;img src='$biometrics.get($key).get("CapturedLeftSlap")' border=0 width=85 height=80/&gt;&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; #end &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightSlap") ) &lt;td style=text-align:-webkit-center&gt; #if( !$isPreview ) &lt;table&gt; &lt;tr&gt; &lt;td&gt; &lt;div class=biometrics&gt; &lt;h5 class=rightIndex&gt;$biometrics.get($key).get("rightIndex")&lt;/h5&gt; &lt;h5 class=rightMiddle&gt;$biometrics.get($key).get("rightMiddle")&lt;/h5&gt; &lt;h5 class=rightRing&gt;$biometrics.get($key).get("rightRing")&lt;/h5&gt; &lt;h5 class=rightLittle&gt;$biometrics.get($key).get("rightLittle")&lt;/h5&gt; &lt;/div&gt; &lt;/td&gt;&lt;/tr&gt; &lt;tr&gt; &lt;td&gt;&lt;img src='$biometrics.get($key).get("CapturedRightSlap")' border=0 width=85 height=80/&gt;&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; #end &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedThumbs") ) &lt;td style=text-align:-webkit-center&gt; #if( !$isPreview ) &lt;table&gt; &lt;tr&gt; &lt;td&gt; &lt;div class=biometrics&gt; &lt;h5 class=leftThumb&gt;$biometrics.get($key).get("leftThumb")&lt;/h5&gt; &lt;h5 class=rightThumb&gt;$biometrics.get($key).get("rightThumb")&lt;/h5&gt; &lt;/div&gt; &lt;/td&gt;&lt;/tr&gt; &lt;tr&gt; &lt;td&gt;&lt;img src='$biometrics.get($key).get("CapturedThumbs")' border=0 width=85 height=80/&gt;&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; #end &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;br/&gt; &lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("FaceImageSource") ) &lt;td&gt; &lt;p class=headings&gt;${FaceLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("subType") == "applicant" &amp;&amp; $ExceptionImageSource ) &lt;td&gt; &lt;p class=headings&gt;${ExceptionPhotoLabel}&lt;/p&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;tr&gt; #if( $biometrics.get($key).get("FaceImageSource") ) &lt;td&gt;&lt;img src='$biometrics.get($key).get("FaceImageSource")' border=0 width=85 height=80/&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("subType") == "applicant" &amp;&amp; $ExceptionImageSource ) &lt;td&gt; &lt;img src="${ExceptionImageSource}" border=0 width=85 height=80/&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;/table&gt; #end &lt;br/&gt;&lt;div class="ackPostBioBlock" style="display:block;clear:both;width:100%;"&gt;#if( $SignatureSectionVisible )&lt;div data-mosip-ack-signature="1" style="display:block;width:100%;"&gt;&lt;br/&gt;&lt;hr/&gt;&lt;p class=head style="display:block;"&gt;${SignatureLabel}&lt;/p&gt;&lt;hr/&gt;&lt;/div&gt;#end&lt;table class="dataTable" style="width:100%;table-layout:fixed;border-collapse:collapse;display:table;clear:both;"&gt;#if( $SignatureSectionVisible )&lt;tr&gt;&lt;td style="vertical-align:top;width:50%;"&gt;&lt;p class=headings&gt;#if( $SignatureCaptured )${SignatureCapturedLabel}#else${SignatureNotCapturedLabel}#end&lt;/p&gt;&lt;br/&gt;&lt;p&gt;#if( $SignatureCaptured )&lt;span style="color:#2E7D32;font-size:18px;"&gt;&amp;#10004;&lt;/span&gt; &lt;span style="color:#2E7D32;"&gt;${SignatureCapturedLabel}&lt;/span&gt;#else&lt;span style="color:#808080;font-size:18px;"&gt;&amp;#10007;&lt;/span&gt; &lt;span style="color:#808080;"&gt;${SignatureNotCapturedLabel}&lt;/span&gt;#end&lt;/p&gt;&lt;/td&gt;#if( $SignatureCaptured )&lt;td style="vertical-align:top;width:50%;"&gt;&lt;p class=headings&gt;${SignatureLabel}&lt;/p&gt;&lt;br/&gt;&lt;p&gt;&lt;img data-mosip-applicant-signature="1" src="${SignatureImageSource}" border="0" width="200" height="85" style="max-width:200px;max-height:85px;object-fit:contain;border:1px solid #b0b0b0;background:#fff;display:block;"/&gt;&lt;/p&gt;&lt;/td&gt;#else&lt;td style="vertical-align:top;width:50%;"&gt;&lt;/td&gt;#end&lt;/tr&gt;#end&lt;tr&gt;&lt;td&gt;&lt;p class=headings&gt;${RONameLabel}&lt;/p&gt;&lt;br/&gt;&lt;p&gt;${ROName}&lt;/p&gt;&lt;/td&gt;&lt;td&gt;&lt;p class=headings&gt;${RegCenterLabel}&lt;/p&gt;&lt;br/&gt;&lt;p&gt;${RegCenter}&lt;/p&gt;&lt;/td&gt;&lt;/tr&gt;&lt;/table&gt;&lt;hr/&gt;&lt;br/&gt;&lt;/div&gt;&lt;div&gt;&lt;p&gt;${ImportantGuidelines}&lt;/p&gt; &lt;ul&gt; #foreach( $line in $Guidelines ) &lt;li&gt;&lt;span&gt;${line}&lt;/span&gt;&lt;/li&gt; #end &lt;/ul&gt;&lt;/div&gt;&lt;/div&gt;&lt;/div&gt;&lt;/body&gt;&lt;/html&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;!DOCTYPE html&gt;&lt;html $rtl&gt;&lt;head&gt;&lt;meta charset="UTF-8"/&gt;&lt;style&gt;body,.head,.headings,th,td,p,b,strong{font-family:system-ui,"Segoe UI","Nirmala UI","Iskoola Pota","Latha",sans-serif;}table, .head{font-size:13px;}.demoDiv{width: 85%;float: left;}.photoDiv{width: 15%;float:right;}.form{display:inline-block;}.section{align:center;padding:30px;width:800px;margin:auto;}.headings{color:#808080;font-size:11px;}p{display:inline;}.dataTable{word-wrap:break-word;table-layout:fixed;width:70%;}.headerTable{width:90%;}.uinHeaderTable{width:100%;}h5{display:inline;position:absolute;}.iris{top:-15px;left:152px;}.irisWithoutException{top:-15px;left:114px;}.tableWithoutException{width:50%;text-align:center;table-layout:fixed;margin:0 auto;}.biometricsTable{width:100%;text-align:center;table-layout:fixed;}.biometrics{position:relative;}.leftLittle{top:15px;left:11px;display:inline;position:absolute;}.leftRing{top:3px;left:23px;}.leftMiddle{top:-7px;left:37px;}.leftIndex{top:3px;left:54px;}.rightIndex{top:3px;left:26px;}.rightMiddle{top:-7px;left:39px;}.rightRing{top:3px;left:55px;}.rightLittle{top:15px;left:68px;}.leftThumb{top:-4px;left:24px;}.rightThumb{top:-4px;left:54px;}.parentStyle{top:-15px;left:152px;}.parentIris1{top:-15px;left:212px;}.parentIris2{top:-15px;left:214px;}li span{color:black;font-size:12px;} li{color:lightgrey}button{float:right;font-size:12px;border:none;background-color:transparent;outline:none;}button:active{background-color:black;color:white;}.bottom{vertical-align:bottom;}.consent-block{font-size:13px;border-radius: 8px;margin-top: 10px;margin-bottom: 10px;border: 2px solid #E88E3F;padding-top: -50px;padding:10px;}.consent-text{margin-left: 7px;margin-bottom: 4px;}input[type="radio"] {display: none;} input[type="radio"] + label:before { content: ""; display: inline-block; width: 15px; height: 15px; padding: 3px; margin-right: 5px; background-clip: content-box; border: 1px solid grey; background-color: #fff; border-radius: 50%;}input[type="radio"]:checked + label:before { background-color: #FF4081; border-color:#FF4081;}*,*:before,*:after { box-sizing: border-box;}.consent-block label { display: inline-flex; align-items: center;}.demoDiv&gt;table{width:100%}.demoDiv&gt;table&gt;tbody&gt;tr&gt;th{color:#808080;font-size:10px; width:25%; text-align: left;padding: 2px}.demoDiv&gt;table&gt;tbody&gt;tr&gt;td{width:25%; text-align: left;padding: 2px}.demoSection{display:block;color:#808080;font-size:11px;font-weight:bold;margin:12px 0 4px 0;}.demoDiv&gt;p.demoSection:first-child{margin-top:0;}.demoDiv&gt;table&gt;tbody&gt;tr&gt;th{font-weight:normal;}&lt;/style&gt;&lt;script&gt;function changeColour(element) { var div = document.getElementById("radioId"); if(element.value == "yes"){div.style = "border: 2px solid #68A933";} if(element.value == "no"){div.style = "border: 2px solid #FF0000";}} document.onreadystatechange = function () {if(document.readyState === "complete"){var body = document.getElementsByTagName("body")[0]; body.addEventListener("dragstart", function(event) {event.preventDefault();}); body.addEventListener("selectstart", function(event) {event.preventDefault();});}}&lt;/script&gt;&lt;/head&gt;&lt;body&gt; &lt;div class=section&gt; &lt;div class=form&gt; &lt;table class=headerTable&gt; &lt;tr&gt; &lt;td class=bottom&gt;&lt;p class=headings&gt;${ApplicationIDLabel}&lt;/p&gt;&lt;br/&gt;${ApplicationID}&lt;/td&gt; #if ( $UIN ) &lt;td class=bottom&gt;&lt;p class=headings&gt;${UINLabel}&lt;/p&gt;&lt;br/&gt;${UIN}&lt;/td&gt; #end &lt;td class=bottom&gt;&lt;p class=headings&gt;${DateLabel}&lt;/p&gt;&lt;br/&gt;${Date}&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; &lt;br/&gt; #if ( $name ) &lt;table class=headerTable&gt; &lt;tr&gt;&lt;td&gt;&lt;p class=headings&gt;${NameLabel}&lt;/p&gt;&lt;br/&gt;${NameValue}&lt;/td&gt;&lt;/tr&gt; &lt;/table&gt; #end &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;&lt;b&gt;${DemographicInfo}&lt;/b&gt;&lt;/p&gt;&lt;hr/&gt;&lt;div class="demoDiv"&gt;#if( $demographics.get("familyName") || $demographics.get("name") || $demographics.get("surname") || $demographics.get("gender") || $demographics.get("dateOfBirth") || $demographics.get("referenceIdentityNumber") )&lt;p class="demoSection"&gt;Personal Details&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("familyName") )&lt;th&gt;$demographics.get("familyName").get("label")&lt;/th&gt;#end#if( $demographics.get("name") )&lt;th&gt;$demographics.get("name").get("label")&lt;/th&gt;#end#if( $demographics.get("surname") )&lt;th&gt;$demographics.get("surname").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("familyName") )&lt;td&gt;$demographics.get("familyName").get("value")&lt;/td&gt;#end#if( $demographics.get("name") )&lt;td&gt;$demographics.get("name").get("value")&lt;/td&gt;#end#if( $demographics.get("surname") )&lt;td&gt;$demographics.get("surname").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("gender") )&lt;th&gt;$demographics.get("gender").get("label")&lt;/th&gt;#end#if( $demographics.get("dateOfBirth") )&lt;th&gt;$demographics.get("dateOfBirth").get("label")&lt;/th&gt;#end#if( $demographics.get("referenceIdentityNumber") )&lt;th&gt;$demographics.get("referenceIdentityNumber").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("gender") )&lt;td&gt;$demographics.get("gender").get("value")&lt;/td&gt;#end#if( $demographics.get("dateOfBirth") )&lt;td&gt;$demographics.get("dateOfBirth").get("value")&lt;/td&gt;#end#if( $demographics.get("referenceIdentityNumber") )&lt;td&gt;$demographics.get("referenceIdentityNumber").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end#if( $demographics.get("placeOfBirth") || $demographics.get("districtOfBirth") || $demographics.get("divisionalSecretariatOfBirth") )&lt;p class="demoSection"&gt;Place of Birth&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("placeOfBirth") )&lt;th&gt;$demographics.get("placeOfBirth").get("label")&lt;/th&gt;#end#if( $demographics.get("districtOfBirth") )&lt;th&gt;$demographics.get("districtOfBirth").get("label")&lt;/th&gt;#end#if( $demographics.get("divisionalSecretariatOfBirth") )&lt;th&gt;$demographics.get("divisionalSecretariatOfBirth").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("placeOfBirth") )&lt;td&gt;$demographics.get("placeOfBirth").get("value")&lt;/td&gt;#end#if( $demographics.get("districtOfBirth") )&lt;td&gt;$demographics.get("districtOfBirth").get("value")&lt;/td&gt;#end#if( $demographics.get("divisionalSecretariatOfBirth") )&lt;td&gt;$demographics.get("divisionalSecretariatOfBirth").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end#if( $demographics.get("addressLine1") || $demographics.get("addressLine2") || $demographics.get("addressLine3") || $demographics.get("province") || $demographics.get("district") || $demographics.get("divisionalSecretariat") || $demographics.get("grammaNiladhari") || $demographics.get("postalCode") )&lt;p class="demoSection"&gt;Permanent Address&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("addressLine1") )&lt;th&gt;$demographics.get("addressLine1").get("label")&lt;/th&gt;#end#if( $demographics.get("addressLine2") )&lt;th&gt;$demographics.get("addressLine2").get("label")&lt;/th&gt;#end#if( $demographics.get("addressLine3") )&lt;th&gt;$demographics.get("addressLine3").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("addressLine1") )&lt;td&gt;$demographics.get("addressLine1").get("value")&lt;/td&gt;#end#if( $demographics.get("addressLine2") )&lt;td&gt;$demographics.get("addressLine2").get("value")&lt;/td&gt;#end#if( $demographics.get("addressLine3") )&lt;td&gt;$demographics.get("addressLine3").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("province") )&lt;th&gt;$demographics.get("province").get("label")&lt;/th&gt;#end#if( $demographics.get("district") )&lt;th&gt;$demographics.get("district").get("label")&lt;/th&gt;#end#if( $demographics.get("divisionalSecretariat") )&lt;th&gt;$demographics.get("divisionalSecretariat").get("label")&lt;/th&gt;#end#if( $demographics.get("grammaNiladhari") )&lt;th&gt;$demographics.get("grammaNiladhari").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("province") )&lt;td&gt;$demographics.get("province").get("value")&lt;/td&gt;#end#if( $demographics.get("district") )&lt;td&gt;$demographics.get("district").get("value")&lt;/td&gt;#end#if( $demographics.get("divisionalSecretariat") )&lt;td&gt;$demographics.get("divisionalSecretariat").get("value")&lt;/td&gt;#end#if( $demographics.get("grammaNiladhari") )&lt;td&gt;$demographics.get("grammaNiladhari").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("postalCode") )&lt;th&gt;$demographics.get("postalCode").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("postalCode") )&lt;td&gt;$demographics.get("postalCode").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end#if( $demographics.get("currentAddressLine1") || $demographics.get("currentAddressLine2") || $demographics.get("currentAddressLine3") || $demographics.get("currentProvince") || $demographics.get("currentDistrict") || $demographics.get("currentDivisionalSecretariat") || $demographics.get("currentGramaNiladhari") || $demographics.get("currentPostalCode") )&lt;p class="demoSection"&gt;Current Address&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("currentAddressLine1") )&lt;th&gt;$demographics.get("currentAddressLine1").get("label")&lt;/th&gt;#end#if( $demographics.get("currentAddressLine2") )&lt;th&gt;$demographics.get("currentAddressLine2").get("label")&lt;/th&gt;#end#if( $demographics.get("currentAddressLine3") )&lt;th&gt;$demographics.get("currentAddressLine3").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("currentAddressLine1") )&lt;td&gt;$demographics.get("currentAddressLine1").get("value")&lt;/td&gt;#end#if( $demographics.get("currentAddressLine2") )&lt;td&gt;$demographics.get("currentAddressLine2").get("value")&lt;/td&gt;#end#if( $demographics.get("currentAddressLine3") )&lt;td&gt;$demographics.get("currentAddressLine3").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("currentProvince") )&lt;th&gt;$demographics.get("currentProvince").get("label")&lt;/th&gt;#end#if( $demographics.get("currentDistrict") )&lt;th&gt;$demographics.get("currentDistrict").get("label")&lt;/th&gt;#end#if( $demographics.get("currentDivisionalSecretariat") )&lt;th&gt;$demographics.get("currentDivisionalSecretariat").get("label")&lt;/th&gt;#end#if( $demographics.get("currentGramaNiladhari") )&lt;th&gt;$demographics.get("currentGramaNiladhari").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("currentProvince") )&lt;td&gt;$demographics.get("currentProvince").get("value")&lt;/td&gt;#end#if( $demographics.get("currentDistrict") )&lt;td&gt;$demographics.get("currentDistrict").get("value")&lt;/td&gt;#end#if( $demographics.get("currentDivisionalSecretariat") )&lt;td&gt;$demographics.get("currentDivisionalSecretariat").get("value")&lt;/td&gt;#end#if( $demographics.get("currentGramaNiladhari") )&lt;td&gt;$demographics.get("currentGramaNiladhari").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("currentPostalCode") )&lt;th&gt;$demographics.get("currentPostalCode").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("currentPostalCode") )&lt;td&gt;$demographics.get("currentPostalCode").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end#if( $demographics.get("phone") || $demographics.get("email") || $demographics.get("preferredLang") )&lt;p class="demoSection"&gt;Contact Details&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("phone") )&lt;th&gt;$demographics.get("phone").get("label")&lt;/th&gt;#end#if( $demographics.get("email") )&lt;th&gt;$demographics.get("email").get("label")&lt;/th&gt;#end#if( $demographics.get("preferredLang") )&lt;th&gt;$demographics.get("preferredLang").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("phone") )&lt;td&gt;$demographics.get("phone").get("value")&lt;/td&gt;#end#if( $demographics.get("email") )&lt;td&gt;$demographics.get("email").get("value")&lt;/td&gt;#end#if( $demographics.get("preferredLang") )&lt;td&gt;$demographics.get("preferredLang").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end#if( $demographics.get("introducerName") || $demographics.get("introducerRID") || $demographics.get("introducerUIN") )&lt;p class="demoSection"&gt;Introducer Details&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("introducerName") )&lt;th&gt;$demographics.get("introducerName").get("label")&lt;/th&gt;#end#if( $demographics.get("introducerRID") )&lt;th&gt;$demographics.get("introducerRID").get("label")&lt;/th&gt;#end#if( $demographics.get("introducerUIN") )&lt;th&gt;$demographics.get("introducerUIN").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("introducerName") )&lt;td&gt;$demographics.get("introducerName").get("value")&lt;/td&gt;#end#if( $demographics.get("introducerRID") )&lt;td&gt;$demographics.get("introducerRID").get("value")&lt;/td&gt;#end#if( $demographics.get("introducerUIN") )&lt;td&gt;$demographics.get("introducerUIN").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end&lt;/div&gt; #if ( $ApplicantImageSource ) &lt;div class="photoDiv"&gt; &lt;table&gt; &lt;tr&gt; &lt;td&gt; &lt;p&gt;${Photo}&lt;/p&gt; &lt;/td&gt; &lt;/tr&gt; &lt;tr&gt; &lt;td&gt;&lt;img src="${ApplicantImageSource}" border=0 width=100 height=100/&gt;&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; &lt;/div&gt; #end &lt;div style="width: 100%; height: 50%; clear:both"&gt;&lt;/div&gt; &lt;br&gt; &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;&lt;b&gt;${DocumentsLabel}&lt;/b&gt;&lt;/p&gt; &lt;hr/&gt; &lt;table class=dataTable&gt; #foreach( $key in $documents.keySet() ) &lt;tr&gt; &lt;td&gt; &lt;p class=headings&gt;$documents.get($key).get("label")&lt;/p&gt; &lt;br/&gt; &lt;p&gt; $documents.get($key).get("value")&lt;/p&gt; &lt;/td&gt; &lt;/tr&gt; #end &lt;/table&gt; &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;&lt;b&gt;${BiometricsLabel}&lt;/b&gt;&lt;/p&gt; &lt;hr/&gt; #foreach( $key in $biometrics.keySet() ) &lt;table&gt; &lt;tr&gt; &lt;td&gt; $biometrics.get($key).get("label")&lt;br/&gt; &lt;p class=headings&gt;${Fingers} ( $biometrics.get($key).get("FingerCount") ),${Iris} ( $biometrics.get($key).get("IrisCount") ),${Face} ( $biometrics.get($key).get("FaceCount") )&lt;br/&gt;&lt;/p&gt; &lt;br/&gt; &lt;/td&gt; &lt;/tr&gt;&lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftEye") ) &lt;td&gt;&lt;p class=headings&gt;${LeftEyeLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightEye") ) &lt;td&gt; &lt;p class=headings&gt;${RightEyeLabel}&lt;/p&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftEye") ) &lt;td&gt; #if( $biometrics.get($key).get("CapturedLeftEye") ) &lt;img src='$biometrics.get($key).get("CapturedLeftEye")' border=0 width=85 height=80/&gt; #end &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightEye") ) &lt;td&gt; #if( $biometrics.get($key).get("CapturedRightEye") ) &lt;img src='$biometrics.get($key).get("CapturedRightEye")' border=0 width=85 height=80/&gt; #end &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftSlap") ) &lt;td&gt; &lt;p class=headings&gt;${LeftPalmLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightSlap") ) &lt;td&gt; &lt;p class=headings&gt;${RightPalmLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedThumbs") ) &lt;td&gt; &lt;p class=headings&gt;${ThumbsLabel}&lt;/p&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftSlap") ) &lt;td style="text-align:-webkit-center"&gt; &lt;img src='$biometrics.get($key).get("CapturedLeftSlap")' border=0 width=85 height=80/&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightSlap") ) &lt;td style="text-align:-webkit-center"&gt; &lt;img src='$biometrics.get($key).get("CapturedRightSlap")' border=0 width=85 height=80/&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedThumbs") ) &lt;td style="text-align:-webkit-center"&gt; &lt;img src='$biometrics.get($key).get("CapturedThumbs")' border=0 width=85 height=80/&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;br/&gt; &lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("FaceImageSource") ) &lt;td&gt; &lt;p class=headings&gt;${FaceLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("subType") == "applicant" &amp;&amp; $ExceptionImageSource ) &lt;td&gt; &lt;p class=headings&gt;${ExceptionPhotoLabel}&lt;/p&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;tr&gt; #if( $biometrics.get($key).get("FaceImageSource") ) &lt;td&gt; &lt;img src='$biometrics.get($key).get("FaceImageSource")' border=0 width=85 height=80/&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("subType") == "applicant" &amp;&amp; $ExceptionImageSource ) &lt;td&gt; &lt;img src="${ExceptionImageSource}" border=0 width=85 height=80/&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;/table&gt; #end &lt;br/&gt; &lt;/div&gt; &lt;/body&gt; &lt;/html&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;!DOCTYPE html&gt;&lt;html $rtl&gt;&lt;head&gt;&lt;meta charset="UTF-8"/&gt;&lt;style&gt;body,.head,.headings,th,td,p,b,strong{font-family:system-ui,"Segoe UI","Nirmala UI","Iskoola Pota","Latha",sans-serif;}table, .head{font-size:13px;}.demoDiv{width: 85%;float: left;}.photoDiv{width: 15%;float:right;}.form{display:inline-block;}.section{align:center;padding:30px;width:800px;margin:auto;}.headings{color:#808080;font-size:11px;}p{display:inline;}.dataTable{word-wrap:break-word;table-layout:fixed;width:70%;}.headerTable{width:90%;}.uinHeaderTable{width:100%;}h5{display:inline;position:absolute;}.iris{top:-15px;left:152px;}.irisWithoutException{top:-15px;left:114px;}.tableWithoutException{width:50%;text-align:center;table-layout:fixed;margin:0 auto;}.biometricsTable{width:100%;text-align:center;table-layout:fixed;}.biometrics{position:relative;}.leftLittle{top:15px;left:11px;display:inline;position:absolute;}.leftRing{top:3px;left:23px;}.leftMiddle{top:-7px;left:37px;}.leftIndex{top:3px;left:54px;}.rightIndex{top:3px;left:26px;}.rightMiddle{top:-7px;left:39px;}.rightRing{top:3px;left:55px;}.rightLittle{top:15px;left:68px;}.leftThumb{top:-4px;left:24px;}.rightThumb{top:-4px;left:54px;}.parentStyle{top:-15px;left:152px;}.parentIris1{top:-15px;left:212px;}.parentIris2{top:-15px;left:214px;}li span{color:black;font-size:12px;} li{color:lightgrey}button{float:right;font-size:12px;border:none;background-color:transparent;outline:none;}button:active{background-color:black;color:white;}.bottom{vertical-align:bottom;}.consent-block{font-size:13px;border-radius: 8px;margin-top: 10px;margin-bottom: 10px;border: 2px solid #E88E3F;padding-top: -50px;padding:10px;}.consent-text{margin-left: 7px;margin-bottom: 4px;}input[type="radio"] {display: none;} input[type="radio"] + label:before { content: ""; display: inline-block; width: 15px; height: 15px; padding: 3px; margin-right: 5px; background-clip: content-box; border: 1px solid grey; background-color: #fff; border-radius: 50%;}input[type="radio"]:checked + label:before { background-color: #FF4081; border-color:#FF4081;}*,*:before,*:after { box-sizing: border-box;}.consent-block label { display: inline-flex; align-items: center;}.demoDiv&gt;table{width:100%}.demoDiv&gt;table&gt;tbody&gt;tr&gt;th{color:#808080;font-size:10px; width:25%; text-align: left;padding: 2px}.demoDiv&gt;table&gt;tbody&gt;tr&gt;td{width:25%; text-align: left;padding: 2px}.demoSection{display:block;color:#808080;font-size:11px;font-weight:bold;margin:12px 0 4px 0;}.demoDiv&gt;p.demoSection:first-child{margin-top:0;}.demoDiv&gt;table&gt;tbody&gt;tr&gt;th{font-weight:normal;}&lt;/style&gt;&lt;script&gt;function changeColour(element) { var div = document.getElementById("radioId"); if(element.value == "yes"){div.style = "border: 2px solid #68A933";} if(element.value == "no"){div.style = "border: 2px solid #FF0000";}} document.onreadystatechange = function () {if(document.readyState === "complete"){var body = document.getElementsByTagName("body")[0]; body.addEventListener("dragstart", function(event) {event.preventDefault();}); body.addEventListener("selectstart", function(event) {event.preventDefault();});}}&lt;/script&gt;&lt;/head&gt;&lt;body&gt; &lt;div class=section&gt; &lt;div class=form&gt; &lt;table class=headerTable&gt; &lt;tr&gt; &lt;td class=bottom&gt;&lt;p class=headings&gt;${ApplicationIDLabel}&lt;/p&gt;&lt;br/&gt;${ApplicationID}&lt;/td&gt; #if ( $UIN ) &lt;td class=bottom&gt;&lt;p class=headings&gt;${UINLabel}&lt;/p&gt;&lt;br/&gt;${UIN}&lt;/td&gt; #end &lt;td class=bottom&gt;&lt;p class=headings&gt;${DateLabel}&lt;/p&gt;&lt;br/&gt;${Date}&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; &lt;br/&gt; #if ( $name ) &lt;table class=headerTable&gt; &lt;tr&gt;&lt;td&gt;&lt;p class=headings&gt;${NameLabel}&lt;/p&gt;&lt;br/&gt;${NameValue}&lt;/td&gt;&lt;/tr&gt; &lt;/table&gt; #end &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;&lt;b&gt;${DemographicInfo}&lt;/b&gt;&lt;/p&gt;&lt;hr/&gt;&lt;div class="demoDiv"&gt;#if( $demographics.get("familyName") || $demographics.get("name") || $demographics.get("surname") || $demographics.get("gender") || $demographics.get("dateOfBirth") || $demographics.get("referenceIdentityNumber") )&lt;p class="demoSection"&gt;පෞද්ගලික විස්තර&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("familyName") )&lt;th&gt;$demographics.get("familyName").get("label")&lt;/th&gt;#end#if( $demographics.get("name") )&lt;th&gt;$demographics.get("name").get("label")&lt;/th&gt;#end#if( $demographics.get("surname") )&lt;th&gt;$demographics.get("surname").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("familyName") )&lt;td&gt;$demographics.get("familyName").get("value")&lt;/td&gt;#end#if( $demographics.get("name") )&lt;td&gt;$demographics.get("name").get("value")&lt;/td&gt;#end#if( $demographics.get("surname") )&lt;td&gt;$demographics.get("surname").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("gender") )&lt;th&gt;$demographics.get("gender").get("label")&lt;/th&gt;#end#if( $demographics.get("dateOfBirth") )&lt;th&gt;$demographics.get("dateOfBirth").get("label")&lt;/th&gt;#end#if( $demographics.get("referenceIdentityNumber") )&lt;th&gt;$demographics.get("referenceIdentityNumber").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("gender") )&lt;td&gt;$demographics.get("gender").get("value")&lt;/td&gt;#end#if( $demographics.get("dateOfBirth") )&lt;td&gt;$demographics.get("dateOfBirth").get("value")&lt;/td&gt;#end#if( $demographics.get("referenceIdentityNumber") )&lt;td&gt;$demographics.get("referenceIdentityNumber").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end#if( $demographics.get("placeOfBirth") || $demographics.get("districtOfBirth") || $demographics.get("divisionalSecretariatOfBirth") )&lt;p class="demoSection"&gt;උපන් ස්ථානය&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("placeOfBirth") )&lt;th&gt;$demographics.get("placeOfBirth").get("label")&lt;/th&gt;#end#if( $demographics.get("districtOfBirth") )&lt;th&gt;$demographics.get("districtOfBirth").get("label")&lt;/th&gt;#end#if( $demographics.get("divisionalSecretariatOfBirth") )&lt;th&gt;$demographics.get("divisionalSecretariatOfBirth").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("placeOfBirth") )&lt;td&gt;$demographics.get("placeOfBirth").get("value")&lt;/td&gt;#end#if( $demographics.get("districtOfBirth") )&lt;td&gt;$demographics.get("districtOfBirth").get("value")&lt;/td&gt;#end#if( $demographics.get("divisionalSecretariatOfBirth") )&lt;td&gt;$demographics.get("divisionalSecretariatOfBirth").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end#if( $demographics.get("addressLine1") || $demographics.get("addressLine2") || $demographics.get("addressLine3") || $demographics.get("province") || $demographics.get("district") || $demographics.get("divisionalSecretariat") || $demographics.get("grammaNiladhari") || $demographics.get("postalCode") )&lt;p class="demoSection"&gt;ස්ථිර ලිපිනය&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("addressLine1") )&lt;th&gt;$demographics.get("addressLine1").get("label")&lt;/th&gt;#end#if( $demographics.get("addressLine2") )&lt;th&gt;$demographics.get("addressLine2").get("label")&lt;/th&gt;#end#if( $demographics.get("addressLine3") )&lt;th&gt;$demographics.get("addressLine3").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("addressLine1") )&lt;td&gt;$demographics.get("addressLine1").get("value")&lt;/td&gt;#end#if( $demographics.get("addressLine2") )&lt;td&gt;$demographics.get("addressLine2").get("value")&lt;/td&gt;#end#if( $demographics.get("addressLine3") )&lt;td&gt;$demographics.get("addressLine3").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("province") )&lt;th&gt;$demographics.get("province").get("label")&lt;/th&gt;#end#if( $demographics.get("district") )&lt;th&gt;$demographics.get("district").get("label")&lt;/th&gt;#end#if( $demographics.get("divisionalSecretariat") )&lt;th&gt;$demographics.get("divisionalSecretariat").get("label")&lt;/th&gt;#end#if( $demographics.get("grammaNiladhari") )&lt;th&gt;$demographics.get("grammaNiladhari").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("province") )&lt;td&gt;$demographics.get("province").get("value")&lt;/td&gt;#end#if( $demographics.get("district") )&lt;td&gt;$demographics.get("district").get("value")&lt;/td&gt;#end#if( $demographics.get("divisionalSecretariat") )&lt;td&gt;$demographics.get("divisionalSecretariat").get("value")&lt;/td&gt;#end#if( $demographics.get("grammaNiladhari") )&lt;td&gt;$demographics.get("grammaNiladhari").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("postalCode") )&lt;th&gt;$demographics.get("postalCode").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("postalCode") )&lt;td&gt;$demographics.get("postalCode").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end#if( $demographics.get("currentAddressLine1") || $demographics.get("currentAddressLine2") || $demographics.get("currentAddressLine3") || $demographics.get("currentProvince") || $demographics.get("currentDistrict") || $demographics.get("currentDivisionalSecretariat") || $demographics.get("currentGramaNiladhari") || $demographics.get("currentPostalCode") )&lt;p class="demoSection"&gt;වත්මන් ලිපිනය&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("currentAddressLine1") )&lt;th&gt;$demographics.get("currentAddressLine1").get("label")&lt;/th&gt;#end#if( $demographics.get("currentAddressLine2") )&lt;th&gt;$demographics.get("currentAddressLine2").get("label")&lt;/th&gt;#end#if( $demographics.get("currentAddressLine3") )&lt;th&gt;$demographics.get("currentAddressLine3").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("currentAddressLine1") )&lt;td&gt;$demographics.get("currentAddressLine1").get("value")&lt;/td&gt;#end#if( $demographics.get("currentAddressLine2") )&lt;td&gt;$demographics.get("currentAddressLine2").get("value")&lt;/td&gt;#end#if( $demographics.get("currentAddressLine3") )&lt;td&gt;$demographics.get("currentAddressLine3").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("currentProvince") )&lt;th&gt;$demographics.get("currentProvince").get("label")&lt;/th&gt;#end#if( $demographics.get("currentDistrict") )&lt;th&gt;$demographics.get("currentDistrict").get("label")&lt;/th&gt;#end#if( $demographics.get("currentDivisionalSecretariat") )&lt;th&gt;$demographics.get("currentDivisionalSecretariat").get("label")&lt;/th&gt;#end#if( $demographics.get("currentGramaNiladhari") )&lt;th&gt;$demographics.get("currentGramaNiladhari").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("currentProvince") )&lt;td&gt;$demographics.get("currentProvince").get("value")&lt;/td&gt;#end#if( $demographics.get("currentDistrict") )&lt;td&gt;$demographics.get("currentDistrict").get("value")&lt;/td&gt;#end#if( $demographics.get("currentDivisionalSecretariat") )&lt;td&gt;$demographics.get("currentDivisionalSecretariat").get("value")&lt;/td&gt;#end#if( $demographics.get("currentGramaNiladhari") )&lt;td&gt;$demographics.get("currentGramaNiladhari").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("currentPostalCode") )&lt;th&gt;$demographics.get("currentPostalCode").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("currentPostalCode") )&lt;td&gt;$demographics.get("currentPostalCode").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end#if( $demographics.get("phone") || $demographics.get("email") || $demographics.get("preferredLang") )&lt;p class="demoSection"&gt;සම්බන්ධතා විස්තර&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("phone") )&lt;th&gt;$demographics.get("phone").get("label")&lt;/th&gt;#end#if( $demographics.get("email") )&lt;th&gt;$demographics.get("email").get("label")&lt;/th&gt;#end#if( $demographics.get("preferredLang") )&lt;th&gt;$demographics.get("preferredLang").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("phone") )&lt;td&gt;$demographics.get("phone").get("value")&lt;/td&gt;#end#if( $demographics.get("email") )&lt;td&gt;$demographics.get("email").get("value")&lt;/td&gt;#end#if( $demographics.get("preferredLang") )&lt;td&gt;$demographics.get("preferredLang").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end#if( $demographics.get("introducerName") || $demographics.get("introducerRID") || $demographics.get("introducerUIN") )&lt;p class="demoSection"&gt;හඳුන්වා දෙන්නාගේ විස්තර&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("introducerName") )&lt;th&gt;$demographics.get("introducerName").get("label")&lt;/th&gt;#end#if( $demographics.get("introducerRID") )&lt;th&gt;$demographics.get("introducerRID").get("label")&lt;/th&gt;#end#if( $demographics.get("introducerUIN") )&lt;th&gt;$demographics.get("introducerUIN").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("introducerName") )&lt;td&gt;$demographics.get("introducerName").get("value")&lt;/td&gt;#end#if( $demographics.get("introducerRID") )&lt;td&gt;$demographics.get("introducerRID").get("value")&lt;/td&gt;#end#if( $demographics.get("introducerUIN") )&lt;td&gt;$demographics.get("introducerUIN").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end&lt;/div&gt; #if ( $ApplicantImageSource ) &lt;div class="photoDiv"&gt; &lt;table&gt; &lt;tr&gt; &lt;td&gt; &lt;p&gt;${Photo}&lt;/p&gt; &lt;/td&gt; &lt;/tr&gt; &lt;tr&gt; &lt;td&gt;&lt;img src="${ApplicantImageSource}" border=0 width=100 height=100/&gt;&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; &lt;/div&gt; #end &lt;div style="width: 100%; height: 50%; clear:both"&gt;&lt;/div&gt; &lt;br&gt; &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;&lt;b&gt;${DocumentsLabel}&lt;/b&gt;&lt;/p&gt; &lt;hr/&gt; &lt;table class=dataTable&gt; #foreach( $key in $documents.keySet() ) &lt;tr&gt; &lt;td&gt; &lt;p class=headings&gt;$documents.get($key).get("label")&lt;/p&gt; &lt;br/&gt; &lt;p&gt; $documents.get($key).get("value")&lt;/p&gt; &lt;/td&gt; &lt;/tr&gt; #end &lt;/table&gt; &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;&lt;b&gt;${BiometricsLabel}&lt;/b&gt;&lt;/p&gt; &lt;hr/&gt; #foreach( $key in $biometrics.keySet() ) &lt;table&gt; &lt;tr&gt; &lt;td&gt; $biometrics.get($key).get("label")&lt;br/&gt; &lt;p class=headings&gt;${Fingers} ( $biometrics.get($key).get("FingerCount") ),${Iris} ( $biometrics.get($key).get("IrisCount") ),${Face} ( $biometrics.get($key).get("FaceCount") )&lt;br/&gt;&lt;/p&gt; &lt;br/&gt; &lt;/td&gt; &lt;/tr&gt;&lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftEye") ) &lt;td&gt;&lt;p class=headings&gt;${LeftEyeLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightEye") ) &lt;td&gt; &lt;p class=headings&gt;${RightEyeLabel}&lt;/p&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftEye") ) &lt;td&gt; #if( $biometrics.get($key).get("CapturedLeftEye") ) &lt;img src='$biometrics.get($key).get("CapturedLeftEye")' border=0 width=85 height=80/&gt; #end &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightEye") ) &lt;td&gt; #if( $biometrics.get($key).get("CapturedRightEye") ) &lt;img src='$biometrics.get($key).get("CapturedRightEye")' border=0 width=85 height=80/&gt; #end &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftSlap") ) &lt;td&gt; &lt;p class=headings&gt;${LeftPalmLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightSlap") ) &lt;td&gt; &lt;p class=headings&gt;${RightPalmLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedThumbs") ) &lt;td&gt; &lt;p class=headings&gt;${ThumbsLabel}&lt;/p&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftSlap") ) &lt;td style="text-align:-webkit-center"&gt; &lt;img src='$biometrics.get($key).get("CapturedLeftSlap")' border=0 width=85 height=80/&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightSlap") ) &lt;td style="text-align:-webkit-center"&gt; &lt;img src='$biometrics.get($key).get("CapturedRightSlap")' border=0 width=85 height=80/&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedThumbs") ) &lt;td style="text-align:-webkit-center"&gt; &lt;img src='$biometrics.get($key).get("CapturedThumbs")' border=0 width=85 height=80/&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;br/&gt; &lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("FaceImageSource") ) &lt;td&gt; &lt;p class=headings&gt;${FaceLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("subType") == "applicant" &amp;&amp; $ExceptionImageSource ) &lt;td&gt; &lt;p class=headings&gt;${ExceptionPhotoLabel}&lt;/p&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;tr&gt; #if( $biometrics.get($key).get("FaceImageSource") ) &lt;td&gt; &lt;img src='$biometrics.get($key).get("FaceImageSource")' border=0 width=85 height=80/&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("subType") == "applicant" &amp;&amp; $ExceptionImageSource ) &lt;td&gt; &lt;img src="${ExceptionImageSource}" border=0 width=85 height=80/&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;/table&gt; #end &lt;br/&gt; &lt;/div&gt; &lt;/body&gt; &lt;/html&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;!DOCTYPE html&gt;&lt;html $rtl&gt;&lt;head&gt;&lt;meta charset="UTF-8"/&gt;&lt;style&gt;body,.head,.headings,th,td,p,b,strong{font-family:system-ui,"Segoe UI","Nirmala UI","Iskoola Pota","Latha",sans-serif;}table, .head{font-size:13px;}.demoDiv{width: 85%;float: left;}.photoDiv{width: 15%;float:right;}.form{display:inline-block;}.section{align:center;padding:30px;width:800px;margin:auto;}.headings{color:#808080;font-size:11px;}p{display:inline;}.dataTable{word-wrap:break-word;table-layout:fixed;width:70%;}.headerTable{width:90%;}.uinHeaderTable{width:100%;}h5{display:inline;position:absolute;}.iris{top:-15px;left:152px;}.irisWithoutException{top:-15px;left:114px;}.tableWithoutException{width:50%;text-align:center;table-layout:fixed;margin:0 auto;}.biometricsTable{width:100%;text-align:center;table-layout:fixed;}.biometrics{position:relative;}.leftLittle{top:15px;left:11px;display:inline;position:absolute;}.leftRing{top:3px;left:23px;}.leftMiddle{top:-7px;left:37px;}.leftIndex{top:3px;left:54px;}.rightIndex{top:3px;left:26px;}.rightMiddle{top:-7px;left:39px;}.rightRing{top:3px;left:55px;}.rightLittle{top:15px;left:68px;}.leftThumb{top:-4px;left:24px;}.rightThumb{top:-4px;left:54px;}.parentStyle{top:-15px;left:152px;}.parentIris1{top:-15px;left:212px;}.parentIris2{top:-15px;left:214px;}li span{color:black;font-size:12px;} li{color:lightgrey}button{float:right;font-size:12px;border:none;background-color:transparent;outline:none;}button:active{background-color:black;color:white;}.bottom{vertical-align:bottom;}.consent-block{font-size:13px;border-radius: 8px;margin-top: 10px;margin-bottom: 10px;border: 2px solid #E88E3F;padding-top: -50px;padding:10px;}.consent-text{margin-left: 7px;margin-bottom: 4px;}input[type="radio"] {display: none;} input[type="radio"] + label:before { content: ""; display: inline-block; width: 15px; height: 15px; padding: 3px; margin-right: 5px; background-clip: content-box; border: 1px solid grey; background-color: #fff; border-radius: 50%;}input[type="radio"]:checked + label:before { background-color: #FF4081; border-color:#FF4081;}*,*:before,*:after { box-sizing: border-box;}.consent-block label { display: inline-flex; align-items: center;}.demoDiv&gt;table{width:100%}.demoDiv&gt;table&gt;tbody&gt;tr&gt;th{color:#808080;font-size:10px; width:25%; text-align: left;padding: 2px}.demoDiv&gt;table&gt;tbody&gt;tr&gt;td{width:25%; text-align: left;padding: 2px}.demoSection{display:block;color:#808080;font-size:11px;font-weight:bold;margin:12px 0 4px 0;}.demoDiv&gt;p.demoSection:first-child{margin-top:0;}.demoDiv&gt;table&gt;tbody&gt;tr&gt;th{font-weight:normal;}&lt;/style&gt;&lt;script&gt;function changeColour(element) { var div = document.getElementById("radioId"); if(element.value == "yes"){div.style = "border: 2px solid #68A933";} if(element.value == "no"){div.style = "border: 2px solid #FF0000";}} document.onreadystatechange = function () {if(document.readyState === "complete"){var body = document.getElementsByTagName("body")[0]; body.addEventListener("dragstart", function(event) {event.preventDefault();}); body.addEventListener("selectstart", function(event) {event.preventDefault();});}}&lt;/script&gt;&lt;/head&gt;&lt;body&gt; &lt;div class=section&gt; &lt;div class=form&gt; &lt;table class=headerTable&gt; &lt;tr&gt; &lt;td class=bottom&gt;&lt;p class=headings&gt;${ApplicationIDLabel}&lt;/p&gt;&lt;br/&gt;${ApplicationID}&lt;/td&gt; #if ( $UIN ) &lt;td class=bottom&gt;&lt;p class=headings&gt;${UINLabel}&lt;/p&gt;&lt;br/&gt;${UIN}&lt;/td&gt; #end &lt;td class=bottom&gt;&lt;p class=headings&gt;${DateLabel}&lt;/p&gt;&lt;br/&gt;${Date}&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; &lt;br/&gt; #if ( $name ) &lt;table class=headerTable&gt; &lt;tr&gt;&lt;td&gt;&lt;p class=headings&gt;${NameLabel}&lt;/p&gt;&lt;br/&gt;${NameValue}&lt;/td&gt;&lt;/tr&gt; &lt;/table&gt; #end &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;&lt;b&gt;${DemographicInfo}&lt;/b&gt;&lt;/p&gt;&lt;hr/&gt;&lt;div class="demoDiv"&gt;#if( $demographics.get("familyName") || $demographics.get("name") || $demographics.get("surname") || $demographics.get("gender") || $demographics.get("dateOfBirth") || $demographics.get("referenceIdentityNumber") )&lt;p class="demoSection"&gt;தனிப்பட்ட விவரங்கள்&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("familyName") )&lt;th&gt;$demographics.get("familyName").get("label")&lt;/th&gt;#end#if( $demographics.get("name") )&lt;th&gt;$demographics.get("name").get("label")&lt;/th&gt;#end#if( $demographics.get("surname") )&lt;th&gt;$demographics.get("surname").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("familyName") )&lt;td&gt;$demographics.get("familyName").get("value")&lt;/td&gt;#end#if( $demographics.get("name") )&lt;td&gt;$demographics.get("name").get("value")&lt;/td&gt;#end#if( $demographics.get("surname") )&lt;td&gt;$demographics.get("surname").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("gender") )&lt;th&gt;$demographics.get("gender").get("label")&lt;/th&gt;#end#if( $demographics.get("dateOfBirth") )&lt;th&gt;$demographics.get("dateOfBirth").get("label")&lt;/th&gt;#end#if( $demographics.get("referenceIdentityNumber") )&lt;th&gt;$demographics.get("referenceIdentityNumber").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("gender") )&lt;td&gt;$demographics.get("gender").get("value")&lt;/td&gt;#end#if( $demographics.get("dateOfBirth") )&lt;td&gt;$demographics.get("dateOfBirth").get("value")&lt;/td&gt;#end#if( $demographics.get("referenceIdentityNumber") )&lt;td&gt;$demographics.get("referenceIdentityNumber").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end#if( $demographics.get("placeOfBirth") || $demographics.get("districtOfBirth") || $demographics.get("divisionalSecretariatOfBirth") )&lt;p class="demoSection"&gt;பிறந்த இடம்&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("placeOfBirth") )&lt;th&gt;$demographics.get("placeOfBirth").get("label")&lt;/th&gt;#end#if( $demographics.get("districtOfBirth") )&lt;th&gt;$demographics.get("districtOfBirth").get("label")&lt;/th&gt;#end#if( $demographics.get("divisionalSecretariatOfBirth") )&lt;th&gt;$demographics.get("divisionalSecretariatOfBirth").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("placeOfBirth") )&lt;td&gt;$demographics.get("placeOfBirth").get("value")&lt;/td&gt;#end#if( $demographics.get("districtOfBirth") )&lt;td&gt;$demographics.get("districtOfBirth").get("value")&lt;/td&gt;#end#if( $demographics.get("divisionalSecretariatOfBirth") )&lt;td&gt;$demographics.get("divisionalSecretariatOfBirth").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end#if( $demographics.get("addressLine1") || $demographics.get("addressLine2") || $demographics.get("addressLine3") || $demographics.get("province") || $demographics.get("district") || $demographics.get("divisionalSecretariat") || $demographics.get("grammaNiladhari") || $demographics.get("postalCode") )&lt;p class="demoSection"&gt;நிரந்தர முகவரி&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("addressLine1") )&lt;th&gt;$demographics.get("addressLine1").get("label")&lt;/th&gt;#end#if( $demographics.get("addressLine2") )&lt;th&gt;$demographics.get("addressLine2").get("label")&lt;/th&gt;#end#if( $demographics.get("addressLine3") )&lt;th&gt;$demographics.get("addressLine3").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("addressLine1") )&lt;td&gt;$demographics.get("addressLine1").get("value")&lt;/td&gt;#end#if( $demographics.get("addressLine2") )&lt;td&gt;$demographics.get("addressLine2").get("value")&lt;/td&gt;#end#if( $demographics.get("addressLine3") )&lt;td&gt;$demographics.get("addressLine3").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("province") )&lt;th&gt;$demographics.get("province").get("label")&lt;/th&gt;#end#if( $demographics.get("district") )&lt;th&gt;$demographics.get("district").get("label")&lt;/th&gt;#end#if( $demographics.get("divisionalSecretariat") )&lt;th&gt;$demographics.get("divisionalSecretariat").get("label")&lt;/th&gt;#end#if( $demographics.get("grammaNiladhari") )&lt;th&gt;$demographics.get("grammaNiladhari").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("province") )&lt;td&gt;$demographics.get("province").get("value")&lt;/td&gt;#end#if( $demographics.get("district") )&lt;td&gt;$demographics.get("district").get("value")&lt;/td&gt;#end#if( $demographics.get("divisionalSecretariat") )&lt;td&gt;$demographics.get("divisionalSecretariat").get("value")&lt;/td&gt;#end#if( $demographics.get("grammaNiladhari") )&lt;td&gt;$demographics.get("grammaNiladhari").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("postalCode") )&lt;th&gt;$demographics.get("postalCode").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("postalCode") )&lt;td&gt;$demographics.get("postalCode").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end#if( $demographics.get("currentAddressLine1") || $demographics.get("currentAddressLine2") || $demographics.get("currentAddressLine3") || $demographics.get("currentProvince") || $demographics.get("currentDistrict") || $demographics.get("currentDivisionalSecretariat") || $demographics.get("currentGramaNiladhari") || $demographics.get("currentPostalCode") )&lt;p class="demoSection"&gt;தற்போதைய முகவரி&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("currentAddressLine1") )&lt;th&gt;$demographics.get("currentAddressLine1").get("label")&lt;/th&gt;#end#if( $demographics.get("currentAddressLine2") )&lt;th&gt;$demographics.get("currentAddressLine2").get("label")&lt;/th&gt;#end#if( $demographics.get("currentAddressLine3") )&lt;th&gt;$demographics.get("currentAddressLine3").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("currentAddressLine1") )&lt;td&gt;$demographics.get("currentAddressLine1").get("value")&lt;/td&gt;#end#if( $demographics.get("currentAddressLine2") )&lt;td&gt;$demographics.get("currentAddressLine2").get("value")&lt;/td&gt;#end#if( $demographics.get("currentAddressLine3") )&lt;td&gt;$demographics.get("currentAddressLine3").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("currentProvince") )&lt;th&gt;$demographics.get("currentProvince").get("label")&lt;/th&gt;#end#if( $demographics.get("currentDistrict") )&lt;th&gt;$demographics.get("currentDistrict").get("label")&lt;/th&gt;#end#if( $demographics.get("currentDivisionalSecretariat") )&lt;th&gt;$demographics.get("currentDivisionalSecretariat").get("label")&lt;/th&gt;#end#if( $demographics.get("currentGramaNiladhari") )&lt;th&gt;$demographics.get("currentGramaNiladhari").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("currentProvince") )&lt;td&gt;$demographics.get("currentProvince").get("value")&lt;/td&gt;#end#if( $demographics.get("currentDistrict") )&lt;td&gt;$demographics.get("currentDistrict").get("value")&lt;/td&gt;#end#if( $demographics.get("currentDivisionalSecretariat") )&lt;td&gt;$demographics.get("currentDivisionalSecretariat").get("value")&lt;/td&gt;#end#if( $demographics.get("currentGramaNiladhari") )&lt;td&gt;$demographics.get("currentGramaNiladhari").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("currentPostalCode") )&lt;th&gt;$demographics.get("currentPostalCode").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("currentPostalCode") )&lt;td&gt;$demographics.get("currentPostalCode").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end#if( $demographics.get("phone") || $demographics.get("email") || $demographics.get("preferredLang") )&lt;p class="demoSection"&gt;தொடர்பு விவரங்கள்&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("phone") )&lt;th&gt;$demographics.get("phone").get("label")&lt;/th&gt;#end#if( $demographics.get("email") )&lt;th&gt;$demographics.get("email").get("label")&lt;/th&gt;#end#if( $demographics.get("preferredLang") )&lt;th&gt;$demographics.get("preferredLang").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("phone") )&lt;td&gt;$demographics.get("phone").get("value")&lt;/td&gt;#end#if( $demographics.get("email") )&lt;td&gt;$demographics.get("email").get("value")&lt;/td&gt;#end#if( $demographics.get("preferredLang") )&lt;td&gt;$demographics.get("preferredLang").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end#if( $demographics.get("introducerName") || $demographics.get("introducerRID") || $demographics.get("introducerUIN") )&lt;p class="demoSection"&gt;அறிமுகப்படுத்துபவர் விவரங்கள்&lt;/p&gt;&lt;table&gt;&lt;tr&gt;#if( $demographics.get("introducerName") )&lt;th&gt;$demographics.get("introducerName").get("label")&lt;/th&gt;#end#if( $demographics.get("introducerRID") )&lt;th&gt;$demographics.get("introducerRID").get("label")&lt;/th&gt;#end#if( $demographics.get("introducerUIN") )&lt;th&gt;$demographics.get("introducerUIN").get("label")&lt;/th&gt;#end&lt;/tr&gt;&lt;tr&gt;#if( $demographics.get("introducerName") )&lt;td&gt;$demographics.get("introducerName").get("value")&lt;/td&gt;#end#if( $demographics.get("introducerRID") )&lt;td&gt;$demographics.get("introducerRID").get("value")&lt;/td&gt;#end#if( $demographics.get("introducerUIN") )&lt;td&gt;$demographics.get("introducerUIN").get("value")&lt;/td&gt;#end&lt;/tr&gt;&lt;/table&gt;#end&lt;/div&gt; #if ( $ApplicantImageSource ) &lt;div class="photoDiv"&gt; &lt;table&gt; &lt;tr&gt; &lt;td&gt; &lt;p&gt;${Photo}&lt;/p&gt; &lt;/td&gt; &lt;/tr&gt; &lt;tr&gt; &lt;td&gt;&lt;img src="${ApplicantImageSource}" border=0 width=100 height=100/&gt;&lt;/td&gt; &lt;/tr&gt; &lt;/table&gt; &lt;/div&gt; #end &lt;div style="width: 100%; height: 50%; clear:both"&gt;&lt;/div&gt; &lt;br&gt; &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;&lt;b&gt;${DocumentsLabel}&lt;/b&gt;&lt;/p&gt; &lt;hr/&gt; &lt;table class=dataTable&gt; #foreach( $key in $documents.keySet() ) &lt;tr&gt; &lt;td&gt; &lt;p class=headings&gt;$documents.get($key).get("label")&lt;/p&gt; &lt;br/&gt; &lt;p&gt; $documents.get($key).get("value")&lt;/p&gt; &lt;/td&gt; &lt;/tr&gt; #end &lt;/table&gt; &lt;br/&gt; &lt;hr/&gt; &lt;p class=head&gt;&lt;b&gt;${BiometricsLabel}&lt;/b&gt;&lt;/p&gt; &lt;hr/&gt; #foreach( $key in $biometrics.keySet() ) &lt;table&gt; &lt;tr&gt; &lt;td&gt; $biometrics.get($key).get("label")&lt;br/&gt; &lt;p class=headings&gt;${Fingers} ( $biometrics.get($key).get("FingerCount") ),${Iris} ( $biometrics.get($key).get("IrisCount") ),${Face} ( $biometrics.get($key).get("FaceCount") )&lt;br/&gt;&lt;/p&gt; &lt;br/&gt; &lt;/td&gt; &lt;/tr&gt;&lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftEye") ) &lt;td&gt;&lt;p class=headings&gt;${LeftEyeLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightEye") ) &lt;td&gt; &lt;p class=headings&gt;${RightEyeLabel}&lt;/p&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftEye") ) &lt;td&gt; #if( $biometrics.get($key).get("CapturedLeftEye") ) &lt;img src='$biometrics.get($key).get("CapturedLeftEye")' border=0 width=85 height=80/&gt; #end &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightEye") ) &lt;td&gt; #if( $biometrics.get($key).get("CapturedRightEye") ) &lt;img src='$biometrics.get($key).get("CapturedRightEye")' border=0 width=85 height=80/&gt; #end &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftSlap") ) &lt;td&gt; &lt;p class=headings&gt;${LeftPalmLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightSlap") ) &lt;td&gt; &lt;p class=headings&gt;${RightPalmLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedThumbs") ) &lt;td&gt; &lt;p class=headings&gt;${ThumbsLabel}&lt;/p&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;tr&gt; #if( $biometrics.get($key).get("CapturedLeftSlap") ) &lt;td style="text-align:-webkit-center"&gt; &lt;img src='$biometrics.get($key).get("CapturedLeftSlap")' border=0 width=85 height=80/&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedRightSlap") ) &lt;td style="text-align:-webkit-center"&gt; &lt;img src='$biometrics.get($key).get("CapturedRightSlap")' border=0 width=85 height=80/&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("CapturedThumbs") ) &lt;td style="text-align:-webkit-center"&gt; &lt;img src='$biometrics.get($key).get("CapturedThumbs")' border=0 width=85 height=80/&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;br/&gt; &lt;table class=biometricsTable&gt; &lt;tr&gt; #if( $biometrics.get($key).get("FaceImageSource") ) &lt;td&gt; &lt;p class=headings&gt;${FaceLabel}&lt;/p&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("subType") == "applicant" &amp;&amp; $ExceptionImageSource ) &lt;td&gt; &lt;p class=headings&gt;${ExceptionPhotoLabel}&lt;/p&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;tr&gt; #if( $biometrics.get($key).get("FaceImageSource") ) &lt;td&gt; &lt;img src='$biometrics.get($key).get("FaceImageSource")' border=0 width=85 height=80/&gt; &lt;/td&gt; #end #if( $biometrics.get($key).get("subType") == "applicant" &amp;&amp; $ExceptionImageSource ) &lt;td&gt; &lt;img src="${ExceptionImageSource}" border=0 width=85 height=80/&gt; &lt;/td&gt; #end &lt;/tr&gt; &lt;/table&gt; &lt;/table&gt; #end &lt;br/&gt; &lt;/div&gt; &lt;/body&gt; &lt;/html&gt;</t>
   </si>
   <si>
     <t>&lt;!DOCTYPE html&gt;&lt;html&gt;&lt;head&gt;&lt;meta charset="UTF-8"/&gt;&lt;title&gt;சம்மதம்&lt;/title&gt;&lt;style&gt;body,div,p,b,strong{font-family:system-ui,"Segoe UI","Nirmala UI","Iskoola Pota","Latha",sans-serif;}&lt;/style&gt;&lt;/head&gt;&lt;body&gt;&lt;div&gt;பதிவின் போது குறிப்பிட்ட அதிகாரசபையினால் என்னைப் பற்றிச் சேகரிக்கப்படும் தரவுகளில் பின்வருவன அடங்கும் என்பதை நான் புரிந்துகொள்கிறேன் &lt;br&gt;&lt;br&gt;&amp;#x2022; பெயர் &lt;br&gt; &amp;#x2022; பிறந்த தேதி &lt;br&gt; &amp;#x2022; பாலினம் &lt;br&gt; &amp;#x2022; முகவரி &lt;br&gt; &amp;#x2022; தொடர்பு விவரங்கள் &lt;br&gt; &amp;#x2022; ஆவணங்கள்&lt;br&gt; &amp;#x2022; உயிரளவியல் தரவு &lt;br&gt; &lt;br&gt;பல்வேறு சேவைகளைப் பெறுவதற்காக எனது அடையாளத்தை உறுதிப்படுத்தும் நோக்கத்திற்காக அல்லது சட்டரீதியான கடப்பாட்டுக்கு இணங்குவதற்காக இந்தத் தகவல்கள் சேமிக்கப்பட்டுச் செயலாக்கப்படும் என்பதையும் நான் புரிந்துகொள்கிறேன். இந்த நோக்கத்திற்காக இத்தரவுகளைச் சேகரிப்பதற்கு நான் எனது சம்மதத்தை அளிக்கிறேன்.&lt;/div&gt;&lt;/body&gt;&lt;/html&gt;</t>

</xml_diff>